<commit_message>
Preserve personal exclusions across policy updates
</commit_message>
<xml_diff>
--- a/exports/all.xlsx
+++ b/exports/all.xlsx
@@ -942,7 +942,7 @@
       <c r="E1" s="46" t="inlineStr">
         <is>
           <t>原始发布日期：1900-01-01 至 2026-09-29
-含首尾；导出时间（北京）2026-09-29 13:57</t>
+含首尾；导出时间（北京）2026-09-29 14:01</t>
         </is>
       </c>
     </row>
@@ -4674,7 +4674,7 @@
       </c>
       <c r="B7" s="59" t="inlineStr">
         <is>
-          <t>2026-09-29 13:57:07</t>
+          <t>2026-09-29 14:01:58</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Hide table guidance behind help buttons and speed up loading
</commit_message>
<xml_diff>
--- a/exports/all.xlsx
+++ b/exports/all.xlsx
@@ -942,7 +942,7 @@
       <c r="E1" s="46" t="inlineStr">
         <is>
           <t>原始发布日期：1900-01-01 至 2026-09-29
-含首尾；导出时间（北京）2026-09-29 14:01</t>
+含首尾；导出时间（北京）2026-09-29 14:09</t>
         </is>
       </c>
     </row>
@@ -4674,7 +4674,7 @@
       </c>
       <c r="B7" s="59" t="inlineStr">
         <is>
-          <t>2026-09-29 14:01:58</t>
+          <t>2026-09-29 14:09:22</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Speed up policy dashboard startup
</commit_message>
<xml_diff>
--- a/exports/all.xlsx
+++ b/exports/all.xlsx
@@ -942,7 +942,7 @@
       <c r="E1" s="46" t="inlineStr">
         <is>
           <t>原始发布日期：1900-01-01 至 2026-09-29
-含首尾；导出时间（北京）2026-09-29 14:09</t>
+含首尾；导出时间（北京）2026-09-29 16:05</t>
         </is>
       </c>
     </row>
@@ -4674,7 +4674,7 @@
       </c>
       <c r="B7" s="59" t="inlineStr">
         <is>
-          <t>2026-09-29 14:09:22</t>
+          <t>2026-09-29 16:05:37</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove note panel from policy details
</commit_message>
<xml_diff>
--- a/exports/all.xlsx
+++ b/exports/all.xlsx
@@ -942,7 +942,7 @@
       <c r="E1" s="46" t="inlineStr">
         <is>
           <t>原始发布日期：1900-01-01 至 2026-09-29
-含首尾；导出时间（北京）2026-09-29 16:05</t>
+含首尾；导出时间（北京）2026-09-29 16:40</t>
         </is>
       </c>
     </row>
@@ -4674,7 +4674,7 @@
       </c>
       <c r="B7" s="59" t="inlineStr">
         <is>
-          <t>2026-09-29 16:05:37</t>
+          <t>2026-09-29 16:40:39</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Cache bust dashboard assets
</commit_message>
<xml_diff>
--- a/exports/all.xlsx
+++ b/exports/all.xlsx
@@ -942,7 +942,7 @@
       <c r="E1" s="46" t="inlineStr">
         <is>
           <t>原始发布日期：1900-01-01 至 2026-09-29
-含首尾；导出时间（北京）2026-09-29 16:40</t>
+含首尾；导出时间（北京）2026-09-29 16:43</t>
         </is>
       </c>
     </row>
@@ -4674,7 +4674,7 @@
       </c>
       <c r="B7" s="59" t="inlineStr">
         <is>
-          <t>2026-09-29 16:40:39</t>
+          <t>2026-09-29 16:43:58</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh policy snapshot after September 30 collection retry
</commit_message>
<xml_diff>
--- a/exports/all.xlsx
+++ b/exports/all.xlsx
@@ -941,8 +941,8 @@
       </c>
       <c r="E1" s="46" t="inlineStr">
         <is>
-          <t>原始发布日期：1900-01-01 至 2026-09-29
-含首尾；导出时间（北京）2026-09-29 16:43</t>
+          <t>原始发布日期：1900-01-01 至 2026-09-30
+含首尾；导出时间（北京）2026-09-30 11:28</t>
         </is>
       </c>
     </row>
@@ -2155,7 +2155,7 @@
       </c>
       <c r="C37" s="51" t="inlineStr">
         <is>
-          <t>原始发布日期 1900-01-01—2026-09-29（含首尾）；官方出处及完整证据见政策明细。</t>
+          <t>原始发布日期 1900-01-01—2026-09-30（含首尾）；官方出处及完整证据见政策明细。</t>
         </is>
       </c>
       <c r="D37" s="20" t="n"/>
@@ -2285,7 +2285,7 @@
       </c>
       <c r="C42" s="50" t="inlineStr">
         <is>
-          <t>原始发布日期 1900-01-01—2026-09-29（含首尾）；官方出处及完整证据见政策明细。</t>
+          <t>原始发布日期 1900-01-01—2026-09-30（含首尾）；官方出处及完整证据见政策明细。</t>
         </is>
       </c>
       <c r="D42" s="44" t="n"/>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="C48" s="49" t="inlineStr">
         <is>
-          <t>原始发布日期 1900-01-01—2026-09-29（含首尾）；官方出处及完整证据见政策明细。</t>
+          <t>原始发布日期 1900-01-01—2026-09-30（含首尾）；官方出处及完整证据见政策明细。</t>
         </is>
       </c>
       <c r="D48" s="45" t="n"/>
@@ -2548,7 +2548,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C原发日期 1900-01-01 至 2026-09-29（含两端）&amp;R第 &amp;P 页 / 共 &amp;N 页</oddFooter>
+    <oddFooter>&amp;C原发日期 1900-01-01 至 2026-09-30（含两端）&amp;R第 &amp;P 页 / 共 &amp;N 页</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -4614,7 +4614,7 @@
       </c>
       <c r="B2" s="59" t="inlineStr">
         <is>
-          <t>1900-01-01 至 2026-09-29（含起止两日，闭区间；不按转载日期筛选）</t>
+          <t>1900-01-01 至 2026-09-30（含起止两日，闭区间；不按转载日期筛选）</t>
         </is>
       </c>
     </row>
@@ -4674,7 +4674,7 @@
       </c>
       <c r="B7" s="59" t="inlineStr">
         <is>
-          <t>2026-09-29 16:43:58</t>
+          <t>2026-09-30 11:28:39</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update public policy dashboard
</commit_message>
<xml_diff>
--- a/exports/all.xlsx
+++ b/exports/all.xlsx
@@ -15,9 +15,9 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'事项监控表'!$A$1:$F$48</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'政策明细'!$A$1:$M$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'政策明细'!$A$1:$M$59</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'政策明细'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'参考资料'!$A$1:$M$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'参考资料'!$A$1:$M$8</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'参考资料'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -941,8 +941,8 @@
       </c>
       <c r="E1" s="46" t="inlineStr">
         <is>
-          <t>原始发布日期：1900-01-01 至 2026-09-30
-含首尾；导出时间（北京）2026-09-30 11:28</t>
+          <t>原始发布日期：1900-01-01 至 2026-10-13
+含首尾；导出时间（北京）2026-10-13 09:43</t>
         </is>
       </c>
     </row>
@@ -981,12 +981,12 @@
       </c>
       <c r="C3" s="48" t="inlineStr">
         <is>
-          <t>【本地政策｜已采集｜明细1】
+          <t>【本地政策｜已采集｜明细5】
 2026-09-24 北京市住房和城乡建设委员会等4部门关于发布本市贯彻落实《关于完善商品住房销售制度的通知》的实施意见
 官方原文：https://zjw.beijing.gov.cn/bjjs/xxgk/zcwj2024/qtzcwj/xxyx13/744131235/index.shtml
 官方原文：https://gjj.beijing.gov.cn/web/zwgk61/2024zcwj/436433464/436433468/744131565/index.html
 原文摘录（非模型总结）：为贯彻落实《住房城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知》（建房规〔2026〕3号）有关要求，加快构建房地产发展新模式，稳步推进商品住房销售制度改革，结合本市实际，提出如下实施意见 。
-【国家基准｜已采集｜明细4】
+【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：为贯彻落实党中央、国务院关于加快构建房地产发展新模式的决策部署,坚持稳中求进、先立后破,稳步推进商品住房销售制度改革,现就有关事项通知如下。</t>
@@ -1013,7 +1013,7 @@
       </c>
       <c r="C4" s="48" t="inlineStr">
         <is>
-          <t>【国家基准｜已采集｜明细4】
+          <t>【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：为贯彻落实党中央、国务院关于加快构建房地产发展新模式的决策部署,坚持稳中求进、先立后破,稳步推进商品住房销售制度改革,现就有关事项通知如下。</t>
@@ -1038,7 +1038,7 @@
       </c>
       <c r="C5" s="48" t="inlineStr">
         <is>
-          <t>【国家基准｜已采集｜明细4】
+          <t>【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：为贯彻落实党中央、国务院关于加快构建房地产发展新模式的决策部署,坚持稳中求进、先立后破,稳步推进商品住房销售制度改革,现就有关事项通知如下。</t>
@@ -1064,12 +1064,12 @@
       <c r="C6" s="50" t="inlineStr">
         <is>
           <t>三亚：
-【国家基准｜已采集｜明细4】
+【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：为贯彻落实党中央、国务院关于加快构建房地产发展新模式的决策部署,坚持稳中求进、先立后破,稳步推进商品住房销售制度改革,现就有关事项通知如下。
 陵水：
-【国家基准｜已采集｜明细4】
+【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：为贯彻落实党中央、国务院关于加快构建房地产发展新模式的决策部署,坚持稳中求进、先立后破,稳步推进商品住房销售制度改革,现就有关事项通知如下。</t>
@@ -1150,13 +1150,13 @@
       </c>
       <c r="C10" s="51" t="inlineStr">
         <is>
-          <t>【本地政策｜已采集｜明细1】
+          <t>【本地政策｜已采集｜明细5】
 2026-09-24 北京市住房和城乡建设委员会等4部门关于发布本市贯彻落实《关于完善商品住房销售制度的通知》的实施意见
 官方原文：https://zjw.beijing.gov.cn/bjjs/xxgk/zcwj2024/qtzcwj/xxyx13/744131235/index.shtml
 官方原文：https://gjj.beijing.gov.cn/web/zwgk61/2024zcwj/436433464/436433468/744131565/index.html
 原文摘录（非模型总结）：（二）在途项目。 2026年8月28日（含）前，已取得 （含部分取得） 建设工程规划许可证但未办理预售许可的商品住房项目 ，申请 预售的，预售条件、预售资金监管等按原有政策规定执行。
 2026年8月28日（含）前，已取得 （含正在出让） 国有建设用地使用权但未取得建设工程规划许可证的商品住房项目， 原则上按新取得土地项目执行预售管理政策， 各区政府 确保 能够按时建成交付 的 ， 在加强预售资金监管的情况下， 报市级部门 备案 后， 在2027年底前仍可 按原 有预售条件申请预售， 但资金监管按以下要求执行：
-【国家基准｜已采集｜明细4】
+【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：(三)优化存量项目预售管理。本通知施行之日前已取得建设工程规划许可证的商品住房项目,实行预售的,预售条件、预售资金监管等按原有政策规定执行。应合理确定监管额度,优化预售资金使用,严格预售资金监管,保障预售资金安全。</t>
@@ -1164,7 +1164,7 @@
       </c>
       <c r="D10" s="52" t="inlineStr">
         <is>
-          <t>【国家基准｜已采集｜明细4】
+          <t>【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：(三)优化存量项目预售管理。本通知施行之日前已取得建设工程规划许可证的商品住房项目,实行预售的,预售条件、预售资金监管等按原有政策规定执行。应合理确定监管额度,优化预售资金使用,严格预售资金监管,保障预售资金安全。</t>
@@ -1172,7 +1172,7 @@
       </c>
       <c r="E10" s="52" t="inlineStr">
         <is>
-          <t>【国家基准｜已采集｜明细4】
+          <t>【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：(三)优化存量项目预售管理。本通知施行之日前已取得建设工程规划许可证的商品住房项目,实行预售的,预售条件、预售资金监管等按原有政策规定执行。应合理确定监管额度,优化预售资金使用,严格预售资金监管,保障预售资金安全。</t>
@@ -1181,12 +1181,12 @@
       <c r="F10" s="51" t="inlineStr">
         <is>
           <t>三亚：
-【国家基准｜已采集｜明细4】
+【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：(三)优化存量项目预售管理。本通知施行之日前已取得建设工程规划许可证的商品住房项目,实行预售的,预售条件、预售资金监管等按原有政策规定执行。应合理确定监管额度,优化预售资金使用,严格预售资金监管,保障预售资金安全。
 陵水：
-【国家基准｜已采集｜明细4】
+【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：(三)优化存量项目预售管理。本通知施行之日前已取得建设工程规划许可证的商品住房项目,实行预售的,预售条件、预售资金监管等按原有政策规定执行。应合理确定监管额度,优化预售资金使用,严格预售资金监管,保障预售资金安全。</t>
@@ -1202,13 +1202,13 @@
       </c>
       <c r="C11" s="51" t="inlineStr">
         <is>
-          <t>【本地政策｜已采集｜明细1】
+          <t>【本地政策｜已采集｜明细5】
 2026-09-24 北京市住房和城乡建设委员会等4部门关于发布本市贯彻落实《关于完善商品住房销售制度的通知》的实施意见
 官方原文：https://zjw.beijing.gov.cn/bjjs/xxgk/zcwj2024/qtzcwj/xxyx13/744131235/index.shtml
 官方原文：https://gjj.beijing.gov.cn/web/zwgk61/2024zcwj/436433464/436433468/744131565/index.html
 原文摘录（非模型总结）：（二）在途项目。 2026年8月28日（含）前，已取得 （含部分取得） 建设工程规划许可证但未办理预售许可的商品住房项目 ，申请 预售的，预售条件、预售资金监管等按原有政策规定执行。
 2026年8月28日（含）前，已取得 （含正在出让） 国有建设用地使用权但未取得建设工程规划许可证的商品住房项目， 原则上按新取得土地项目执行预售管理政策， 各区政府 确保 能够按时建成交付 的 ， 在加强预售资金监管的情况下， 报市级部门 备案 后， 在2027年底前仍可 按原 有预售条件申请预售， 但资金监管按以下要求执行：
-【国家基准｜已采集｜明细4】
+【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：(三)优化存量项目预售管理。本通知施行之日前已取得建设工程规划许可证的商品住房项目,实行预售的,预售条件、预售资金监管等按原有政策规定执行。应合理确定监管额度,优化预售资金使用,严格预售资金监管,保障预售资金安全。</t>
@@ -1216,7 +1216,7 @@
       </c>
       <c r="D11" s="52" t="inlineStr">
         <is>
-          <t>【国家基准｜已采集｜明细4】
+          <t>【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：(三)优化存量项目预售管理。本通知施行之日前已取得建设工程规划许可证的商品住房项目,实行预售的,预售条件、预售资金监管等按原有政策规定执行。应合理确定监管额度,优化预售资金使用,严格预售资金监管,保障预售资金安全。</t>
@@ -1224,7 +1224,7 @@
       </c>
       <c r="E11" s="52" t="inlineStr">
         <is>
-          <t>【国家基准｜已采集｜明细4】
+          <t>【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：(三)优化存量项目预售管理。本通知施行之日前已取得建设工程规划许可证的商品住房项目,实行预售的,预售条件、预售资金监管等按原有政策规定执行。应合理确定监管额度,优化预售资金使用,严格预售资金监管,保障预售资金安全。</t>
@@ -1233,12 +1233,12 @@
       <c r="F11" s="51" t="inlineStr">
         <is>
           <t>三亚：
-【国家基准｜已采集｜明细4】
+【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：(三)优化存量项目预售管理。本通知施行之日前已取得建设工程规划许可证的商品住房项目,实行预售的,预售条件、预售资金监管等按原有政策规定执行。应合理确定监管额度,优化预售资金使用,严格预售资金监管,保障预售资金安全。
 陵水：
-【国家基准｜已采集｜明细4】
+【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：(三)优化存量项目预售管理。本通知施行之日前已取得建设工程规划许可证的商品住房项目,实行预售的,预售条件、预售资金监管等按原有政策规定执行。应合理确定监管额度,优化预售资金使用,严格预售资金监管,保障预售资金安全。</t>
@@ -1377,13 +1377,13 @@
       </c>
       <c r="C17" s="51" t="inlineStr">
         <is>
-          <t>【本地政策｜已采集｜明细1】
+          <t>【本地政策｜已采集｜明细5】
 2026-09-24 北京市住房和城乡建设委员会等4部门关于发布本市贯彻落实《关于完善商品住房销售制度的通知》的实施意见
 官方原文：https://zjw.beijing.gov.cn/bjjs/xxgk/zcwj2024/qtzcwj/xxyx13/744131235/index.shtml
 官方原文：https://gjj.beijing.gov.cn/web/zwgk61/2024zcwj/436433464/436433468/744131565/index.html
 原文摘录（非模型总结）：（一）新取得土地项目。 2026年8月28日后 新发布国有 建设用地 使用权出让公告的商品住房项目， 申请 预售 的 ，单体建筑 应 完成主体结构封顶 （楼栋顶板及楼顶构筑物、配套设施完成混凝土浇筑）， 项目 建设单位、勘察、设计、施工、监理 等单位 应出具 签字 盖章 的《主体结构分部工程验收记录》 。项目 预售资金全额 、全过程监管 ，项目 联合验收后 ， 方可 解除资金监管。 具体预售资金监管办法另行印发。
 （二）在途项目。 2026年8月28日（含）前，已取得 （含部分取得） 建设工程规划许可证但未办理预售许可的商品住房项目 ，申请 预售的，预售条件、预售资金监管等按原有政策规定执行。
-【国家基准｜已采集｜明细4】
+【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：各地要规范商品住房预售条件,加强预售资金监管,保障预售资金安全,有效防范商品住房交付风险,维护购房人合法权益。
@@ -1392,7 +1392,7 @@
       </c>
       <c r="D17" s="54" t="inlineStr">
         <is>
-          <t>【国家基准｜已采集｜明细4】
+          <t>【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：各地要规范商品住房预售条件,加强预售资金监管,保障预售资金安全,有效防范商品住房交付风险,维护购房人合法权益。
@@ -1401,7 +1401,7 @@
       </c>
       <c r="E17" s="55" t="inlineStr">
         <is>
-          <t>【国家基准｜已采集｜明细4】
+          <t>【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：各地要规范商品住房预售条件,加强预售资金监管,保障预售资金安全,有效防范商品住房交付风险,维护购房人合法权益。
@@ -1411,13 +1411,13 @@
       <c r="F17" s="54" t="inlineStr">
         <is>
           <t>三亚：
-【国家基准｜已采集｜明细4】
+【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：各地要规范商品住房预售条件,加强预售资金监管,保障预售资金安全,有效防范商品住房交付风险,维护购房人合法权益。
 (一)规范预售条件。商品住房项目实行预售的,单体建筑应完成主体结构封顶,具体条件由各地根据实际情况确定。
 陵水：
-【国家基准｜已采集｜明细4】
+【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：各地要规范商品住房预售条件,加强预售资金监管,保障预售资金安全,有效防范商品住房交付风险,维护购房人合法权益。
@@ -1434,12 +1434,12 @@
       </c>
       <c r="C18" s="51" t="inlineStr">
         <is>
-          <t>【本地政策｜已采集｜明细1】
+          <t>【本地政策｜已采集｜明细5】
 2026-09-24 北京市住房和城乡建设委员会等4部门关于发布本市贯彻落实《关于完善商品住房销售制度的通知》的实施意见
 官方原文：https://zjw.beijing.gov.cn/bjjs/xxgk/zcwj2024/qtzcwj/xxyx13/744131235/index.shtml
 官方原文：https://gjj.beijing.gov.cn/web/zwgk61/2024zcwj/436433464/436433468/744131565/index.html
 原文摘录（非模型总结）：（一）规范个人按揭贷款发放。 2026年8月28日后取得预售许可证的项目，竣工备案后方可发放个人住房按揭贷款（含公积金贷款），贷款资金应当通过受托支付方式支付至预售资金监管账户。
-【国家基准｜已采集｜明细5】
+【国家基准｜已采集｜明细9】
 2026-08-28 中国人民银行 国家金融监督管理总局印发《关于改革完善房地产信贷管理 推动加快构建房地产发展新模式的意见》的通知（银发〔2026〕171号）
 官方原文：https://hunan.gov.cn/zqt/zcsd/202609/t20260907_34058152.html
 原文摘录（非模型总结）：第二十二条 所购新建住房实行现房销售的,个人住房贷款应在销售备案后发放;实行预售的,应严格在项目竣工备案后发放。
@@ -1448,7 +1448,7 @@
       </c>
       <c r="D18" s="57" t="inlineStr">
         <is>
-          <t>【国家基准｜已采集｜明细5】
+          <t>【国家基准｜已采集｜明细9】
 2026-08-28 中国人民银行 国家金融监督管理总局印发《关于改革完善房地产信贷管理 推动加快构建房地产发展新模式的意见》的通知（银发〔2026〕171号）
 官方原文：https://hunan.gov.cn/zqt/zcsd/202609/t20260907_34058152.html
 原文摘录（非模型总结）：第二十二条 所购新建住房实行现房销售的,个人住房贷款应在销售备案后发放;实行预售的,应严格在项目竣工备案后发放。
@@ -1457,7 +1457,7 @@
       </c>
       <c r="E18" s="52" t="inlineStr">
         <is>
-          <t>【国家基准｜已采集｜明细5】
+          <t>【国家基准｜已采集｜明细9】
 2026-08-28 中国人民银行 国家金融监督管理总局印发《关于改革完善房地产信贷管理 推动加快构建房地产发展新模式的意见》的通知（银发〔2026〕171号）
 官方原文：https://hunan.gov.cn/zqt/zcsd/202609/t20260907_34058152.html
 原文摘录（非模型总结）：第二十二条 所购新建住房实行现房销售的,个人住房贷款应在销售备案后发放;实行预售的,应严格在项目竣工备案后发放。
@@ -1467,13 +1467,13 @@
       <c r="F18" s="54" t="inlineStr">
         <is>
           <t>三亚：
-【国家基准｜已采集｜明细5】
+【国家基准｜已采集｜明细9】
 2026-08-28 中国人民银行 国家金融监督管理总局印发《关于改革完善房地产信贷管理 推动加快构建房地产发展新模式的意见》的通知（银发〔2026〕171号）
 官方原文：https://hunan.gov.cn/zqt/zcsd/202609/t20260907_34058152.html
 原文摘录（非模型总结）：第二十二条 所购新建住房实行现房销售的,个人住房贷款应在销售备案后发放;实行预售的,应严格在项目竣工备案后发放。
 个人住房贷款应通过受托支付方式发放。对实行现房销售的,受托支付至项目公司在主办银行开立的资金账户;对实行预售的,受托支付至项目预售资金监管账户。所购住房为再交易住房的,受托支付至贷款合同约定的借款人交易对象账户。
 陵水：
-【国家基准｜已采集｜明细5】
+【国家基准｜已采集｜明细9】
 2026-08-28 中国人民银行 国家金融监督管理总局印发《关于改革完善房地产信贷管理 推动加快构建房地产发展新模式的意见》的通知（银发〔2026〕171号）
 官方原文：https://hunan.gov.cn/zqt/zcsd/202609/t20260907_34058152.html
 原文摘录（非模型总结）：第二十二条 所购新建住房实行现房销售的,个人住房贷款应在销售备案后发放;实行预售的,应严格在项目竣工备案后发放。
@@ -1490,12 +1490,12 @@
       </c>
       <c r="C19" s="51" t="inlineStr">
         <is>
-          <t>【本地政策｜已采集｜明细1】
+          <t>【本地政策｜已采集｜明细5】
 2026-09-24 北京市住房和城乡建设委员会等4部门关于发布本市贯彻落实《关于完善商品住房销售制度的通知》的实施意见
 官方原文：https://zjw.beijing.gov.cn/bjjs/xxgk/zcwj2024/qtzcwj/xxyx13/744131235/index.shtml
 官方原文：https://gjj.beijing.gov.cn/web/zwgk61/2024zcwj/436433464/436433468/744131565/index.html
 原文摘录（非模型总结）：（一）规范个人按揭贷款发放。 2026年8月28日后取得预售许可证的项目，竣工备案后方可发放个人住房按揭贷款（含公积金贷款），贷款资金应当通过受托支付方式支付至预售资金监管账户。
-【国家基准｜已采集｜明细5】
+【国家基准｜已采集｜明细9】
 2026-08-28 中国人民银行 国家金融监督管理总局印发《关于改革完善房地产信贷管理 推动加快构建房地产发展新模式的意见》的通知（银发〔2026〕171号）
 官方原文：https://hunan.gov.cn/zqt/zcsd/202609/t20260907_34058152.html
 原文摘录（非模型总结）：第二十二条 所购新建住房实行现房销售的,个人住房贷款应在销售备案后发放;实行预售的,应严格在项目竣工备案后发放。
@@ -1504,7 +1504,7 @@
       </c>
       <c r="D19" s="52" t="inlineStr">
         <is>
-          <t>【国家基准｜已采集｜明细5】
+          <t>【国家基准｜已采集｜明细9】
 2026-08-28 中国人民银行 国家金融监督管理总局印发《关于改革完善房地产信贷管理 推动加快构建房地产发展新模式的意见》的通知（银发〔2026〕171号）
 官方原文：https://hunan.gov.cn/zqt/zcsd/202609/t20260907_34058152.html
 原文摘录（非模型总结）：第二十二条 所购新建住房实行现房销售的,个人住房贷款应在销售备案后发放;实行预售的,应严格在项目竣工备案后发放。
@@ -1513,7 +1513,7 @@
       </c>
       <c r="E19" s="52" t="inlineStr">
         <is>
-          <t>【国家基准｜已采集｜明细5】
+          <t>【国家基准｜已采集｜明细9】
 2026-08-28 中国人民银行 国家金融监督管理总局印发《关于改革完善房地产信贷管理 推动加快构建房地产发展新模式的意见》的通知（银发〔2026〕171号）
 官方原文：https://hunan.gov.cn/zqt/zcsd/202609/t20260907_34058152.html
 原文摘录（非模型总结）：第二十二条 所购新建住房实行现房销售的,个人住房贷款应在销售备案后发放;实行预售的,应严格在项目竣工备案后发放。
@@ -1523,13 +1523,13 @@
       <c r="F19" s="54" t="inlineStr">
         <is>
           <t>三亚：
-【国家基准｜已采集｜明细5】
+【国家基准｜已采集｜明细9】
 2026-08-28 中国人民银行 国家金融监督管理总局印发《关于改革完善房地产信贷管理 推动加快构建房地产发展新模式的意见》的通知（银发〔2026〕171号）
 官方原文：https://hunan.gov.cn/zqt/zcsd/202609/t20260907_34058152.html
 原文摘录（非模型总结）：第二十二条 所购新建住房实行现房销售的,个人住房贷款应在销售备案后发放;实行预售的,应严格在项目竣工备案后发放。
 个人住房贷款应通过受托支付方式发放。对实行现房销售的,受托支付至项目公司在主办银行开立的资金账户;对实行预售的,受托支付至项目预售资金监管账户。所购住房为再交易住房的,受托支付至贷款合同约定的借款人交易对象账户。
 陵水：
-【国家基准｜已采集｜明细5】
+【国家基准｜已采集｜明细9】
 2026-08-28 中国人民银行 国家金融监督管理总局印发《关于改革完善房地产信贷管理 推动加快构建房地产发展新模式的意见》的通知（银发〔2026〕171号）
 官方原文：https://hunan.gov.cn/zqt/zcsd/202609/t20260907_34058152.html
 原文摘录（非模型总结）：第二十二条 所购新建住房实行现房销售的,个人住房贷款应在销售备案后发放;实行预售的,应严格在项目竣工备案后发放。
@@ -1560,12 +1560,12 @@
       </c>
       <c r="C21" s="51" t="inlineStr">
         <is>
-          <t>【本地政策｜已采集｜明细1】
+          <t>【本地政策｜已采集｜明细5】
 2026-09-24 北京市住房和城乡建设委员会等4部门关于发布本市贯彻落实《关于完善商品住房销售制度的通知》的实施意见
 官方原文：https://zjw.beijing.gov.cn/bjjs/xxgk/zcwj2024/qtzcwj/xxyx13/744131235/index.shtml
 官方原文：https://gjj.beijing.gov.cn/web/zwgk61/2024zcwj/436433464/436433468/744131565/index.html
 原文摘录（非模型总结）：2026年8月28日起，新发布国有 建设用地 使用权出让公告的商品住房项目 优先 选择 现房销售。房地产开发企业在取得房屋首次登记后，编制现房销售方案，向房屋所在区住房城乡建设 （ 房管 ） 部门申请现房销售备案 后 ，按现房销售方案 组织 销售，所销售房屋及建设用地使用权应无抵押、查封等情形。
-【国家基准｜已采集｜明细4】
+【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：(一)推进商品住房现房销售。本通知施行之日起,新出让土地的商品住房项目和已出让土地未取得建设工程规划许可证的商品住房项目,优先选择现房销售;已取得建设工程规划许可证的商品住房项目,鼓励实行现房销售。
@@ -1574,7 +1574,7 @@
       </c>
       <c r="D21" s="52" t="inlineStr">
         <is>
-          <t>【国家基准｜已采集｜明细4】
+          <t>【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：(一)推进商品住房现房销售。本通知施行之日起,新出让土地的商品住房项目和已出让土地未取得建设工程规划许可证的商品住房项目,优先选择现房销售;已取得建设工程规划许可证的商品住房项目,鼓励实行现房销售。
@@ -1583,7 +1583,7 @@
       </c>
       <c r="E21" s="52" t="inlineStr">
         <is>
-          <t>【国家基准｜已采集｜明细4】
+          <t>【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：(一)推进商品住房现房销售。本通知施行之日起,新出让土地的商品住房项目和已出让土地未取得建设工程规划许可证的商品住房项目,优先选择现房销售;已取得建设工程规划许可证的商品住房项目,鼓励实行现房销售。
@@ -1593,13 +1593,13 @@
       <c r="F21" s="54" t="inlineStr">
         <is>
           <t>三亚：
-【国家基准｜已采集｜明细4】
+【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：(一)推进商品住房现房销售。本通知施行之日起,新出让土地的商品住房项目和已出让土地未取得建设工程规划许可证的商品住房项目,优先选择现房销售;已取得建设工程规划许可证的商品住房项目,鼓励实行现房销售。
 (一)优化土地供应管理。市县要优化国土空间规划和土地利用方式,按照住房发展规划和年度计划,合理确定房地产用地供应规模。统筹规划、合理布局商品住宅用地,优化土地出让方案,可带规划方案出让。房地产开发企业须用自有资金购地,可按国家规定分期缴纳土地出让价款,具体缴纳比例和时限由市县人民政府确定。对于实行现房销售的项目,在土地出让公告中向社会公开现房销售相关信息。
 陵水：
-【国家基准｜已采集｜明细4】
+【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：(一)推进商品住房现房销售。本通知施行之日起,新出让土地的商品住房项目和已出让土地未取得建设工程规划许可证的商品住房项目,优先选择现房销售;已取得建设工程规划许可证的商品住房项目,鼓励实行现房销售。
@@ -1616,12 +1616,12 @@
       </c>
       <c r="C22" s="51" t="inlineStr">
         <is>
-          <t>【本地政策｜已采集｜明细1】
+          <t>【本地政策｜已采集｜明细5】
 2026-09-24 北京市住房和城乡建设委员会等4部门关于发布本市贯彻落实《关于完善商品住房销售制度的通知》的实施意见
 官方原文：https://zjw.beijing.gov.cn/bjjs/xxgk/zcwj2024/qtzcwj/xxyx13/744131235/index.shtml
 官方原文：https://gjj.beijing.gov.cn/web/zwgk61/2024zcwj/436433464/436433468/744131565/index.html
 原文摘录（非模型总结）：2026年8月28日起，新发布国有 建设用地 使用权出让公告的商品住房项目 优先 选择 现房销售。房地产开发企业在取得房屋首次登记后，编制现房销售方案，向房屋所在区住房城乡建设 （ 房管 ） 部门申请现房销售备案 后 ，按现房销售方案 组织 销售，所销售房屋及建设用地使用权应无抵押、查封等情形。
-【国家基准｜已采集｜明细4】
+【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：(一)推进商品住房现房销售。本通知施行之日起,新出让土地的商品住房项目和已出让土地未取得建设工程规划许可证的商品住房项目,优先选择现房销售;已取得建设工程规划许可证的商品住房项目,鼓励实行现房销售。</t>
@@ -1629,7 +1629,7 @@
       </c>
       <c r="D22" s="52" t="inlineStr">
         <is>
-          <t>【国家基准｜已采集｜明细4】
+          <t>【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：(一)推进商品住房现房销售。本通知施行之日起,新出让土地的商品住房项目和已出让土地未取得建设工程规划许可证的商品住房项目,优先选择现房销售;已取得建设工程规划许可证的商品住房项目,鼓励实行现房销售。</t>
@@ -1637,7 +1637,7 @@
       </c>
       <c r="E22" s="52" t="inlineStr">
         <is>
-          <t>【国家基准｜已采集｜明细4】
+          <t>【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：(一)推进商品住房现房销售。本通知施行之日起,新出让土地的商品住房项目和已出让土地未取得建设工程规划许可证的商品住房项目,优先选择现房销售;已取得建设工程规划许可证的商品住房项目,鼓励实行现房销售。</t>
@@ -1646,12 +1646,12 @@
       <c r="F22" s="54" t="inlineStr">
         <is>
           <t>三亚：
-【国家基准｜已采集｜明细4】
+【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：(一)推进商品住房现房销售。本通知施行之日起,新出让土地的商品住房项目和已出让土地未取得建设工程规划许可证的商品住房项目,优先选择现房销售;已取得建设工程规划许可证的商品住房项目,鼓励实行现房销售。
 陵水：
-【国家基准｜已采集｜明细4】
+【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：(一)推进商品住房现房销售。本通知施行之日起,新出让土地的商品住房项目和已出让土地未取得建设工程规划许可证的商品住房项目,优先选择现房销售;已取得建设工程规划许可证的商品住房项目,鼓励实行现房销售。</t>
@@ -1667,17 +1667,17 @@
       </c>
       <c r="C23" s="51" t="inlineStr">
         <is>
-          <t>【本地政策｜已采集｜明细1】
+          <t>【本地政策｜已采集｜明细5】
 2026-09-24 北京市住房和城乡建设委员会等4部门关于发布本市贯彻落实《关于完善商品住房销售制度的通知》的实施意见
 官方原文：https://zjw.beijing.gov.cn/bjjs/xxgk/zcwj2024/qtzcwj/xxyx13/744131235/index.shtml
 官方原文：https://gjj.beijing.gov.cn/web/zwgk61/2024zcwj/436433464/436433468/744131565/index.html
 原文摘录（非模型总结）：实行现房销售的商品住房项目，房地产开发企业可 在取得建筑工程施工许可证后， 与购房人签订购房定金合同， 一般 收取不超过总房价款1%的定金。房地产开发企业违约不能按期交房的，购房人有权按照合同约定提出解除定金合同。
 房地产开发企业在主办银行开立资金账户，项目存续期间，开发贷款、项目自有资金、现房销售资金等与项目相关的全部资金均应纳入在主办银行开立的资金账户管理。市住房资金管理中心在主办银行开立资金监管账户，用于存放监管项目预售资金和现房定金。
-【国家基准｜已采集｜明细4】
+【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：(三)推行现房销售定金制。实行现房销售的商品住房项目,在取得建筑工程施工许可证后,房地产开发企业可与购房人签订购房定金合同,依法收取少量定金。购房定金合同应约定定金金额、商品住房售价、交付时间及不能按期履约的责任等,保护双方合法权益。市县住房和城乡建设部门履行定金监管职责,住房资金监管机构承担定金监管工作,在项目的主办银行开立定金监管账户。房屋具备交付条件后,解除定金监管。房地产开发企业违约不能按期交房的,购房人有权按照合同约定提出解除定金合同,房地产开发企业依法返还定金,承担违约责任。各地要结合实际制定购房定金合同示范文本。
-【国家基准｜已采集｜明细5】
+【国家基准｜已采集｜明细9】
 2026-08-28 中国人民银行 国家金融监督管理总局印发《关于改革完善房地产信贷管理 推动加快构建房地产发展新模式的意见》的通知（银发〔2026〕171号）
 官方原文：https://hunan.gov.cn/zqt/zcsd/202609/t20260907_34058152.html
 原文摘录（非模型总结）：项目公司应在主办银行开立资金账户。项目存续期间,除按规定要求监管的预售资金、定金等外,房地产开发贷款、项目自有资金、现房销售资金等与项目相关的全部资金均应纳入在主办银行开立的资金账户管理。主办银行和资金账户在房地产开发贷款结清前原则上不得变更。
@@ -1686,11 +1686,11 @@
       </c>
       <c r="D23" s="52" t="inlineStr">
         <is>
-          <t>【国家基准｜已采集｜明细4】
+          <t>【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：(三)推行现房销售定金制。实行现房销售的商品住房项目,在取得建筑工程施工许可证后,房地产开发企业可与购房人签订购房定金合同,依法收取少量定金。购房定金合同应约定定金金额、商品住房售价、交付时间及不能按期履约的责任等,保护双方合法权益。市县住房和城乡建设部门履行定金监管职责,住房资金监管机构承担定金监管工作,在项目的主办银行开立定金监管账户。房屋具备交付条件后,解除定金监管。房地产开发企业违约不能按期交房的,购房人有权按照合同约定提出解除定金合同,房地产开发企业依法返还定金,承担违约责任。各地要结合实际制定购房定金合同示范文本。
-【国家基准｜已采集｜明细5】
+【国家基准｜已采集｜明细9】
 2026-08-28 中国人民银行 国家金融监督管理总局印发《关于改革完善房地产信贷管理 推动加快构建房地产发展新模式的意见》的通知（银发〔2026〕171号）
 官方原文：https://hunan.gov.cn/zqt/zcsd/202609/t20260907_34058152.html
 原文摘录（非模型总结）：项目公司应在主办银行开立资金账户。项目存续期间,除按规定要求监管的预售资金、定金等外,房地产开发贷款、项目自有资金、现房销售资金等与项目相关的全部资金均应纳入在主办银行开立的资金账户管理。主办银行和资金账户在房地产开发贷款结清前原则上不得变更。
@@ -1699,11 +1699,11 @@
       </c>
       <c r="E23" s="52" t="inlineStr">
         <is>
-          <t>【国家基准｜已采集｜明细4】
+          <t>【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：(三)推行现房销售定金制。实行现房销售的商品住房项目,在取得建筑工程施工许可证后,房地产开发企业可与购房人签订购房定金合同,依法收取少量定金。购房定金合同应约定定金金额、商品住房售价、交付时间及不能按期履约的责任等,保护双方合法权益。市县住房和城乡建设部门履行定金监管职责,住房资金监管机构承担定金监管工作,在项目的主办银行开立定金监管账户。房屋具备交付条件后,解除定金监管。房地产开发企业违约不能按期交房的,购房人有权按照合同约定提出解除定金合同,房地产开发企业依法返还定金,承担违约责任。各地要结合实际制定购房定金合同示范文本。
-【国家基准｜已采集｜明细5】
+【国家基准｜已采集｜明细9】
 2026-08-28 中国人民银行 国家金融监督管理总局印发《关于改革完善房地产信贷管理 推动加快构建房地产发展新模式的意见》的通知（银发〔2026〕171号）
 官方原文：https://hunan.gov.cn/zqt/zcsd/202609/t20260907_34058152.html
 原文摘录（非模型总结）：项目公司应在主办银行开立资金账户。项目存续期间,除按规定要求监管的预售资金、定金等外,房地产开发贷款、项目自有资金、现房销售资金等与项目相关的全部资金均应纳入在主办银行开立的资金账户管理。主办银行和资金账户在房地产开发贷款结清前原则上不得变更。
@@ -1713,21 +1713,21 @@
       <c r="F23" s="54" t="inlineStr">
         <is>
           <t>三亚：
-【国家基准｜已采集｜明细4】
+【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：(三)推行现房销售定金制。实行现房销售的商品住房项目,在取得建筑工程施工许可证后,房地产开发企业可与购房人签订购房定金合同,依法收取少量定金。购房定金合同应约定定金金额、商品住房售价、交付时间及不能按期履约的责任等,保护双方合法权益。市县住房和城乡建设部门履行定金监管职责,住房资金监管机构承担定金监管工作,在项目的主办银行开立定金监管账户。房屋具备交付条件后,解除定金监管。房地产开发企业违约不能按期交房的,购房人有权按照合同约定提出解除定金合同,房地产开发企业依法返还定金,承担违约责任。各地要结合实际制定购房定金合同示范文本。
-【国家基准｜已采集｜明细5】
+【国家基准｜已采集｜明细9】
 2026-08-28 中国人民银行 国家金融监督管理总局印发《关于改革完善房地产信贷管理 推动加快构建房地产发展新模式的意见》的通知（银发〔2026〕171号）
 官方原文：https://hunan.gov.cn/zqt/zcsd/202609/t20260907_34058152.html
 原文摘录（非模型总结）：项目公司应在主办银行开立资金账户。项目存续期间,除按规定要求监管的预售资金、定金等外,房地产开发贷款、项目自有资金、现房销售资金等与项目相关的全部资金均应纳入在主办银行开立的资金账户管理。主办银行和资金账户在房地产开发贷款结清前原则上不得变更。
 项目预售资金监管账户和定金账户应按规定在主办银行开立。项目公司对外负债、投资等影响金融债务安全的重大事项,应事先告知主办银行。
 陵水：
-【国家基准｜已采集｜明细4】
+【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：(三)推行现房销售定金制。实行现房销售的商品住房项目,在取得建筑工程施工许可证后,房地产开发企业可与购房人签订购房定金合同,依法收取少量定金。购房定金合同应约定定金金额、商品住房售价、交付时间及不能按期履约的责任等,保护双方合法权益。市县住房和城乡建设部门履行定金监管职责,住房资金监管机构承担定金监管工作,在项目的主办银行开立定金监管账户。房屋具备交付条件后,解除定金监管。房地产开发企业违约不能按期交房的,购房人有权按照合同约定提出解除定金合同,房地产开发企业依法返还定金,承担违约责任。各地要结合实际制定购房定金合同示范文本。
-【国家基准｜已采集｜明细5】
+【国家基准｜已采集｜明细9】
 2026-08-28 中国人民银行 国家金融监督管理总局印发《关于改革完善房地产信贷管理 推动加快构建房地产发展新模式的意见》的通知（银发〔2026〕171号）
 官方原文：https://hunan.gov.cn/zqt/zcsd/202609/t20260907_34058152.html
 原文摘录（非模型总结）：项目公司应在主办银行开立资金账户。项目存续期间,除按规定要求监管的预售资金、定金等外,房地产开发贷款、项目自有资金、现房销售资金等与项目相关的全部资金均应纳入在主办银行开立的资金账户管理。主办银行和资金账户在房地产开发贷款结清前原则上不得变更。
@@ -1927,7 +1927,7 @@
       </c>
       <c r="C31" s="51" t="inlineStr">
         <is>
-          <t>【本地政策｜已采集｜明细1】
+          <t>【本地政策｜已采集｜明细5】
 2026-09-24 北京市住房和城乡建设委员会等4部门关于发布本市贯彻落实《关于完善商品住房销售制度的通知》的实施意见
 官方原文：https://zjw.beijing.gov.cn/bjjs/xxgk/zcwj2024/qtzcwj/xxyx13/744131235/index.shtml
 官方原文：https://gjj.beijing.gov.cn/web/zwgk61/2024zcwj/436433464/436433468/744131565/index.html
@@ -2007,18 +2007,18 @@
       </c>
       <c r="C34" s="51" t="inlineStr">
         <is>
-          <t>【本地政策｜已采集｜明细1】
+          <t>【本地政策｜已采集｜明细5】
 2026-09-24 北京市住房和城乡建设委员会等4部门关于发布本市贯彻落实《关于完善商品住房销售制度的通知》的实施意见
 官方原文：https://zjw.beijing.gov.cn/bjjs/xxgk/zcwj2024/qtzcwj/xxyx13/744131235/index.shtml
 官方原文：https://gjj.beijing.gov.cn/web/zwgk61/2024zcwj/436433464/436433468/744131565/index.html
 原文摘录（非模型总结）：（一）新取得土地项目。 2026年8月28日后 新发布国有 建设用地 使用权出让公告的商品住房项目， 申请 预售 的 ，单体建筑 应 完成主体结构封顶 （楼栋顶板及楼顶构筑物、配套设施完成混凝土浇筑）， 项目 建设单位、勘察、设计、施工、监理 等单位 应出具 签字 盖章 的《主体结构分部工程验收记录》 。项目 预售资金全额 、全过程监管 ，项目 联合验收后 ， 方可 解除资金监管。 具体预售资金监管办法另行印发。
 （二）在途项目。 2026年8月28日（含）前，已取得 （含部分取得） 建设工程规划许可证但未办理预售许可的商品住房项目 ，申请 预售的，预售条件、预售资金监管等按原有政策规定执行。
-【国家基准｜已采集｜明细4】
+【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：各地要规范商品住房预售条件,加强预售资金监管,保障预售资金安全,有效防范商品住房交付风险,维护购房人合法权益。
 (二)加强预售资金监管。市县住房和城乡建设部门履行预售资金监管职责,由住房资金监管机构承担具体监管工作。住房资金监管机构应与房地产开发企业签订资金监管协议,并在项目的主办银行开立资金监管账户。购房人支付的首付款、个人住房贷款等购房资金应全部存入资金监管账户。商品住房项目竣工验收、水电气热等配套设施具备交付条件后,解除资金监管。房地产开发企业违约不能按期交房的,购房人有权按照合同约定提出解除购房合同,房地产开发企业须按照合同约定退还购房资金并承担违约责任。房地产开发企业应与购房人在购房合同中约定购房资金存入资金监管账户的相关权利责任。
-【国家基准｜已采集｜明细5】
+【国家基准｜已采集｜明细9】
 2026-08-28 中国人民银行 国家金融监督管理总局印发《关于改革完善房地产信贷管理 推动加快构建房地产发展新模式的意见》的通知（银发〔2026〕171号）
 官方原文：https://hunan.gov.cn/zqt/zcsd/202609/t20260907_34058152.html
 原文摘录（非模型总结）：项目公司应在主办银行开立资金账户。项目存续期间,除按规定要求监管的预售资金、定金等外,房地产开发贷款、项目自有资金、现房销售资金等与项目相关的全部资金均应纳入在主办银行开立的资金账户管理。主办银行和资金账户在房地产开发贷款结清前原则上不得变更。
@@ -2027,12 +2027,12 @@
       </c>
       <c r="D34" s="51" t="inlineStr">
         <is>
-          <t>【国家基准｜已采集｜明细4】
+          <t>【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：各地要规范商品住房预售条件,加强预售资金监管,保障预售资金安全,有效防范商品住房交付风险,维护购房人合法权益。
 (二)加强预售资金监管。市县住房和城乡建设部门履行预售资金监管职责,由住房资金监管机构承担具体监管工作。住房资金监管机构应与房地产开发企业签订资金监管协议,并在项目的主办银行开立资金监管账户。购房人支付的首付款、个人住房贷款等购房资金应全部存入资金监管账户。商品住房项目竣工验收、水电气热等配套设施具备交付条件后,解除资金监管。房地产开发企业违约不能按期交房的,购房人有权按照合同约定提出解除购房合同,房地产开发企业须按照合同约定退还购房资金并承担违约责任。房地产开发企业应与购房人在购房合同中约定购房资金存入资金监管账户的相关权利责任。
-【国家基准｜已采集｜明细5】
+【国家基准｜已采集｜明细9】
 2026-08-28 中国人民银行 国家金融监督管理总局印发《关于改革完善房地产信贷管理 推动加快构建房地产发展新模式的意见》的通知（银发〔2026〕171号）
 官方原文：https://hunan.gov.cn/zqt/zcsd/202609/t20260907_34058152.html
 原文摘录（非模型总结）：项目公司应在主办银行开立资金账户。项目存续期间,除按规定要求监管的预售资金、定金等外,房地产开发贷款、项目自有资金、现房销售资金等与项目相关的全部资金均应纳入在主办银行开立的资金账户管理。主办银行和资金账户在房地产开发贷款结清前原则上不得变更。
@@ -2041,12 +2041,12 @@
       </c>
       <c r="E34" s="52" t="inlineStr">
         <is>
-          <t>【国家基准｜已采集｜明细4】
+          <t>【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：各地要规范商品住房预售条件,加强预售资金监管,保障预售资金安全,有效防范商品住房交付风险,维护购房人合法权益。
 (二)加强预售资金监管。市县住房和城乡建设部门履行预售资金监管职责,由住房资金监管机构承担具体监管工作。住房资金监管机构应与房地产开发企业签订资金监管协议,并在项目的主办银行开立资金监管账户。购房人支付的首付款、个人住房贷款等购房资金应全部存入资金监管账户。商品住房项目竣工验收、水电气热等配套设施具备交付条件后,解除资金监管。房地产开发企业违约不能按期交房的,购房人有权按照合同约定提出解除购房合同,房地产开发企业须按照合同约定退还购房资金并承担违约责任。房地产开发企业应与购房人在购房合同中约定购房资金存入资金监管账户的相关权利责任。
-【国家基准｜已采集｜明细5】
+【国家基准｜已采集｜明细9】
 2026-08-28 中国人民银行 国家金融监督管理总局印发《关于改革完善房地产信贷管理 推动加快构建房地产发展新模式的意见》的通知（银发〔2026〕171号）
 官方原文：https://hunan.gov.cn/zqt/zcsd/202609/t20260907_34058152.html
 原文摘录（非模型总结）：项目公司应在主办银行开立资金账户。项目存续期间,除按规定要求监管的预售资金、定金等外,房地产开发贷款、项目自有资金、现房销售资金等与项目相关的全部资金均应纳入在主办银行开立的资金账户管理。主办银行和资金账户在房地产开发贷款结清前原则上不得变更。
@@ -2056,23 +2056,23 @@
       <c r="F34" s="54" t="inlineStr">
         <is>
           <t>三亚：
-【国家基准｜已采集｜明细4】
+【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：各地要规范商品住房预售条件,加强预售资金监管,保障预售资金安全,有效防范商品住房交付风险,维护购房人合法权益。
 (二)加强预售资金监管。市县住房和城乡建设部门履行预售资金监管职责,由住房资金监管机构承担具体监管工作。住房资金监管机构应与房地产开发企业签订资金监管协议,并在项目的主办银行开立资金监管账户。购房人支付的首付款、个人住房贷款等购房资金应全部存入资金监管账户。商品住房项目竣工验收、水电气热等配套设施具备交付条件后,解除资金监管。房地产开发企业违约不能按期交房的,购房人有权按照合同约定提出解除购房合同,房地产开发企业须按照合同约定退还购房资金并承担违约责任。房地产开发企业应与购房人在购房合同中约定购房资金存入资金监管账户的相关权利责任。
-【国家基准｜已采集｜明细5】
+【国家基准｜已采集｜明细9】
 2026-08-28 中国人民银行 国家金融监督管理总局印发《关于改革完善房地产信贷管理 推动加快构建房地产发展新模式的意见》的通知（银发〔2026〕171号）
 官方原文：https://hunan.gov.cn/zqt/zcsd/202609/t20260907_34058152.html
 原文摘录（非模型总结）：项目公司应在主办银行开立资金账户。项目存续期间,除按规定要求监管的预售资金、定金等外,房地产开发贷款、项目自有资金、现房销售资金等与项目相关的全部资金均应纳入在主办银行开立的资金账户管理。主办银行和资金账户在房地产开发贷款结清前原则上不得变更。
 项目预售资金监管账户和定金账户应按规定在主办银行开立。项目公司对外负债、投资等影响金融债务安全的重大事项,应事先告知主办银行。
 陵水：
-【国家基准｜已采集｜明细4】
+【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：各地要规范商品住房预售条件,加强预售资金监管,保障预售资金安全,有效防范商品住房交付风险,维护购房人合法权益。
 (二)加强预售资金监管。市县住房和城乡建设部门履行预售资金监管职责,由住房资金监管机构承担具体监管工作。住房资金监管机构应与房地产开发企业签订资金监管协议,并在项目的主办银行开立资金监管账户。购房人支付的首付款、个人住房贷款等购房资金应全部存入资金监管账户。商品住房项目竣工验收、水电气热等配套设施具备交付条件后,解除资金监管。房地产开发企业违约不能按期交房的,购房人有权按照合同约定提出解除购房合同,房地产开发企业须按照合同约定退还购房资金并承担违约责任。房地产开发企业应与购房人在购房合同中约定购房资金存入资金监管账户的相关权利责任。
-【国家基准｜已采集｜明细5】
+【国家基准｜已采集｜明细9】
 2026-08-28 中国人民银行 国家金融监督管理总局印发《关于改革完善房地产信贷管理 推动加快构建房地产发展新模式的意见》的通知（银发〔2026〕171号）
 官方原文：https://hunan.gov.cn/zqt/zcsd/202609/t20260907_34058152.html
 原文摘录（非模型总结）：项目公司应在主办银行开立资金账户。项目存续期间,除按规定要求监管的预售资金、定金等外,房地产开发贷款、项目自有资金、现房销售资金等与项目相关的全部资金均应纳入在主办银行开立的资金账户管理。主办银行和资金账户在房地产开发贷款结清前原则上不得变更。
@@ -2155,7 +2155,7 @@
       </c>
       <c r="C37" s="51" t="inlineStr">
         <is>
-          <t>原始发布日期 1900-01-01—2026-09-30（含首尾）；官方出处及完整证据见政策明细。</t>
+          <t>原始发布日期 1900-01-01—2026-10-13（含首尾）；官方出处及完整证据见政策明细。</t>
         </is>
       </c>
       <c r="D37" s="20" t="n"/>
@@ -2285,7 +2285,7 @@
       </c>
       <c r="C42" s="50" t="inlineStr">
         <is>
-          <t>原始发布日期 1900-01-01—2026-09-30（含首尾）；官方出处及完整证据见政策明细。</t>
+          <t>原始发布日期 1900-01-01—2026-10-13（含首尾）；官方出处及完整证据见政策明细。</t>
         </is>
       </c>
       <c r="D42" s="44" t="n"/>
@@ -2347,16 +2347,16 @@
       </c>
       <c r="C45" s="52" t="inlineStr">
         <is>
-          <t>【本地政策｜已采集｜明细1】
+          <t>【本地政策｜已采集｜明细5】
 2026-09-24 北京市住房和城乡建设委员会等4部门关于发布本市贯彻落实《关于完善商品住房销售制度的通知》的实施意见
 官方原文：https://zjw.beijing.gov.cn/bjjs/xxgk/zcwj2024/qtzcwj/xxyx13/744131235/index.shtml
 官方原文：https://gjj.beijing.gov.cn/web/zwgk61/2024zcwj/436433464/436433468/744131565/index.html
 原文摘录（非模型总结）：2026年8月28日后签订开发贷合同的商品住房项目，贷款银行单独提供开发贷的，贷款银行为主办银行；贷款银行组建银团提供贷款的， 银团贷款牵头银行为主办银行 。
-【国家基准｜已采集｜明细4】
+【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：(二)加大融资支持力度。房地产项目实行主办银行制,房地产项目开发公司和主办银行双向选择,一个项目确定一家主办银行,主办银行单独或牵头组建银团提供开发贷款等融资服务。房地产项目开发公司以土地使用权抵押申请开发贷款的,应以分户土地使用权集合设定抵押,相关办法另行制定。支持房地产项目开发公司通过股权、债券等多种方式开展融资。对实行现房销售和预售的项目,按照市场化原则满足项目合理融资需求,实现开发贷款发放与项目建设周期相匹配。
-【国家基准｜已采集｜明细5】
+【国家基准｜已采集｜明细9】
 2026-08-28 中国人民银行 国家金融监督管理总局印发《关于改革完善房地产信贷管理 推动加快构建房地产发展新模式的意见》的通知（银发〔2026〕171号）
 官方原文：https://hunan.gov.cn/zqt/zcsd/202609/t20260907_34058152.html
 原文摘录（非模型总结）：第十二条 房地产开发贷款实行主办银行制,单个房地产项目对应一家银行作为主办银行(单家贷款行或银团贷款牵头行),对项目资金进行封闭管理。</t>
@@ -2364,11 +2364,11 @@
       </c>
       <c r="D45" s="52" t="inlineStr">
         <is>
-          <t>【国家基准｜已采集｜明细4】
+          <t>【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：(二)加大融资支持力度。房地产项目实行主办银行制,房地产项目开发公司和主办银行双向选择,一个项目确定一家主办银行,主办银行单独或牵头组建银团提供开发贷款等融资服务。房地产项目开发公司以土地使用权抵押申请开发贷款的,应以分户土地使用权集合设定抵押,相关办法另行制定。支持房地产项目开发公司通过股权、债券等多种方式开展融资。对实行现房销售和预售的项目,按照市场化原则满足项目合理融资需求,实现开发贷款发放与项目建设周期相匹配。
-【国家基准｜已采集｜明细5】
+【国家基准｜已采集｜明细9】
 2026-08-28 中国人民银行 国家金融监督管理总局印发《关于改革完善房地产信贷管理 推动加快构建房地产发展新模式的意见》的通知（银发〔2026〕171号）
 官方原文：https://hunan.gov.cn/zqt/zcsd/202609/t20260907_34058152.html
 原文摘录（非模型总结）：第十二条 房地产开发贷款实行主办银行制,单个房地产项目对应一家银行作为主办银行(单家贷款行或银团贷款牵头行),对项目资金进行封闭管理。</t>
@@ -2376,11 +2376,11 @@
       </c>
       <c r="E45" s="52" t="inlineStr">
         <is>
-          <t>【国家基准｜已采集｜明细4】
+          <t>【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：(二)加大融资支持力度。房地产项目实行主办银行制,房地产项目开发公司和主办银行双向选择,一个项目确定一家主办银行,主办银行单独或牵头组建银团提供开发贷款等融资服务。房地产项目开发公司以土地使用权抵押申请开发贷款的,应以分户土地使用权集合设定抵押,相关办法另行制定。支持房地产项目开发公司通过股权、债券等多种方式开展融资。对实行现房销售和预售的项目,按照市场化原则满足项目合理融资需求,实现开发贷款发放与项目建设周期相匹配。
-【国家基准｜已采集｜明细5】
+【国家基准｜已采集｜明细9】
 2026-08-28 中国人民银行 国家金融监督管理总局印发《关于改革完善房地产信贷管理 推动加快构建房地产发展新模式的意见》的通知（银发〔2026〕171号）
 官方原文：https://hunan.gov.cn/zqt/zcsd/202609/t20260907_34058152.html
 原文摘录（非模型总结）：第十二条 房地产开发贷款实行主办银行制,单个房地产项目对应一家银行作为主办银行(单家贷款行或银团贷款牵头行),对项目资金进行封闭管理。</t>
@@ -2389,20 +2389,20 @@
       <c r="F45" s="52" t="inlineStr">
         <is>
           <t>三亚：
-【国家基准｜已采集｜明细4】
+【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：(二)加大融资支持力度。房地产项目实行主办银行制,房地产项目开发公司和主办银行双向选择,一个项目确定一家主办银行,主办银行单独或牵头组建银团提供开发贷款等融资服务。房地产项目开发公司以土地使用权抵押申请开发贷款的,应以分户土地使用权集合设定抵押,相关办法另行制定。支持房地产项目开发公司通过股权、债券等多种方式开展融资。对实行现房销售和预售的项目,按照市场化原则满足项目合理融资需求,实现开发贷款发放与项目建设周期相匹配。
-【国家基准｜已采集｜明细5】
+【国家基准｜已采集｜明细9】
 2026-08-28 中国人民银行 国家金融监督管理总局印发《关于改革完善房地产信贷管理 推动加快构建房地产发展新模式的意见》的通知（银发〔2026〕171号）
 官方原文：https://hunan.gov.cn/zqt/zcsd/202609/t20260907_34058152.html
 原文摘录（非模型总结）：第十二条 房地产开发贷款实行主办银行制,单个房地产项目对应一家银行作为主办银行(单家贷款行或银团贷款牵头行),对项目资金进行封闭管理。
 陵水：
-【国家基准｜已采集｜明细4】
+【国家基准｜已采集｜明细8】
 2026-08-28 住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知
 官方原文：https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html
 原文摘录（非模型总结）：(二)加大融资支持力度。房地产项目实行主办银行制,房地产项目开发公司和主办银行双向选择,一个项目确定一家主办银行,主办银行单独或牵头组建银团提供开发贷款等融资服务。房地产项目开发公司以土地使用权抵押申请开发贷款的,应以分户土地使用权集合设定抵押,相关办法另行制定。支持房地产项目开发公司通过股权、债券等多种方式开展融资。对实行现房销售和预售的项目,按照市场化原则满足项目合理融资需求,实现开发贷款发放与项目建设周期相匹配。
-【国家基准｜已采集｜明细5】
+【国家基准｜已采集｜明细9】
 2026-08-28 中国人民银行 国家金融监督管理总局印发《关于改革完善房地产信贷管理 推动加快构建房地产发展新模式的意见》的通知（银发〔2026〕171号）
 官方原文：https://hunan.gov.cn/zqt/zcsd/202609/t20260907_34058152.html
 原文摘录（非模型总结）：第十二条 房地产开发贷款实行主办银行制,单个房地产项目对应一家银行作为主办银行(单家贷款行或银团贷款牵头行),对项目资金进行封闭管理。</t>
@@ -2420,7 +2420,7 @@
       </c>
       <c r="C46" s="52" t="inlineStr">
         <is>
-          <t>【本地政策｜已采集｜明细1】
+          <t>【本地政策｜已采集｜明细5】
 2026-09-24 北京市住房和城乡建设委员会等4部门关于发布本市贯彻落实《关于完善商品住房销售制度的通知》的实施意见
 官方原文：https://zjw.beijing.gov.cn/bjjs/xxgk/zcwj2024/qtzcwj/xxyx13/744131235/index.shtml
 官方原文：https://gjj.beijing.gov.cn/web/zwgk61/2024zcwj/436433464/436433468/744131565/index.html
@@ -2492,7 +2492,7 @@
       </c>
       <c r="C48" s="49" t="inlineStr">
         <is>
-          <t>原始发布日期 1900-01-01—2026-09-30（含首尾）；官方出处及完整证据见政策明细。</t>
+          <t>原始发布日期 1900-01-01—2026-10-13（含首尾）；官方出处及完整证据见政策明细。</t>
         </is>
       </c>
       <c r="D48" s="45" t="n"/>
@@ -2548,7 +2548,7 @@
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader/>
-    <oddFooter>&amp;C原发日期 1900-01-01 至 2026-09-30（含两端）&amp;R第 &amp;P 页 / 共 &amp;N 页</oddFooter>
+    <oddFooter>&amp;C原发日期 1900-01-01 至 2026-10-13（含两端）&amp;R第 &amp;P 页 / 共 &amp;N 页</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -2614,7 +2614,7 @@
       </c>
       <c r="B2" s="59" t="inlineStr">
         <is>
-          <t>【国家基准｜已采集｜明细6】
+          <t>【国家基准｜已采集｜明细10】
 2026-08-18 国务院关于修改《住房公积金管理条例》的决定
 官方原文：https://www.changzhi.gov.cn/xxgkml/zfxxgkml/szfzssydw/czszfgjj/gkgd_202/202608/t20260825_3199027.shtml
 官方原文：https://www.sjzgjj.cn/gjjwj/2486.jhtml
@@ -2623,7 +2623,7 @@
       </c>
       <c r="C2" s="59" t="inlineStr">
         <is>
-          <t>【国家基准｜已采集｜明细6】
+          <t>【国家基准｜已采集｜明细10】
 2026-08-18 国务院关于修改《住房公积金管理条例》的决定
 官方原文：https://www.changzhi.gov.cn/xxgkml/zfxxgkml/szfzssydw/czszfgjj/gkgd_202/202608/t20260825_3199027.shtml
 官方原文：https://www.sjzgjj.cn/gjjwj/2486.jhtml
@@ -2632,7 +2632,7 @@
       </c>
       <c r="D2" s="59" t="inlineStr">
         <is>
-          <t>【本地政策｜已采集｜明细2】
+          <t>【本地政策｜已采集｜明细6】
 2026-09-18 关于调整住房公积金贷款有关政策的通知
 官方原文：https://www.sjzgjj.cn/tzgg/2489.jhtml
 原文摘录（非模型总结）：1
@@ -2679,7 +2679,7 @@
 统计。 
 （二）缴存人家庭购买非住宅建设用地上住房申请公积金
 贷款的，贷款额度不超过房屋总价的50%。
-【国家基准｜已采集｜明细6】
+【国家基准｜已采集｜明细10】
 2026-08-18 国务院关于修改《住房公积金管理条例》的决定
 官方原文：https://www.changzhi.gov.cn/xxgkml/zfxxgkml/szfzssydw/czszfgjj/gkgd_202/202608/t20260825_3199027.shtml
 官方原文：https://www.sjzgjj.cn/gjjwj/2486.jhtml
@@ -2688,7 +2688,7 @@
       </c>
       <c r="E2" s="59" t="inlineStr">
         <is>
-          <t>【国家基准｜已采集｜明细6】
+          <t>【国家基准｜已采集｜明细10】
 2026-08-18 国务院关于修改《住房公积金管理条例》的决定
 官方原文：https://www.changzhi.gov.cn/xxgkml/zfxxgkml/szfzssydw/czszfgjj/gkgd_202/202608/t20260825_3199027.shtml
 官方原文：https://www.sjzgjj.cn/gjjwj/2486.jhtml
@@ -2697,7 +2697,7 @@
       </c>
       <c r="F2" s="59" t="inlineStr">
         <is>
-          <t>【国家基准｜已采集｜明细6】
+          <t>【国家基准｜已采集｜明细10】
 2026-08-18 国务院关于修改《住房公积金管理条例》的决定
 官方原文：https://www.changzhi.gov.cn/xxgkml/zfxxgkml/szfzssydw/czszfgjj/gkgd_202/202608/t20260825_3199027.shtml
 官方原文：https://www.sjzgjj.cn/gjjwj/2486.jhtml
@@ -2723,7 +2723,7 @@
       </c>
       <c r="D3" s="59" t="inlineStr">
         <is>
-          <t>【本地政策｜已采集｜明细2】
+          <t>【本地政策｜已采集｜明细6】
 2026-09-18 关于调整住房公积金贷款有关政策的通知
 官方原文：https://www.sjzgjj.cn/tzgg/2489.jhtml
 原文摘录（非模型总结）：2
@@ -2780,7 +2780,7 @@
       </c>
       <c r="D4" s="59" t="inlineStr">
         <is>
-          <t>【本地政策｜已采集｜明细3】
+          <t>【本地政策｜已采集｜明细7】
 2026-09-18 关于开展装修提取住房公积金业务的通知
 官方原文：https://www.sjzgjj.cn/tzgg/2488.jhtml
 原文摘录（非模型总结）：石家庄住房公积金管理中心关于开展装修提取住房公积金业务的通知.pdf
@@ -2835,7 +2835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:M59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2920,39 +2920,2217 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="409" customHeight="1">
+    <row r="2" ht="55" customHeight="1">
       <c r="A2" s="60" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="60" t="inlineStr">
         <is>
+          <t>关于转发《海南省财政厅 海南省住房和城乡建设厅 海南省自然资源和规划厅关于城市基础设施配套费有关事项的补充通知》的函</t>
+        </is>
+      </c>
+      <c r="C2" s="60" t="inlineStr">
+        <is>
+          <t>三亚</t>
+        </is>
+      </c>
+      <c r="D2" s="60" t="inlineStr">
+        <is>
+          <t>住建 / 房管</t>
+        </is>
+      </c>
+      <c r="E2" s="61" t="n">
+        <v>46305</v>
+      </c>
+      <c r="F2" s="60" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G2" s="60" t="inlineStr">
+        <is>
+          <t>正式文件</t>
+        </is>
+      </c>
+      <c r="H2" s="60" t="inlineStr">
+        <is>
+          <t>未关联监测事项</t>
+        </is>
+      </c>
+      <c r="I2" s="60" t="inlineStr">
+        <is>
+          <t>待补齐正文；未生成政策摘要</t>
+        </is>
+      </c>
+      <c r="J2" s="60" t="inlineStr"/>
+      <c r="K2" s="60" t="inlineStr">
+        <is>
+          <t>https://zj.sanya.gov.cn/zjjsite/tzgg/202610/3033d8a087614eeab8d78e1c871f0c7d.shtml</t>
+        </is>
+      </c>
+      <c r="L2" s="60" t="inlineStr">
+        <is>
+          <t>待补齐正文</t>
+        </is>
+      </c>
+      <c r="M2" s="60" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="409" customHeight="1">
+      <c r="A3" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="62" t="inlineStr">
+        <is>
+          <t>市住房城乡建设委市财政局关于印发进一步规范公有住房出售收入管理实施意见的通知</t>
+        </is>
+      </c>
+      <c r="C3" s="62" t="inlineStr">
+        <is>
+          <t>天津</t>
+        </is>
+      </c>
+      <c r="D3" s="62" t="inlineStr">
+        <is>
+          <t>住建 / 房管</t>
+        </is>
+      </c>
+      <c r="E3" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F3" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G3" s="62" t="inlineStr">
+        <is>
+          <t>正式文件</t>
+        </is>
+      </c>
+      <c r="H3" s="62" t="inlineStr">
+        <is>
+          <t>未关联监测事项</t>
+        </is>
+      </c>
+      <c r="I3" s="62" t="inlineStr">
+        <is>
+          <t>原文摘录（非模型总结）
+为继续做好本市公有住房出售收入管理工作，市住房城乡建设委和市财政局对现行公有住房出售收入管理文件进行整合，制定了《关于进一步规范公有住房出售收入管理的实施意见》。现印发给你们，请遵照执行。
+为加强公有住房出售收入管理，提高资金使用效能，确保公有住房出售收入依法归集使用和资金安全，结合工作实际，制定本意见。</t>
+        </is>
+      </c>
+      <c r="J3" s="62" t="inlineStr">
+        <is>
+          <t>原文依据：各有关单位：
+原文依据：为继续做好本市公有住房出售收入管理工作，市住房城乡建设委和市财政局对现行公有住房出售收入管理文件进行整合，制定了《关于进一步规范公有住房出售收入管理的实施意见》。现印发给你们，请遵照执行。
+原文依据：市住房城乡建设委 市财政局
+原文依据：2026年9月29日
+原文依据：关于进一步规范公有住房出售收入 管理的实施意见
+原文依据：为加强公有住房出售收入管理，提高资金使用效能，确保公有住房出售收入依法归集使用和资金安全，结合工作实际，制定本意见。
+原文依据：一、管理部门
+原文依据：市住房城乡建设委负责全市公有住房出售收入集中管理的政策制定、业务指导。市住房保障服务中心（以下简称“市住保中心”）负责全市公有住房出售收入集中管理账户的核算等相关工作。
+原文依据：二、资金分配比例和用途
+原文依据：（一）专项维修资金
+原文依据：公有住房出售收入提取24.4%的资金，与个人按照购房款1%交纳的资金，共25.4%建立公房售后专项维修资金，其中：11%用于售后公有住房共用部位、共用设施设备保修期满后的维修；14.4%用于售后公有住房共用部位、共用设施设备保修期满后的更新改造；高层住宅再按照每建筑平方米提取100元，用于电梯、水泵的更新改造。
+原文依据：（二）住房基金
+原文依据：公有住房出售收入剩余资金（75.6%）建立住房基金。
+原文依据：其中，5.6%建立应急抢险资金，主要用于售后公有住房的应急抢险，也可用于小区维修和完善小区配套设施等。直管公产住房应急抢险资金由各区直管公产住房管理单位统筹使用，保管自修和单位产公有住房应急抢险资金由各售房单位使用。
+原文依据：70%的资金根据公有住房管理类型，按照以下比例分配和使用：
+原文依据：1.市内六区直管公产住房
+原文依据：全部资金上交市财政，其中：43%房屋管理储备资金用于房屋管理单位转换经营机制、住房保障和房屋管理等相关工作；25%维保改造资金用于直管公房售前维修及售后保修，以及严重损坏直管公房的安全监测、翻建、加固修缮及维修期内住户安置周转费等；2%售房经费用于市、区直管公产住房管理单位出售公有住房工作经费。25%维保改造资金、2%售房经费由市房管中心统筹使用。
+原文依据：2.其他区直管公产住房
+原文依据：全部留归区直管公产住房管理单位，参照市内六区直管公产住房资金分</t>
+        </is>
+      </c>
+      <c r="K3" s="62" t="inlineStr">
+        <is>
+          <t>https://zfcxjs.tj.gov.cn/xxgk_70/zcwj/wfwj/zcxwj/202609/t20260930_7386592.html</t>
+        </is>
+      </c>
+      <c r="L3" s="62" t="inlineStr">
+        <is>
+          <t>待关联事项</t>
+        </is>
+      </c>
+      <c r="M3" s="62" t="inlineStr">
+        <is>
+          <t>1/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="409" customHeight="1">
+      <c r="A4" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="62" t="inlineStr"/>
+      <c r="C4" s="62" t="inlineStr"/>
+      <c r="D4" s="62" t="inlineStr"/>
+      <c r="E4" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F4" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G4" s="62" t="inlineStr"/>
+      <c r="H4" s="62" t="inlineStr"/>
+      <c r="I4" s="62" t="inlineStr"/>
+      <c r="J4" s="62" t="inlineStr">
+        <is>
+          <t>配比例和用途使用。
+原文依据：3.保管自修直管公产住房
+原文依据：9%的资金上交市财政，作为房管事业发展基金，用于市房管中心管理保管自修房产工作经费；61%的资金留归售房单位，其中：59%用于保管自修直管公产住房售前维修及售后保修、住房货币分配，以及严重损坏住房的安全监测、翻建、加固修缮及维修期内住户安置周转费等，2%作为售房经费。
+原文依据：4.单位产公有住房
+原文依据：全部留归售房单位，68%用于单位住房售前维修及售后保修、住房货币分配、房屋管理单位转换经营机制，以及严重损坏公有住房的安全监测、翻建、加固修缮及维修期内住户安置周转费等；2%作为售房经费。
+原文依据：三、审核部门
+原文依据：市内六区直管公产住房售后专项维修资金和住房基金中应急抢险资金的使用，由各区直管公产住房管理单位初审，市房产管理服务中心（以下简称“市房管中心”）审核；住房基金中上交市财政资金的使用，按照财政资金使用程序由市住房城乡建设委审核。市内六区保管自修直管公产住房出售收入的使用，由市房管中心审核。其他区直管公产住房（含保管自修直管公产住房）出售收入的使用，由区住房建设委审核。单位产公有住房出售收入的使用，由房屋坐落区住房建设委审核。
+原文依据：四、账户管理
+原文依据：公有住房出售收入以专用账户和直接收付为基础，严格执行总收支账户集中核算制度，统一核算各项收入和支出，确保资金安全完整。所有专用账户由市住保中心开设，经市住房城乡建设委集中批准后报市财政局备案。
+原文依据：（一）承办银行
+原文依据：承办银行负责办理公有住房出售收入归集、支付、结息、对账和查询等金融业务。
+原文依据：（二）账户设置
+原文依据：市住保中心在承办银行设立公房售后专项维修资金和住房基金本金及利息账户，集中核算收入和支出；承办银行下设的经办网点设立公房售后专项维修资金和住房基金代收账户。
+原文依据：承办银行在公房售后专项维修资金、住房基金存款专户下为售房单位设立单位存款分户。在公房售后专项维修资金单位存款分户下设11%维修资金、14.4%更新改造资金和电梯水泵更新改造资金明细账，记账到每套住房。
+原文依据：售房单位在使用公有住房出售收入前，应当到承办银行开立售房款专户作为支出账户。
+原文依据：（三）清理撤销所有自行开设的账户
+原文依据：按照“单一账户，集中收付”的要求，各售房单位应当对未集</t>
+        </is>
+      </c>
+      <c r="K4" s="62" t="inlineStr"/>
+      <c r="L4" s="62" t="inlineStr"/>
+      <c r="M4" s="62" t="inlineStr">
+        <is>
+          <t>2/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="409" customHeight="1">
+      <c r="A5" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="62" t="inlineStr"/>
+      <c r="C5" s="62" t="inlineStr"/>
+      <c r="D5" s="62" t="inlineStr"/>
+      <c r="E5" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F5" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G5" s="62" t="inlineStr"/>
+      <c r="H5" s="62" t="inlineStr"/>
+      <c r="I5" s="62" t="inlineStr"/>
+      <c r="J5" s="62" t="inlineStr">
+        <is>
+          <t>中管理的公有住房出售收入账户进行清理，将余额纳入集中管理。
+原文依据：五、增值收益管理
+原文依据：（一）利息结算
+原文依据：公房售后专项维修资金利息，按照一年定期存款利率计息；住房基金利息，归集当年按照活期利率计息，转年按照协定存款利率计息。
+原文依据：利息每年结算一次，结息日为每年6月30日，按照承办银行结息当日利率结息。利息分别计入账户，转作维修资金和住房基金滚存使用。
+原文依据：（二）增值收益使用
+原文依据：集中管理的公有住房出售收入在合理确定使用准备金后，对其余资金采取定期存款等方式增值。公房售后专项维修资金产生的增值收益，除核定管理费外，其余转作维修资金滚存使用；住房基金产生的增值收益上交市财政，专项用于住房保障、房屋管理等相关工作。
+原文依据：六、工作要求
+原文依据：公有住房出售收入在专用账户内缴存和使用资金，各管理部门、售房单位和承办银行应当建立健全内部控制制度和约束机制，全面规范资金缴存和支出管理程序，认真做好风险防范工作，创建科学规范、监督制衡、管理有序的资金管理和运行程序。
+原文依据：（一）严格账户封闭管理
+原文依据：公有住房出售收入支出应当封闭在专用账户之内，防止收入和支出逸出专用账户的情况发生。
+原文依据：（二）严格拨款管理
+原文依据：公有住房出售收入的申请拨付应当按照用款计划办理，并严格按照《天津市公有住房出售收入管理操作程序》（见附件）执行。
+原文依据：使用公有住房出售收入应当履行审核程序。审核部门应当由经办人员和负责人两人审核签章。市住保中心向银行出具的支付凭证，100万元以上（含100万元）的资金申请应当经出纳、会计、稽核三人审核；100万元以下的资金应当经出纳、会计两人审核。
+原文依据：各审核单位以及承办银行应当对公有住房出售收入支付过程中存在的申请手续不全、用途不明、印章不清、凭证填制不规范等任何一个风险环节和可疑问题提出质疑并拒绝支付，经核实确认无误后再行支付。
+原文依据：（三）严格内部控制
+原文依据：公有住房出售收入管理部门、售房单位和承办银行应当建立健全资金管理岗位人员配置、财务人员定期交流轮岗、实地核查银行账户资金、资金支付动账提醒、实有资金账户监管以及会计档案、印鉴和票据管理等各项管理制度，建立标准化业务操作规程，定期开展资金安全核查工作，为资金全程控制、安全完整和规范运行提供强有力的内部</t>
+        </is>
+      </c>
+      <c r="K5" s="62" t="inlineStr"/>
+      <c r="L5" s="62" t="inlineStr"/>
+      <c r="M5" s="62" t="inlineStr">
+        <is>
+          <t>3/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="409" customHeight="1">
+      <c r="A6" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="62" t="inlineStr"/>
+      <c r="C6" s="62" t="inlineStr"/>
+      <c r="D6" s="62" t="inlineStr"/>
+      <c r="E6" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F6" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G6" s="62" t="inlineStr"/>
+      <c r="H6" s="62" t="inlineStr"/>
+      <c r="I6" s="62" t="inlineStr"/>
+      <c r="J6" s="62" t="inlineStr">
+        <is>
+          <t>控制。
+原文依据：（四）严格财政资金使用管理
+原文依据：使用上交市财政部分资金，相关支出控制在上缴额度内，由市住房城乡建设委按照政策确定用途将年度资金需求报市财政局，市财政局按程序将支出需求编入年度部门预算，预算执行中由市住房城乡建设委提出资金使用申请并按照原渠道拨付使用。
+原文依据：七、 本意见适用于市级直管公产住房（含保管自修）和单位产公有住房，区级直管公产住房（含保管自修）出售收入管理和使用参照执行。
+原文依据：本实施意见自印发之日起施行，有效期五年。《市国土房管局市财政局关于调整公有住房出售收入分配比例的通知》（津国土房保〔2015〕38号）同时废止。
+原文依据：附件：天津市公有住房出售收入管理操作程序
+原文依据：附件：
+原文依据：关于进一步规范公有住房出售收入
+原文依据：管理的实施意见
+原文依据：住房基金
+原文依据：七、本意见适用于市级直管公产住房（含保管自修）和单位产公有住房，区级直管公产住房（含保管自修）出售收入管理和使用参照执行。
+原文依据：附件
+原文依据：天津市公有住房出售收入管理操作程序
+原文依据：为规范公有住房出售收入归集使用业务流程，确保资金安全，提高办事效率，现就公有住房出售收入管理操作程序规定如下：
+原文依据：一、公有住房出售收入的归集
+原文依据：（一）开户
+原文依据：单位出售公有住房时，持公有住房出售批准书或其他相关证明材料及复印件到承办银行领取并填写“天津市公有住房出售收入开户登记表”（以下简称“开户登记表”，见附1）一式四联。承办银行在“开户登记表”上填写售房单位代码、开户日期，并留存相关证明材料复印件。
+原文依据：（二）缴存
+原文依据：1.新缴存的公有住房出售收入
+原文依据：（1）领取《天津市公有住房出售收入交款单》（以下简称“交款单”，见附2）。单位售房前，到区住建委领取“交款单”。
+原文依据：（2）交款。个人购买公有住房时，售房单位填写“交款单”，注明各类资金金额，购房人连同全部售房款交承办银行。
+原文依据：（3）银行受理。购房人持“交款单”到承办银行缴款，承办银行开具公有住房出售“天津市财政票据”（以下简称“售房票据”，见附3）。
+原文依据：（4）单据交接。承办银行每周将“售房票据”交市住保中心。
+原文依据：（5）记账。市住保中心根据“售房票据”记账。
+原文依据：2.存量公有住</t>
+        </is>
+      </c>
+      <c r="K6" s="62" t="inlineStr"/>
+      <c r="L6" s="62" t="inlineStr"/>
+      <c r="M6" s="62" t="inlineStr">
+        <is>
+          <t>4/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="409" customHeight="1">
+      <c r="A7" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="62" t="inlineStr"/>
+      <c r="C7" s="62" t="inlineStr"/>
+      <c r="D7" s="62" t="inlineStr"/>
+      <c r="E7" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F7" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G7" s="62" t="inlineStr"/>
+      <c r="H7" s="62" t="inlineStr"/>
+      <c r="I7" s="62" t="inlineStr"/>
+      <c r="J7" s="62" t="inlineStr">
+        <is>
+          <t>房出售收入划转集中管理账户
+原文依据：2004年1月1日前已在承办银行储存的公有住房出售收入，将1%、10%、90%三个账户合并为25.4%公房售后专项维修资金和75.6%住房基金两个账户。售房单位将全部售房收入划转到集中管理账户后，方可支取使用。具体程序按照《天津市存量公有住房出售收入划转集中管理账户操作程序》（见附4）办理。售房单位可保留一个原有售房款专户作为支出账户。
+原文依据：售房单位也可将资金先行划入集中户，待具备分摊条件时，再按照上述步骤进行分摊整合。
+原文依据：二、公有住房出售收入的使用
+原文依据：（一）申请
+原文依据：单位使用售房资金应当向审核部门提出书面申请。领取并填写“天津市公房售后专项维修资金使用申请书”或“天津市住房基金使用申请书”（以下简称“使用申请书”，见附5、附6）、“天津市公房售后专项维修资金使用分摊明细表”（以下简称“分摊明细表”，见附7）提供以下要件。
+原文依据：1.使用公房售后专项维修资金的，应当提供：
+原文依据：（1）银行对账单；
+原文依据：（2）使用申请书；
+原文依据：（3）分摊明细表。
+原文依据：应当由专有部分面积占比三分之二以上的业主且人数占比三分之二以上的业主参与表决。决定使用专项维修资金的事项，应当经参与表决专有部分面积过半数的业主且参与表决人数过半数的业主同意。
+原文依据：（4）维修方案和维修预算（或维修结算）。
+原文依据：单位可以在工程启动前，先申请50%工程款的划拨手续，待工程结算后，再据实申请剩余资金划拨手续；也可在工程结算后，一次性申请办理资金提取手续。
+原文依据：2.使用住房基金的，应当提供：
+原文依据：（3）其他要件如下：
+原文依据：使用应急抢险资金用于房屋应急抢险的，需提供发生事故说明、社区居委会证明、事故现场查勘表、维修预算（或维修结算）；用于小区维修的，提供维修方案和维修预算（或维修结算）。使用维保改造资金用于售前维修及售后保修的，提供维修方案和维修预算（或维修结算）；用于严损房屋改造的，提供情况说明、严损房屋查勘表、改造方案、改造预算（或改造结算）及相关佐证材料。使用房屋管理储备资金用于管理单位转换经营机制的，提供单位转换经营机制方案、资金使用说明。使用售房经费的，提供资金使用计划。使用住房货币分配资金的，提供经区住房建设委备案的《天津市单位住房货币分配审核备案表》</t>
+        </is>
+      </c>
+      <c r="K7" s="62" t="inlineStr"/>
+      <c r="L7" s="62" t="inlineStr"/>
+      <c r="M7" s="62" t="inlineStr">
+        <is>
+          <t>5/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="409" customHeight="1">
+      <c r="A8" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" s="62" t="inlineStr"/>
+      <c r="C8" s="62" t="inlineStr"/>
+      <c r="D8" s="62" t="inlineStr"/>
+      <c r="E8" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F8" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G8" s="62" t="inlineStr"/>
+      <c r="H8" s="62" t="inlineStr"/>
+      <c r="I8" s="62" t="inlineStr"/>
+      <c r="J8" s="62" t="inlineStr">
+        <is>
+          <t>和资金使用说明。
+原文依据：以上资金用于维修改造的，单位可以在工程启动前，先申请50%工程款的划拨手续，待工程结算后，再据实申请剩余资金划拨手续；也可在工程结算后，一次性申请办理资金提取手续。
+原文依据：（二）受理
+原文依据：经查验各项申请要件齐全的，审核（初审）部门予以受理。
+原文依据：（三）审核
+原文依据：审核（初审）部门在5个工作日内完成审核，填写意见并加盖公章。
+原文依据：市内六区直管公产住房使用维保改造资金、售房经费和房屋管理储备资金的，由市住房城乡建设委向市财政局提交资金使用函，交由市财政局办理资金划拨手续。
+原文依据：（四）资金拨付
+原文依据：1.银行审核记明细账。承办银行确认售房单位资金账户余额大于申请审核金额后，记住房基金单位分户账或专项维修资金业主分户帐，并在“使用申请书”上加盖银行业务受理专用章后，将其交市住保中心。住房基金使用在2个工作日内完成记账，专项维修资金使用在7个工作日内完成记账。
+原文依据：2.划款。市住保中心根据“使用申请书”，在3个工作日内将申请金额划拨到售房单位专用支出账户。
+原文依据：3.记账。售房单位以留存的“使用申请书”和“分摊明细表”以及进账单作为记账凭证。市住保中心以留存的“使用申请书”、“分摊明细表”及银行回单作为记账凭证。
+原文依据：三、公有住房出售收入的转移
+原文依据：（一）业主转让房屋所有权，售房单位更名、合并、分立或破产、撤销办理销户以及住房灭失等应当转移公房售后专项维修资金或住房基金的，按照以下程序办理：
+原文依据：1.申请
+原文依据：申请公有住房出售收入转移的单位，到审核部门领取并填写“天津市公有住房出售收入转移申请书”（以下简称“转移申请书”，见附8），同时提供银行对账单以及如下相应要件：
+原文依据：（1）业主转让房屋所有权的，由售房单位持住房所有权转移证明，申请专项维修资金分户账更名。
+原文依据：（2）售房单位更名的，由售房单位持变更后的单位法人证书和单位更名批准文件，申请单位公房售后专项维修资金和住房基金账户更名。
+原文依据：（3）住房灭失的，售房单位根据灭失住房产权人要求，持“使用申请书”、“天津市国有土地上房屋征收补偿协议”或其他有关房屋灭失的证明，申请支取征收（拆迁）住房专项维修资金个人缴存余额，剩余的公房售后专项维修资金余额转移到住房基金应急抢险资金账户中</t>
+        </is>
+      </c>
+      <c r="K8" s="62" t="inlineStr"/>
+      <c r="L8" s="62" t="inlineStr"/>
+      <c r="M8" s="62" t="inlineStr">
+        <is>
+          <t>6/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="409" customHeight="1">
+      <c r="A9" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" s="62" t="inlineStr"/>
+      <c r="C9" s="62" t="inlineStr"/>
+      <c r="D9" s="62" t="inlineStr"/>
+      <c r="E9" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F9" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G9" s="62" t="inlineStr"/>
+      <c r="H9" s="62" t="inlineStr"/>
+      <c r="I9" s="62" t="inlineStr"/>
+      <c r="J9" s="62" t="inlineStr">
+        <is>
+          <t>。
+原文依据：（4）售房单位将售后公房移交托管单位管理的，需将公房售后专项维修资金余额和应急抢险资金余额转移到房屋托管单位。
+原文依据：（5）售房单位破产或撤销的，售房单位持人民法院破产裁定或单位撤销证明和公房售后专项维修资金托管协议，申请将公房售后专项维修资金余额和应急抢险资金账户余额转移到托管单位，住房基金70%余额按有关规定处理。
+原文依据：（6）当单位申请使用住房基金账户全部余额时，办理相关账户销户；申请使用公房售后专项维修资金全部余额时，办理销户或按照有关规定续存资金。
+原文依据：2.核准
+原文依据：审核部门应在5个工作日内完成核准工作，对核准转移的单位，审批部门在“转移申请书”上加盖单位公章，留存“转移申请书”一联后，交申请单位送承办银行。
+原文依据：3.资金转移
+原文依据：（1）业主转让房屋所有权、售房单位更名。
+原文依据：承办银行为售房单位办理相关手续。“转移申请书”其中一联由售房单位留存，用于办理产权转移。
+原文依据：（2）住房灭失，售房单位合并、分立或破产、撤销办理销户。
+原文依据：①银行审核。承办银行确认售房单位资金账户余额后，在“转移申请书”上加盖银行业务受理专用章后，交市住保中心。
+原文依据：②划款。市住保中心根据“转移申请书”，在3个工作日内完成资金转移。
+原文依据：（二）存量公有住房出售资金划转到承办银行集中管理账户，按照以下程序办理：
+原文依据：1.领表。售房单位到区住建委领取《天津市存量公有住房出售收入划转通知单》（以下简称“存量划转通知单”，见附9）。
+原文依据：2.单位核对余额。单位到原承办银行打印对账单，核对售房款余额。
+原文依据：3.填表审核。单位填写“存量划转通知单”交由区住房建设委审核。
+原文依据：4.交表。单位将“存量划转通知单”交到原承办银行，经审核无误后记账并加盖业务受理专用章，留存一联后，其他联分别交售房单位、审核部门、转入银行、市住保中心。
+原文依据：5.划款。市住保中心接到“存量划转通知单”后核对金额，划款并记账。
+原文依据：6接收承办银行记明细账。接收承办银行接到“存量划转通知单”并确认金额已划入后，要求单位提供住房基金比例情况说明以及专项维修资金分户情况说明，并据此记录单位明细账和分户账。
+原文依据：四、对账和查询
+原文依据：（一）承办银行与核算部门对账。承办银行每</t>
+        </is>
+      </c>
+      <c r="K9" s="62" t="inlineStr"/>
+      <c r="L9" s="62" t="inlineStr"/>
+      <c r="M9" s="62" t="inlineStr">
+        <is>
+          <t>7/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="409" customHeight="1">
+      <c r="A10" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="62" t="inlineStr"/>
+      <c r="C10" s="62" t="inlineStr"/>
+      <c r="D10" s="62" t="inlineStr"/>
+      <c r="E10" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F10" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G10" s="62" t="inlineStr"/>
+      <c r="H10" s="62" t="inlineStr"/>
+      <c r="I10" s="62" t="inlineStr"/>
+      <c r="J10" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">月与市住保中心核对住房基金、维修资金收支及余额情况后，由市住保中心出具余额调节表。
+原文依据：（二）承办银行与售房单位对账。每年6月30日结息后，售房单位可到承办银行领取对账单和业主变更清单进行对账。有疑义的，应及时与承办银行联系。
+原文依据：（三）承办银行业务系统与流水对账。承办银行定期将公有住房出售收入业务管理系统与银行流水余额进行核对，每年末将核对情况书面告知市住保中心。
+原文依据：（四）查询。售房单位可到承办银行查询两个资金账户的归集、使用情况，住房业主可到售房单位查询专项维修资金账户的归集、使用情况。
+原文依据：附：1.天津市公有住房出售收入开户登记表
+原文依据：2.天津市公有住房出售收入交款单
+原文依据：3.天津市财政票据（样式）
+原文依据：4.天津市存量公有住房出售收入划转集中管理账户操
+原文依据：作程序
+原文依据：5.天津市公房售后专项维修资金使用申请书
+原文依据：6.天津市住房基金使用申请书
+原文依据：7.天津市公房售后专项维修资金使用分摊明细表
+原文依据：8.天津市公有住房出售收入转移申请书
+原文依据：9.天津市存量公有住房出售收入划转通知单
+原文依据：附1
+原文依据：天津市公有住房出售收入开户登记表
+原文依据：单位名称（全称）：
+原文依据：本表一式四联，第一联售房单位留存；第二联市住房保障服务中心留存；第三、四联承办银行留存。
+原文依据：附2
+原文依据：天津市公有住房出售收入交款单
+原文依据：收款单位：天津市住房保障服务中心                                             印刷编号：(000001------100000)
+原文依据：本交款通知单一式四联，第一、二联售房单位留存；第三、四联承办银行记账。
+原文依据：附3
+原文依据：天津市财政票据（样式）
+原文依据：票据代码：                                                                               票据号码：
+原文依据：票据名称：天津市出售公有住房票据                                                   电子票据号码：
+原文依据：交款人统一社会信用代码：            </t>
+        </is>
+      </c>
+      <c r="K10" s="62" t="inlineStr"/>
+      <c r="L10" s="62" t="inlineStr"/>
+      <c r="M10" s="62" t="inlineStr">
+        <is>
+          <t>8/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="409" customHeight="1">
+      <c r="A11" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" s="62" t="inlineStr"/>
+      <c r="C11" s="62" t="inlineStr"/>
+      <c r="D11" s="62" t="inlineStr"/>
+      <c r="E11" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F11" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G11" s="62" t="inlineStr"/>
+      <c r="H11" s="62" t="inlineStr"/>
+      <c r="I11" s="62" t="inlineStr"/>
+      <c r="J11" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                                                    校验码：
+原文依据：交款人：XXX                                                                              开票日期：
+原文依据：收款单位（章）                                 复核人：                          收款人：
+原文依据：附4
+原文依据：天津市存量公有住房出售收入划转
+原文依据：集中管理账户操作程序
+原文依据：2004年1月1日前已在承办银行储存的公有住房出售收入，将1%、10%、90%三个账户合并为25.4%公房售后专项维修资金和75.6%住房基金两个账户，操作程序如下。
+原文依据：一、整合调整账户资金
+原文依据：（一）11%维修资金
+原文依据：售房单位将1%、10%账户资金余额合并为11%维修资金，记账到每套住房。售房单位可根据本单位售房款管理情况采取以下三种方法分摊：余额调整法、余额平摊法、单位具结法。
+原文依据：1.余额调整法（以下简称方法一）
+原文依据：售房单位向承办银行提供每个业主10%和1%维修资金的交存、使用日期和金额初值。承办银行计算每个业主10%和1%的本金和利息余额，每年利息并入上年本金滚存计算，计算余额之和与账面余额的差额根据余额调整系数调整。
+原文依据：11%调整系数=计算余额与账面余额的差额/全体业主计算利息之和
+原文依据：某住房分摊的11%维修资金调整差额=该住房计算利息×11%维修资金调整系数
+原文依据：2.余额平摊法（以下简称方法二）
+原文依据：售房单位向承办银行提供每个业主10%和1%维修资金的交存和使用年份和金额初值，以及各年售房单位10%和1%维修资金利息金额小计。承办银行根据售房单位某年10%和1%维修资金余额之和与利息之和计算当年分摊系数，将各年度利息分摊到当年存有本金的业主。
+原文依据：某年11%维修资金分摊系数=某年单位账户11%维修资金利息之和/各套住房该年11%维修资金本金余额之和
+原文依据：某年某住房分摊的11%维修资金利息金额=某年11%维修资金分摊系数×该住房当年11%维修资金本金余额
+原文依据：按照方法二计算的各住房10%</t>
+        </is>
+      </c>
+      <c r="K11" s="62" t="inlineStr"/>
+      <c r="L11" s="62" t="inlineStr"/>
+      <c r="M11" s="62" t="inlineStr">
+        <is>
+          <t>9/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="409" customHeight="1">
+      <c r="A12" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" s="62" t="inlineStr"/>
+      <c r="C12" s="62" t="inlineStr"/>
+      <c r="D12" s="62" t="inlineStr"/>
+      <c r="E12" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F12" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G12" s="62" t="inlineStr"/>
+      <c r="H12" s="62" t="inlineStr"/>
+      <c r="I12" s="62" t="inlineStr"/>
+      <c r="J12" s="62" t="inlineStr">
+        <is>
+          <t>和1%维修资金本金与利息之和与账面余额的差额如大于10元，用计算差额代替分摊系数的分子后，按照原方法重新分摊一次。
+原文依据：3.单位具结法（以下简称方法三）
+原文依据：对于售房单位已将多幢住房的10%和1%维修资金混合用于某幢住房维修，部分或全部使用难以按套分摊的，由单位出具具结意见，负责就专项维修资金记账到每套住房工作向管房组织做好说明解释工作，同时对剩余专项维修资金自行提出分摊意见和每套住房专项维修资金分摊明细，具结意见和分摊明细报审核部门备案。
+原文依据：维修资金未使用或使用资金可按套分摊的，售房单位可选择方法一或方法二，将其记账到每套住房。住宅项目成立业主委员会的，应将结果告知业主委员会。单位能够提供业主购房准确年月日的，可选择方法一；单位只能提供业主购房年份及各年利息的，可选择方法二。对专项维修资金难以按套分摊的，售房单位可选择方法三。售房单位未提取或未足额提取专项维修资金的，应当建立或补充专项维修资金；售房单位未将专项维修资金存入承办银行的，应当将专项维修资金划入承办银行后，记账到每套住房。
+原文依据：各单位将专项维修资金账户内的本金和利息余额分摊到每套住房时，如本金和利息余额为零的，应将支取使用记录进行公示，其公示要求如下：
+原文依据：（1）公示内容
+原文依据：各单位已使用专项维修资金的，应将有关情况制成公示招贴在小区内，公示内容包括：维修项目、维修时间、维修协议书、维修支出金额。
+原文依据：（2）公示方式
+原文依据：公示招贴应张贴在小区入口公示栏和相关业主的楼栋口醒目位置，公示期应当自公示之日起满7个工作日。
+原文依据：（3）资料留存
+原文依据：售房单位应当将公示招贴、公示现场情况的远景和近景照片资料及维修工程施工合同和相关票据原件及复印件留存备查。
+原文依据：（二）14.4%更新改造资金
+原文依据：售房单位从90%售房款账户中，提取14.4%的更新改造资金记账到每套住房，计算方法按照每套住房建筑面积所占单位已售公有住房总建筑面积所占比例分摊。
+原文依据：本意见施行日前已归集的14.4%更新改造资金由记账到幢调整为记账到套，应当经售房单位申请或确认后完成变更。
+原文依据：（三）住房基金
+原文依据：售房单位将90%售房款账户中其余资金的本金及利息，记入住房基金各明细账项目下。
+原文依据：售房单位到承办银行办理专项维修资</t>
+        </is>
+      </c>
+      <c r="K12" s="62" t="inlineStr"/>
+      <c r="L12" s="62" t="inlineStr"/>
+      <c r="M12" s="62" t="inlineStr">
+        <is>
+          <t>10/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="409" customHeight="1">
+      <c r="A13" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B13" s="62" t="inlineStr"/>
+      <c r="C13" s="62" t="inlineStr"/>
+      <c r="D13" s="62" t="inlineStr"/>
+      <c r="E13" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F13" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G13" s="62" t="inlineStr"/>
+      <c r="H13" s="62" t="inlineStr"/>
+      <c r="I13" s="62" t="inlineStr"/>
+      <c r="J13" s="62" t="inlineStr">
+        <is>
+          <t>金分户业务，应当提供资金分摊明细、分摊具结意见书，承办银行据此为单位建立专项维修资金明细账。
+原文依据：二、办理程序
+原文依据：（一）单位领取、填写表册。售房单位到承办银行打印账户查询单，领取并填写“天津市公房售后专项维修资金分套登记总表”（见表一），并提供存量公房售后专项维修资金的明细账册。
+原文依据：采取余额调整法和余额平摊法的售房单位到承办银行领取并填写《天津市公房售后专项维修资金分套登记明细清册》（见表二）；
+原文依据：采取具结法的售房单位填写《天津市公房售后专项维修资金单位具结意见书》（见表三）及《天津市公房售后专项维修资金具结明细清册》（见表四）。
+原文依据：（二）银行录入，单位校对。承办银行录入明细清册相关内容，并将录入内容打印“每套住房专项维修资金余额账户明细”，交单位核对。单位应在10个工作日内将核对确认结果反馈承办银行。
+原文依据：（三）回单。承办银行打印“每套住房专项维修资金余额利息明细”，与售房单位据此建立专项维修资金单位账和业主分套账。
+原文依据：表一
+原文依据：天津市公房售后专项维修资金分套登记总表
+原文依据：表二
+原文依据：天津市公房售后专项维修资金分套登记明细清册（一）
+原文依据：天津市公房售后专项维修资金分套登记明细清册（二）
+原文依据：（余额平摊法年利息表）
+原文依据：表三
+原文依据：天津市公房售后专项维修资金单位具结意见书
+原文依据：表四
+原文依据：天津市公房售后专项维修资金具结明细清册
+原文依据：附5
+原文依据：天津市公房售后专项维修资金使用申请书
+原文依据：本表一式四联，第一联售房单位留存；第二联市住房保障服务中心留存；第三联区住房和建设委员会留存；第四联承办银行留存。第一、二、四联加盖承办银行代天津市出售公有住房业务受理专用章后生效。
+原文依据：附6
+原文依据：天津市住房基金使用申请书
+原文依据：注：第一联退售房单位留存；第二联市住房保障服务中心留存；第三联承办银行留存；第四联审核部门留存。第一至三联加盖承办银行专用章后生效。
+原文依据：附7
+原文依据：天津市公房售后专项维修资金使用分摊明细表
+原文依据：附8
+原文依据：附9
+原文依据：天津市单位产公有住房出售收入存量划转通知单
+原文依据：注：该通知单一式六联,第一联留售房单位,第二联交审核单位，第三联交转出银行，第四</t>
+        </is>
+      </c>
+      <c r="K13" s="62" t="inlineStr"/>
+      <c r="L13" s="62" t="inlineStr"/>
+      <c r="M13" s="62" t="inlineStr">
+        <is>
+          <t>11/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="409" customHeight="1">
+      <c r="A14" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B14" s="62" t="inlineStr"/>
+      <c r="C14" s="62" t="inlineStr"/>
+      <c r="D14" s="62" t="inlineStr"/>
+      <c r="E14" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F14" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G14" s="62" t="inlineStr"/>
+      <c r="H14" s="62" t="inlineStr"/>
+      <c r="I14" s="62" t="inlineStr"/>
+      <c r="J14" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">联交转入银行，第五、六联交市住房保障服务中心。
+原文依据：天津市住房和城乡建设委员会办公室          2026年9月29日印发
+原文依据：| 单位地址： | 单位地址： | 单位地址： | 单位地址： | 单位地址： | 单位地址： | 申请单位公章
+原文依据：开户
+单位
+填写 | 主管区局名称（全称）： | 主管区局名称（全称）： | 主管区局名称（全称）： | 主管区局名称（全称）： | 主管区局代码： | 主管区局代码： |
+原文依据：开户
+单位
+填写 | 经办部门： | 联系人： | 电话： | 电话： | 电话： | 邮政编码： | 经办人：
+原文依据：开户
+单位
+填写 | 出售公有住房产别：直管产（市级□  区级□）    单位产（       ） | 出售公有住房产别：直管产（市级□  区级□）    单位产（       ） | 出售公有住房产别：直管产（市级□  区级□）    单位产（       ） | 职工工资来源：市财政补助（       ）                                  区财政补助（    ）   其他（     ） | 职工工资来源：市财政补助（       ）                                  区财政补助（    ）   其他（     ） | 职工工资来源：市财政补助（       ）                                  区财政补助（    ）   其他（     ） |    年  月   日
+原文依据：承办银行填写 | 　 | 　 | 　 | 　 | 　 | 　 |
+原文依据：购房人 |  | 售房单位全称 |  | 售房单位代码 | 售房单位代码 | 售房单位代码 |  |  |  |
+原文依据：售房许可证号 |  |  | 住房建筑面积（m2） |  |  |  |  |  |  |
+原文依据：主管区局 |  |  |      主管区局代码 |  |  |  |  |  |  |
+原文依据：住房地址 | 区         街道           道（路、街）    号           小区（里）   栋   门   楼   室 | 区         街道           道（路、街） </t>
+        </is>
+      </c>
+      <c r="K14" s="62" t="inlineStr"/>
+      <c r="L14" s="62" t="inlineStr"/>
+      <c r="M14" s="62" t="inlineStr">
+        <is>
+          <t>12/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="295" customHeight="1">
+      <c r="A15" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B15" s="62" t="inlineStr"/>
+      <c r="C15" s="62" t="inlineStr"/>
+      <c r="D15" s="62" t="inlineStr"/>
+      <c r="E15" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F15" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G15" s="62" t="inlineStr"/>
+      <c r="H15" s="62" t="inlineStr"/>
+      <c r="I15" s="62" t="inlineStr"/>
+      <c r="J15" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   号           小区（里）   栋   门   楼   室 | 区         街道           道（路、街）    号           小区（里）   栋   门   楼   室 | 区         街道           道（路、街）    号           小区（里）   栋   门   楼   室 | 区         街道           道（路、街）    号           小区（里）   栋   门   楼   室 | 区         街道           道（路、街）    号           小区（里）   栋   门   楼   室 | 区         街道           道（路、街）    号           小区（里）   栋   门   楼   室 | 区         街道           道（路、街）    号           小区（里）   栋   门   楼   室 | 区         街道           道（路、街）    号           小区（里）   栋   门   楼   室 | 区         街道           道（路、街）    号           小区（里）   栋   门   楼   室
+原文依据：应交款总额（101%） | （大写）    拾     万    仟    佰     拾     元整 | （大写）    拾     万    仟    佰     拾     元整 | （大写）    拾     万    仟    佰     拾     元整 | （大写）    拾     万    仟    佰     拾     元整 | 拾 | 万 | 仟 | 佰 | 拾 | 元
+原文依据：应交款总额（101%） | （大写）    拾     万    仟    佰     拾     元整 | （大写）    拾     万    仟    佰     拾     元整 | （大写）    拾     万    仟    佰     拾     元整 | （大写）    拾     万    仟    佰     拾     元整 |  |  |  |  |  |
+原文依据：</t>
+        </is>
+      </c>
+      <c r="K15" s="62" t="inlineStr"/>
+      <c r="L15" s="62" t="inlineStr"/>
+      <c r="M15" s="62" t="inlineStr">
+        <is>
+          <t>13/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="409" customHeight="1">
+      <c r="A16" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B16" s="62" t="inlineStr"/>
+      <c r="C16" s="62" t="inlineStr"/>
+      <c r="D16" s="62" t="inlineStr"/>
+      <c r="E16" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F16" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G16" s="62" t="inlineStr"/>
+      <c r="H16" s="62" t="inlineStr"/>
+      <c r="I16" s="62" t="inlineStr"/>
+      <c r="J16" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">公房售后专项维修资金（25.4%） | 1%维修资金 | 1%维修资金 | 1%维修资金 | 1%维修资金 |  |  |  |  |  |
+原文依据：公房售后专项维修资金（25.4%） | 10%维修资金 | 10%维修资金 | 10%维修资金 | 10%维修资金 |  |  |  |  |  |
+原文依据：公房售后专项维修资金（25.4%） | 14.4%更新改造资金 | 14.4%更新改造资金 | 14.4%更新改造资金 | 14.4%更新改造资金 |  |  |  |  |  |
+原文依据：公房售后专项维修资金（25.4%） | 电梯、水泵更新改造资金 | 电梯、水泵更新改造资金 | 电梯、水泵更新改造资金 | 电梯、水泵更新改造资金 |  |  |  |  |  |
+原文依据：住房基金75.6% |  |  |  |  |  |  |  |  |  |
+原文依据：售房单位公章
+经办人（章）
+                                              年      月      日 | 售房单位公章
+经办人（章）
+                                              年      月      日 | 售房单位公章
+经办人（章）
+                                              年      月      日 | 售房单位公章
+经办人（章）
+                                              年      月      日 | 售房单位公章
+经办人（章）
+                                              年      月      日 | 售房单位公章
+经办人（章）
+                                              年      月      日 | 售房单位公章
+经办人（章）
+                                              年      月      日 | 售房单位公章
+经办人（章）
+                                   </t>
+        </is>
+      </c>
+      <c r="K16" s="62" t="inlineStr"/>
+      <c r="L16" s="62" t="inlineStr"/>
+      <c r="M16" s="62" t="inlineStr">
+        <is>
+          <t>14/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="409" customHeight="1">
+      <c r="A17" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B17" s="62" t="inlineStr"/>
+      <c r="C17" s="62" t="inlineStr"/>
+      <c r="D17" s="62" t="inlineStr"/>
+      <c r="E17" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F17" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G17" s="62" t="inlineStr"/>
+      <c r="H17" s="62" t="inlineStr"/>
+      <c r="I17" s="62" t="inlineStr"/>
+      <c r="J17" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">           年      月      日 | 售房单位公章
+经办人（章）
+                                              年      月      日 | 售房单位公章
+经办人（章）
+                                              年      月      日 | 售房单位公章
+经办人（章）
+                                              年      月      日
+原文依据：项目编码 | 项目名称 | 单位 | 数量 | 标准 | 金额（元） | 备注
+原文依据：| 售后专项维修资金（25.4%）
+其中：11%维修资金
+      14.4%更新改造资金
+      电梯、水泵更新改造资金
+住房基金（75.6%） | 套
+套
+套
+套
+套 | 1
+1
+1
+1
+1 |  |  |
+原文依据：金额合计（大写）                                                               （小写）￥ | 金额合计（大写）                                                               （小写）￥ | 金额合计（大写）                                                               （小写）￥ | 金额合计（大写）                                                               （小写）￥ | 金额合计（大写）                                                               （小写）￥ | 金额合计（大写）                                                               （小写）￥ | 金额合计（大写）                                                               （小写）￥
+原文依据：其           </t>
+        </is>
+      </c>
+      <c r="K17" s="62" t="inlineStr"/>
+      <c r="L17" s="62" t="inlineStr"/>
+      <c r="M17" s="62" t="inlineStr">
+        <is>
+          <t>15/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="280" customHeight="1">
+      <c r="A18" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B18" s="62" t="inlineStr"/>
+      <c r="C18" s="62" t="inlineStr"/>
+      <c r="D18" s="62" t="inlineStr"/>
+      <c r="E18" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F18" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G18" s="62" t="inlineStr"/>
+      <c r="H18" s="62" t="inlineStr"/>
+      <c r="I18" s="62" t="inlineStr"/>
+      <c r="J18" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                              房屋地址：                                            
+他                                         售房单位全称：                                    售房单位代码：
+信                                         主管区（局）：                                     主管区（局）代码：
+息                                         房屋建筑面积（m2）：                               房屋实际售价（100%）（元）：            
+交款单编号：                                     房屋代码： | 其                                         房屋地址：                                            
+他                                         售房单位全称：                                    售房单位代码：
+信                                         主管区（局）：                                     主管区（局）代码：
+息                                         房屋建筑面积（m2）：                               房屋实际售价（100%）（元）：            
+交款单编号：                                     房屋代码： | 其                                         房屋地址：                                            
+他                             </t>
+        </is>
+      </c>
+      <c r="K18" s="62" t="inlineStr"/>
+      <c r="L18" s="62" t="inlineStr"/>
+      <c r="M18" s="62" t="inlineStr">
+        <is>
+          <t>16/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="280" customHeight="1">
+      <c r="A19" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B19" s="62" t="inlineStr"/>
+      <c r="C19" s="62" t="inlineStr"/>
+      <c r="D19" s="62" t="inlineStr"/>
+      <c r="E19" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F19" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G19" s="62" t="inlineStr"/>
+      <c r="H19" s="62" t="inlineStr"/>
+      <c r="I19" s="62" t="inlineStr"/>
+      <c r="J19" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            售房单位全称：                                    售房单位代码：
+信                                         主管区（局）：                                     主管区（局）代码：
+息                                         房屋建筑面积（m2）：                               房屋实际售价（100%）（元）：            
+交款单编号：                                     房屋代码： | 其                                         房屋地址：                                            
+他                                         售房单位全称：                                    售房单位代码：
+信                                         主管区（局）：                                     主管区（局）代码：
+息                                         房屋建筑面积（m2）：                               房屋实际售价（100%）（元）：            
+交款单编号：                                     房屋代码： | 其                                         房屋地址：                                            
+他                                         售房单位全称：                                    售房单位代码：
+信                                         主管区（局</t>
+        </is>
+      </c>
+      <c r="K19" s="62" t="inlineStr"/>
+      <c r="L19" s="62" t="inlineStr"/>
+      <c r="M19" s="62" t="inlineStr">
+        <is>
+          <t>17/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="280" customHeight="1">
+      <c r="A20" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B20" s="62" t="inlineStr"/>
+      <c r="C20" s="62" t="inlineStr"/>
+      <c r="D20" s="62" t="inlineStr"/>
+      <c r="E20" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F20" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G20" s="62" t="inlineStr"/>
+      <c r="H20" s="62" t="inlineStr"/>
+      <c r="I20" s="62" t="inlineStr"/>
+      <c r="J20" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">）：                                     主管区（局）代码：
+息                                         房屋建筑面积（m2）：                               房屋实际售价（100%）（元）：            
+交款单编号：                                     房屋代码： | 其                                         房屋地址：                                            
+他                                         售房单位全称：                                    售房单位代码：
+信                                         主管区（局）：                                     主管区（局）代码：
+息                                         房屋建筑面积（m2）：                               房屋实际售价（100%）（元）：            
+交款单编号：                                     房屋代码： | 其                                         房屋地址：                                            
+他                                         售房单位全称：                                    售房单位代码：
+信                                         主管区（局）：                                     主管区（局）代码：
+息                                         房屋建筑面积（m2）：        </t>
+        </is>
+      </c>
+      <c r="K20" s="62" t="inlineStr"/>
+      <c r="L20" s="62" t="inlineStr"/>
+      <c r="M20" s="62" t="inlineStr">
+        <is>
+          <t>18/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="400" customHeight="1">
+      <c r="A21" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B21" s="62" t="inlineStr"/>
+      <c r="C21" s="62" t="inlineStr"/>
+      <c r="D21" s="62" t="inlineStr"/>
+      <c r="E21" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F21" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G21" s="62" t="inlineStr"/>
+      <c r="H21" s="62" t="inlineStr"/>
+      <c r="I21" s="62" t="inlineStr"/>
+      <c r="J21" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                       房屋实际售价（100%）（元）：            
+交款单编号：                                     房屋代码：
+原文依据：单位名称（全称）： |  |  |  |  |
+原文依据：单位地址 | 单位地址 | 单位地址 | 单位地址 | 单位地址 | 单位地址
+原文依据：主管局名称（全称） | 主管局名称（全称） | 主管局名称（全称） | 主管局名称（全称） | 主管局代码 | 主管局代码
+原文依据：10%维修资金单位账号 | 10%维修资金单位账号 | 10%维修资金单位账号 | 1%维修资金单位账号 | 1%维修资金单位账号 | 90%售房款账号
+原文依据：经办部门 | 经办部门 | 联系人 | 联系人 | 联系电话 | 邮政编码
+原文依据：出售公有住房产别：直管产□  （保管自修 □ ）  单位产 □ | 出售公有住房产别：直管产□  （保管自修 □ ）  单位产 □ | 出售公有住房产别：直管产□  （保管自修 □ ）  单位产 □ | 职工工资来源：市财政全额拨款（       ）  区财政全额拨款（    ）   其他（     ） | 职工工资来源：市财政全额拨款（       ）  区财政全额拨款（    ）   其他（     ） | 职工工资来源：市财政全额拨款（       ）  区财政全额拨款（    ）   其他（     ）
+原文依据：10%维修资金（余额）             佰           拾          万           仟          佰           拾          元整，包括           户住房 | 10%维修资金（余额）             佰           拾          万           仟          佰           拾          元整，包括           户住房 | 10%维修资金（余额）             佰           拾          万           仟          佰           拾          元整，包括           户住房 | 10%维修资金（余额） </t>
+        </is>
+      </c>
+      <c r="K21" s="62" t="inlineStr"/>
+      <c r="L21" s="62" t="inlineStr"/>
+      <c r="M21" s="62" t="inlineStr">
+        <is>
+          <t>19/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="235" customHeight="1">
+      <c r="A22" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B22" s="62" t="inlineStr"/>
+      <c r="C22" s="62" t="inlineStr"/>
+      <c r="D22" s="62" t="inlineStr"/>
+      <c r="E22" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F22" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G22" s="62" t="inlineStr"/>
+      <c r="H22" s="62" t="inlineStr"/>
+      <c r="I22" s="62" t="inlineStr"/>
+      <c r="J22" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">            佰           拾          万           仟          佰           拾          元整，包括           户住房 | 10%维修资金（余额）             佰           拾          万           仟          佰           拾          元整，包括           户住房 | 10%维修资金（余额）             佰           拾          万           仟          佰           拾          元整，包括           户住房
+原文依据：1%维修资金（余额）              佰           拾          万           仟          佰           拾          元整 ，包括          户住房 | 1%维修资金（余额）              佰           拾          万           仟          佰           拾          元整 ，包括          户住房 | 1%维修资金（余额）              佰           拾          万           仟          佰           拾          元整 ，包括          户住房 | 1%维修资金（余额）              佰           拾          万           仟          佰           拾          元整 ，包括          户住房 | 1%维修资金（余额）              佰           拾          万           仟          佰           拾          元整 ，包括          户住房 | 1%维修资金（余额）              佰           拾          万           仟          佰           拾     </t>
+        </is>
+      </c>
+      <c r="K22" s="62" t="inlineStr"/>
+      <c r="L22" s="62" t="inlineStr"/>
+      <c r="M22" s="62" t="inlineStr">
+        <is>
+          <t>20/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="409" customHeight="1">
+      <c r="A23" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B23" s="62" t="inlineStr"/>
+      <c r="C23" s="62" t="inlineStr"/>
+      <c r="D23" s="62" t="inlineStr"/>
+      <c r="E23" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F23" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G23" s="62" t="inlineStr"/>
+      <c r="H23" s="62" t="inlineStr"/>
+      <c r="I23" s="62" t="inlineStr"/>
+      <c r="J23" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     元整 ，包括          户住房
+原文依据：选择记账到每户住房方法 | 余额调整法 （      ） | 余额调整法 （      ） | 余额调整法 （      ） | 余额平摊法   （    ） | 单位出据具结，自行分摊（        ）
+原文依据：单位加盖预留银行印鉴 | 单位加盖预留银行印鉴 | 单位加盖预留银行印鉴 | 单位加盖预留银行印鉴 | 银行盖章 | 银行盖章
+原文依据：经办人：                             年       月      日 |        经办人：                             年       月      日 |        经办人：                             年       月      日 |        经办人：                             年       月      日 | 经办人：                   年         月           日 | 经办人：                   年         月           日
+原文依据：注：本表一式两联，第一联售房单位留存；第二联承办银行留存。 | 注：本表一式两联，第一联售房单位留存；第二联承办银行留存。 | 注：本表一式两联，第一联售房单位留存；第二联承办银行留存。 | 注：本表一式两联，第一联售房单位留存；第二联承办银行留存。 | 注：本表一式两联，第一联售房单位留存；第二联承办银行留存。 | 注：本表一式两联，第一联售房单位留存；第二联承办银行留存。
+原文依据：|   |   |  |  | 年      月      日 | 年      月      日 | 年      月      日 | 分摊方法 ：余额调整（  ） 余额平摊（  ） | 分摊方法 ：余额调整（  ） 余额平摊（  ） | 分摊方法 ：余额调整（  ） 余额平摊（  ） | 分摊方法 ：余额调整（  ） 余额平摊（  ） | 分摊方法 ：余额调整（  ） 余额平摊（  ）
+原文依据：单位名称（全称）： | 单位名称（全称）： | 单位名称（全称）： |  |  |  |  |  |  |  |  </t>
+        </is>
+      </c>
+      <c r="K23" s="62" t="inlineStr"/>
+      <c r="L23" s="62" t="inlineStr"/>
+      <c r="M23" s="62" t="inlineStr">
+        <is>
+          <t>21/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="409" customHeight="1">
+      <c r="A24" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B24" s="62" t="inlineStr"/>
+      <c r="C24" s="62" t="inlineStr"/>
+      <c r="D24" s="62" t="inlineStr"/>
+      <c r="E24" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F24" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G24" s="62" t="inlineStr"/>
+      <c r="H24" s="62" t="inlineStr"/>
+      <c r="I24" s="62" t="inlineStr"/>
+      <c r="J24" s="62" t="inlineStr">
+        <is>
+          <t>| 单位：元 | 单位：元
+原文依据：10%维修资金单位账号 | 10%维修资金单位账号 | 10%维修资金单位账号 | 10%维修资金单位账号 | 1%维修资金单位账号 | 1%维修资金单位账号 | 1%维修资金单位账号 | 1%维修资金单位账号 | 1%维修资金单位账号 | 1%维修资金单位账号 | 1%维修资金单位账号 | 1%维修资金单位账号 | 1%维修资金单位账号
+原文依据：| 序号 | 住房业主姓名 | 住房地址 | 10%维修资金 | 10%维修资金 | 10%维修资金 | 10%维修资金 | 10%维修资金 | 1%维修资金 | 1%维修资金 | 1%维修资金 | 1%维修资金
+原文依据：| 序号 | 住房业主姓名 | 住房地址 | 年 | 年 | 月 | 日 | 金额 | 年 | 月 | 日 | 金额
+原文依据：| 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 |
+原文依据：业 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 |
+原文依据：主 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 |
+原文依据：明 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 |
+原文依据：细 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 |
+原文依据：| 合计（本页小计） | 合计（本页小计） | 合计（本页小计） | 　 | 　 | 　 |  | 　 | 　 | 　 | 　 |
+原文依据：注：本表一式两联，第一联售房单位留存；第二联承办银行留存。 | 注：本表一式两联，第一联售房单位留存；第二联承办银行留存。 | 注：本表一式两联，第一联售房单位留存；第二联承办银行留存。 | 注：本表一式两联，第一联售房单位留存；第二联承办银行留存。 | 注：本表一式两联，第一联售房单位留存；第二联承办银行留存。 | 注：本表一式两联，第一联售房单位留存；第二联承办银行留存。 | 注：本表一式两联，第一联售房单位留存；第二联承办银行留存。 | 注：本表一式两联，第一联售房单位留存；第二联承办银行留存。 | 注：本表一式两联，第一联售房单位留存；第二联承办银行留存。</t>
+        </is>
+      </c>
+      <c r="K24" s="62" t="inlineStr"/>
+      <c r="L24" s="62" t="inlineStr"/>
+      <c r="M24" s="62" t="inlineStr">
+        <is>
+          <t>22/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="409" customHeight="1">
+      <c r="A25" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B25" s="62" t="inlineStr"/>
+      <c r="C25" s="62" t="inlineStr"/>
+      <c r="D25" s="62" t="inlineStr"/>
+      <c r="E25" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F25" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G25" s="62" t="inlineStr"/>
+      <c r="H25" s="62" t="inlineStr"/>
+      <c r="I25" s="62" t="inlineStr"/>
+      <c r="J25" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | 注：本表一式两联，第一联售房单位留存；第二联承办银行留存。 | 注：本表一式两联，第一联售房单位留存；第二联承办银行留存。 | 注：本表一式两联，第一联售房单位留存；第二联承办银行留存。 | 注：本表一式两联，第一联售房单位留存；第二联承办银行留存。
+原文依据：单位名称（全称）： | 单位名称（全称）： | 单位名称（全称）： | 年            月               日 | 年            月               日 | 年            月               日 | 年            月               日 | 年            月               日 | 年            月               日 |  |  |  | 单位：元
+原文依据：10%维修资金单位账号： | 10%维修资金单位账号： | 10%维修资金单位账号： | 10%维修资金单位账号： | 10%维修资金单位账号： | 10%维修资金单位账号： | 1%维修资金单位账号： | 1%维修资金单位账号： | 1%维修资金单位账号： | 1%维修资金单位账号： | 1%维修资金单位账号： | 1%维修资金单位账号： | 1%维修资金单位账号：
+原文依据：年份 | 1992年 | 1993年 | 1994年 | 1995年 | 1996年 | 1997年 | 1998年 | 1999年 | 2000年 | 2001年 | 2002年 | 2003年
+原文依据：10%维修资金 | 　 | 　 | 　 |   | 　 | 　 | 　 | 　 | 　 | 　 | 　 |
+原文依据：年利息额 | 　 | 　 | 　 |   | 　 | 　 | 　 | 　 | 　 | 　 | 　 |
+原文依据：1%维修资金 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 |
+原文依据：年利息额 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 |
+原文依据：注：本表一式两联，第一联售房单位留存；第二联承办银行留存。 |        注：本表一式两联，第一联售房单位留存；第二联承办银行留存。 |        注：本</t>
+        </is>
+      </c>
+      <c r="K25" s="62" t="inlineStr"/>
+      <c r="L25" s="62" t="inlineStr"/>
+      <c r="M25" s="62" t="inlineStr">
+        <is>
+          <t>23/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="355" customHeight="1">
+      <c r="A26" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B26" s="62" t="inlineStr"/>
+      <c r="C26" s="62" t="inlineStr"/>
+      <c r="D26" s="62" t="inlineStr"/>
+      <c r="E26" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F26" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G26" s="62" t="inlineStr"/>
+      <c r="H26" s="62" t="inlineStr"/>
+      <c r="I26" s="62" t="inlineStr"/>
+      <c r="J26" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">表一式两联，第一联售房单位留存；第二联承办银行留存。 |        注：本表一式两联，第一联售房单位留存；第二联承办银行留存。 |        注：本表一式两联，第一联售房单位留存；第二联承办银行留存。 |        注：本表一式两联，第一联售房单位留存；第二联承办银行留存。 |        注：本表一式两联，第一联售房单位留存；第二联承办银行留存。 | 　 | 　 | 　 | 　 | 　 |
+原文依据：单位名称（全称）： |  |  |  | 　 | 　 |  |  |  |  |  |  |  |  |  |  |
+原文依据：10%维修资金单位账号： | 10%维修资金单位账号： | 10%维修资金单位账号： | 10%维修资金单位账号： | 10%维修资金单位账号： | 1%维修资金单位账号： | 1%维修资金单位账号： | 1%维修资金单位账号： | 1%维修资金单位账号： | 1%维修资金单位账号： | 1%维修资金单位账号： | 1%维修资金单位账号： | 1%维修资金单位账号： | 1%维修资金单位账号： | 1%维修资金单位账号： | 1%维修资金单位账号： | 1%维修资金单位账号：
+原文依据：主管局名称（全称）： | 主管局名称（全称）： | 主管局名称（全称）： | 主管局名称（全称）： | 主管局名称（全称）： | 主管局名称（全称）： | 主管局名称（全称）： | 主管局代码： | 主管局代码： | 主管局代码： | 主管局代码： | 主管局代码： | 主管局代码： | 主管局代码： | 主管局代码： | 主管局代码： | 主管局代码：
+原文依据：我单位出售                    户住房，按售房款10%提取的维修资金                     元，购房人交纳的1%维修资金                    元。我单位 |            我单位出售                    户住房，按售房款10%提取的维修资金                     元，购房人交纳的1%维修资金                    元。我单位 |            我单位出售                    户住房，按售房款10%提取的维修资金               </t>
+        </is>
+      </c>
+      <c r="K26" s="62" t="inlineStr"/>
+      <c r="L26" s="62" t="inlineStr"/>
+      <c r="M26" s="62" t="inlineStr">
+        <is>
+          <t>24/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="235" customHeight="1">
+      <c r="A27" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B27" s="62" t="inlineStr"/>
+      <c r="C27" s="62" t="inlineStr"/>
+      <c r="D27" s="62" t="inlineStr"/>
+      <c r="E27" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F27" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G27" s="62" t="inlineStr"/>
+      <c r="H27" s="62" t="inlineStr"/>
+      <c r="I27" s="62" t="inlineStr"/>
+      <c r="J27" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      元，购房人交纳的1%维修资金                    元。我单位 |            我单位出售                    户住房，按售房款10%提取的维修资金                     元，购房人交纳的1%维修资金                    元。我单位 |            我单位出售                    户住房，按售房款10%提取的维修资金                     元，购房人交纳的1%维修资金                    元。我单位 |            我单位出售                    户住房，按售房款10%提取的维修资金                     元，购房人交纳的1%维修资金                    元。我单位 |            我单位出售                    户住房，按售房款10%提取的维修资金                     元，购房人交纳的1%维修资金                    元。我单位 |            我单位出售                    户住房，按售房款10%提取的维修资金                     元，购房人交纳的1%维修资金                    元。我单位 |            我单位出售                    户住房，按售房款10%提取的维修资金                     元，购房人交纳的1%维修资金                    元。我单位 |            我单位出售                    户住房，按售房款10%提取的维修资金                     元，购房人交纳的1%维修资金                    元。我单位 |            我单位出售                    户住房，按售房款10%提取的维修资金                     元，购房人交纳的1%维修资金                    元。我单位 |            我单位出售</t>
+        </is>
+      </c>
+      <c r="K27" s="62" t="inlineStr"/>
+      <c r="L27" s="62" t="inlineStr"/>
+      <c r="M27" s="62" t="inlineStr">
+        <is>
+          <t>25/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="280" customHeight="1">
+      <c r="A28" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B28" s="62" t="inlineStr"/>
+      <c r="C28" s="62" t="inlineStr"/>
+      <c r="D28" s="62" t="inlineStr"/>
+      <c r="E28" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F28" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G28" s="62" t="inlineStr"/>
+      <c r="H28" s="62" t="inlineStr"/>
+      <c r="I28" s="62" t="inlineStr"/>
+      <c r="J28" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">                    户住房，按售房款10%提取的维修资金                     元，购房人交纳的1%维修资金                    元。我单位 |            我单位出售                    户住房，按售房款10%提取的维修资金                     元，购房人交纳的1%维修资金                    元。我单位 |            我单位出售                    户住房，按售房款10%提取的维修资金                     元，购房人交纳的1%维修资金                    元。我单位 |            我单位出售                    户住房，按售房款10%提取的维修资金                     元，购房人交纳的1%维修资金                    元。我单位 |            我单位出售                    户住房，按售房款10%提取的维修资金                     元，购房人交纳的1%维修资金                    元。我单位 |            我单位出售                    户住房，按售房款10%提取的维修资金                     元，购房人交纳的1%维修资金                    元。我单位
+原文依据：负责对维修资金本息余额自行提出记账到每户住房的分摊意见，并记账到每户住房，同时对使用的维修资金向购房人做好说明解释工作。 | 负责对维修资金本息余额自行提出记账到每户住房的分摊意见，并记账到每户住房，同时对使用的维修资金向购房人做好说明解释工作。 | 负责对维修资金本息余额自行提出记账到每户住房的分摊意见，并记账到每户住房，同时对使用的维修资金向购房人做好说明解释工作。 | 负责对维修资金本息余额自行提出记账到每户住房的分摊意见，并记账到每户住房，同时对使用的维修资金向购房人做好说明解释工作。 | 负责对维修资金本息余额自行提出记账到每户住房的分摊意见，并记账到每户住房，同时对使用的维修资金向购房人做好说明解释工</t>
+        </is>
+      </c>
+      <c r="K28" s="62" t="inlineStr"/>
+      <c r="L28" s="62" t="inlineStr"/>
+      <c r="M28" s="62" t="inlineStr">
+        <is>
+          <t>26/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="370" customHeight="1">
+      <c r="A29" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B29" s="62" t="inlineStr"/>
+      <c r="C29" s="62" t="inlineStr"/>
+      <c r="D29" s="62" t="inlineStr"/>
+      <c r="E29" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F29" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G29" s="62" t="inlineStr"/>
+      <c r="H29" s="62" t="inlineStr"/>
+      <c r="I29" s="62" t="inlineStr"/>
+      <c r="J29" s="62" t="inlineStr">
+        <is>
+          <t>作。 | 负责对维修资金本息余额自行提出记账到每户住房的分摊意见，并记账到每户住房，同时对使用的维修资金向购房人做好说明解释工作。 | 负责对维修资金本息余额自行提出记账到每户住房的分摊意见，并记账到每户住房，同时对使用的维修资金向购房人做好说明解释工作。 | 负责对维修资金本息余额自行提出记账到每户住房的分摊意见，并记账到每户住房，同时对使用的维修资金向购房人做好说明解释工作。 | 负责对维修资金本息余额自行提出记账到每户住房的分摊意见，并记账到每户住房，同时对使用的维修资金向购房人做好说明解释工作。 | 负责对维修资金本息余额自行提出记账到每户住房的分摊意见，并记账到每户住房，同时对使用的维修资金向购房人做好说明解释工作。 | 负责对维修资金本息余额自行提出记账到每户住房的分摊意见，并记账到每户住房，同时对使用的维修资金向购房人做好说明解释工作。 | 负责对维修资金本息余额自行提出记账到每户住房的分摊意见，并记账到每户住房，同时对使用的维修资金向购房人做好说明解释工作。 | 负责对维修资金本息余额自行提出记账到每户住房的分摊意见，并记账到每户住房，同时对使用的维修资金向购房人做好说明解释工作。 | 负责对维修资金本息余额自行提出记账到每户住房的分摊意见，并记账到每户住房，同时对使用的维修资金向购房人做好说明解释工作。 | 负责对维修资金本息余额自行提出记账到每户住房的分摊意见，并记账到每户住房，同时对使用的维修资金向购房人做好说明解释工作。 | 负责对维修资金本息余额自行提出记账到每户住房的分摊意见，并记账到每户住房，同时对使用的维修资金向购房人做好说明解释工作。 | 负责对维修资金本息余额自行提出记账到每户住房的分摊意见，并记账到每户住房，同时对使用的维修资金向购房人做好说明解释工作。
+原文依据：特此具结 |       特此具结 |       特此具结 |       特此具结 |       特此具结 |       特此具结 |       特此具结 |       特此具结 |       特此具结 |       特此具结 |       特此具结 |       特此具结 |       特此具结 |       特此具结 |       特此具结 |       特此具结 |       特此具结
+原文依据：售房单位意见（加盖公章） | 售</t>
+        </is>
+      </c>
+      <c r="K29" s="62" t="inlineStr"/>
+      <c r="L29" s="62" t="inlineStr"/>
+      <c r="M29" s="62" t="inlineStr">
+        <is>
+          <t>27/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="295" customHeight="1">
+      <c r="A30" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B30" s="62" t="inlineStr"/>
+      <c r="C30" s="62" t="inlineStr"/>
+      <c r="D30" s="62" t="inlineStr"/>
+      <c r="E30" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F30" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G30" s="62" t="inlineStr"/>
+      <c r="H30" s="62" t="inlineStr"/>
+      <c r="I30" s="62" t="inlineStr"/>
+      <c r="J30" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">房单位意见（加盖公章） | 售房单位意见（加盖公章） | 单位加盖预留银行印鉴 | 单位加盖预留银行印鉴 | 单位加盖预留银行印鉴 | 单位加盖预留银行印鉴 | 主管区局意见 | 主管区局意见 | 主管区局意见 | 主管区局意见 | 主管区局意见 | 主管区局意见 | 主管区局意见 | 主管区局意见 | 主管区局意见 | 主管区局意见
+原文依据：| 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 |  |  |  |  |  |  | 　 |
+原文依据：经办人：              年      月        日 | 经办人：              年      月        日 | 经办人：              年      月        日 | 经办人：            年      月        日 | 经办人：            年      月        日 | 经办人：            年      月        日 | 经办人：            年      月        日 | 经办人：              年      月        日　 | 经办人：              年      月        日　 | 经办人：              年      月        日　 | 经办人：              年      月        日　 | 经办人：              年      月        日　 | 经办人：              年      月        日　 | 经办人：              年      月        日　 | 经办人：              年      月        日　 | 经办人：              年      月        日　 | 经办人：              年      月        日
+原文依据：年        月        日 |                      年        月        日 |                      年        月        日 |     </t>
+        </is>
+      </c>
+      <c r="K30" s="62" t="inlineStr"/>
+      <c r="L30" s="62" t="inlineStr"/>
+      <c r="M30" s="62" t="inlineStr">
+        <is>
+          <t>28/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="280" customHeight="1">
+      <c r="A31" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B31" s="62" t="inlineStr"/>
+      <c r="C31" s="62" t="inlineStr"/>
+      <c r="D31" s="62" t="inlineStr"/>
+      <c r="E31" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F31" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G31" s="62" t="inlineStr"/>
+      <c r="H31" s="62" t="inlineStr"/>
+      <c r="I31" s="62" t="inlineStr"/>
+      <c r="J31" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">         年        月        日 |              年        月        日 |              年        月        日 |              年        月        日 |                       年        月          日 |                       年        月          日 |                       年        月          日 |                       年        月          日 |                       年        月          日 |                       年        月          日 |                       年        月          日 |                       年        月          日 |                       年        月          日 |                       年        月          日
+原文依据：注：本表一式三联，第一联售房单位留存；第二联承办银行交审核部门备案；第三联承办银行留存。 |     注：本表一式三联，第一联售房单位留存；第二联承办银行交审核部门备案；第三联承办银行留存。 |     注：本表一式三联，第一联售房单位留存；第二联承办银行交审核部门备案；第三联承办银行留存。 |     注：本表一式三联，第一联售房单位留存；第二联承办银行交审核部门备案；第三联承办银行留存。 |     注：本表一式三联，第一联售房单位留存；第二联承办银行交审核部门备案；第三联承办银行留存。 |     注：本表一式三联，第一联售房单位留存；第二联承办银行交审核部门备案；第三联承办银行留存。 |     注：本表一式三联，第一联售房单位留存；第二联承办银行交审核部门备案；第三联承办银行留存。 |     注：本表一式三联，第一联售房单位留存；第二联承办银行交审核部门备案；第三联承办银行留存</t>
+        </is>
+      </c>
+      <c r="K31" s="62" t="inlineStr"/>
+      <c r="L31" s="62" t="inlineStr"/>
+      <c r="M31" s="62" t="inlineStr">
+        <is>
+          <t>29/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="409" customHeight="1">
+      <c r="A32" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B32" s="62" t="inlineStr"/>
+      <c r="C32" s="62" t="inlineStr"/>
+      <c r="D32" s="62" t="inlineStr"/>
+      <c r="E32" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F32" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G32" s="62" t="inlineStr"/>
+      <c r="H32" s="62" t="inlineStr"/>
+      <c r="I32" s="62" t="inlineStr"/>
+      <c r="J32" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">。 |     注：本表一式三联，第一联售房单位留存；第二联承办银行交审核部门备案；第三联承办银行留存。 |     注：本表一式三联，第一联售房单位留存；第二联承办银行交审核部门备案；第三联承办银行留存。 |     注：本表一式三联，第一联售房单位留存；第二联承办银行交审核部门备案；第三联承办银行留存。 |     注：本表一式三联，第一联售房单位留存；第二联承办银行交审核部门备案；第三联承办银行留存。 |     注：本表一式三联，第一联售房单位留存；第二联承办银行交审核部门备案；第三联承办银行留存。 |     注：本表一式三联，第一联售房单位留存；第二联承办银行交审核部门备案；第三联承办银行留存。 |     注：本表一式三联，第一联售房单位留存；第二联承办银行交审核部门备案；第三联承办银行留存。 |     注：本表一式三联，第一联售房单位留存；第二联承办银行交审核部门备案；第三联承办银行留存。 |     注：本表一式三联，第一联售房单位留存；第二联承办银行交审核部门备案；第三联承办银行留存。
+原文依据：单位名称（全称）： | 单位名称（全称）： | 单位名称（全称）： |  | 单位：元
+原文依据：序号 | 业主姓名 | 住房地址 | 10%维修资金余额 | 1%维修资金余额
+原文依据：| 　 | 　 | 　 |
+原文依据：合计（本页小计） | 合计（本页小计） | 合计（本页小计） | 　 |
+原文依据：注：本表一式三联，第一联售房单位留存；第二联承办银行交审核部门备存；第三联承办银行留存。 |     注：本表一式三联，第一联售房单位留存；第二联承办银行交审核部门备存；第三联承办银行留存。 |     注：本表一式三联，第一联售房单位留存；第二联承办银行交审核部门备存；第三联承办银行留存。 |     注：本表一式三联，第一联售房单位留存；第二联承办银行交审核部门备存；第三联承办银行留存。 |     注：本表一式三联，第一联售房单位留存；第二联承办银行交审核部门备存；第三联承办银行留存。
+原文依据：单位名称 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 |
+原文依据：单位代码 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 |
+原文依据：收款开户行 | 　 | 　</t>
+        </is>
+      </c>
+      <c r="K32" s="62" t="inlineStr"/>
+      <c r="L32" s="62" t="inlineStr"/>
+      <c r="M32" s="62" t="inlineStr">
+        <is>
+          <t>30/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="409" customHeight="1">
+      <c r="A33" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B33" s="62" t="inlineStr"/>
+      <c r="C33" s="62" t="inlineStr"/>
+      <c r="D33" s="62" t="inlineStr"/>
+      <c r="E33" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F33" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G33" s="62" t="inlineStr"/>
+      <c r="H33" s="62" t="inlineStr"/>
+      <c r="I33" s="62" t="inlineStr"/>
+      <c r="J33" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 |
+原文依据：收款账号 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 |
+原文依据：维修地点 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 |
+原文依据：涉及售后公房户数（户） | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 |
+原文依据：涉及建筑面积（m2） | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 |
+原文依据：提取金额合计（大写） |  佰    拾    万
+  仟    佰    拾
+  元    角  分整 | 佰 | 拾 | 万 | 仟 | 佰  | 拾 | 元 | 角 | 分 | 分
+原文依据：提取金额合计（大写） |  佰    拾    万
+  仟    佰    拾
+  元    角  分整 | 　 | 　 | 　 | 　 | 　 | 　 | 　 |  |  |
+原文依据：其中 | 11%维修资金 | 　 | 　 | 　 | 　 | 　 | 　 | 　 |  |  |
+原文依据：其中 | 14.4%更新改造资金 |  |  |  |  |  |  |  |  |  |
+原文依据：其中 | 电梯、水泵更新改造资金 | 　 | 　 | 　 | 　 | 　 | 　 | 　 |  |  |
+原文依据：售房单位意见
+（公章）
+经办人：                  负责人：
+年      月     日 | 售房单位意见
+（公章）
+经办人：                  负责人：
+年      月     日 | 
+ | 
+ | 
+ | 
+ | 
+ | 
+ | 
+ | 
+ |
+原文依据：审核部门意见
+（公章）
+经办人：                  负责人：
+                 年       月        日 | 审核部门意见
+（公章）
+经办人：                  负责人：
+                 年       月        日 | 银行受理
+经办人：
+年      月      日 | 银行受理
+经办人：
+年      月      日 | 银行受理
+经办人：
+</t>
+        </is>
+      </c>
+      <c r="K33" s="62" t="inlineStr"/>
+      <c r="L33" s="62" t="inlineStr"/>
+      <c r="M33" s="62" t="inlineStr">
+        <is>
+          <t>31/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="409" customHeight="1">
+      <c r="A34" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B34" s="62" t="inlineStr"/>
+      <c r="C34" s="62" t="inlineStr"/>
+      <c r="D34" s="62" t="inlineStr"/>
+      <c r="E34" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F34" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G34" s="62" t="inlineStr"/>
+      <c r="H34" s="62" t="inlineStr"/>
+      <c r="I34" s="62" t="inlineStr"/>
+      <c r="J34" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">年      月      日 | 银行受理
+经办人：
+年      月      日 | 银行受理
+经办人：
+年      月      日 | 银行受理
+经办人：
+年      月      日 | 银行受理
+经办人：
+年      月      日 | 银行受理
+经办人：
+年      月      日 | 银行受理
+经办人：
+年      月      日
+原文依据：售房单位名称（全称） |  |  | 售房单位代码 | 售房单位代码 | 售房单位代码 | 售房单位代码 | 售房单位代码 | 售房单位代码 |  |  |  |  |  |
+原文依据：收款账号 |  |  | 收款开户行 | 收款开户行 | 收款开户行 | 收款开户行 | 收款开户行 | 收款开户行 |  |  |  |  |  |
+原文依据：售房单位类型 | 直管产（         ）保管自修产（         ）单位产（         ） | 直管产（         ）保管自修产（         ）单位产（         ） | 直管产（         ）保管自修产（         ）单位产（         ） | 直管产（         ）保管自修产（         ）单位产（         ） | 直管产（         ）保管自修产（         ）单位产（         ） | 直管产（         ）保管自修产（         ）单位产（         ） | 直管产（         ）保管自修产（         ）单位产（         ） | 直管产（         ）保管自修产（         ）单位产（         ） | 直管产（         ）保管自修产（         ）单位产（         ） | 直管产（         ）保管自修产（         ）单位产（         ） | 直管产（         ）保管自修产（         ）单位产（         ） | 直管产（         ）保管自修产（         ）单位产（         ） | 直管产（         ）保管自修产（         ）单位产（         ） | 直管产（    </t>
+        </is>
+      </c>
+      <c r="K34" s="62" t="inlineStr"/>
+      <c r="L34" s="62" t="inlineStr"/>
+      <c r="M34" s="62" t="inlineStr">
+        <is>
+          <t>32/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="409" customHeight="1">
+      <c r="A35" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B35" s="62" t="inlineStr"/>
+      <c r="C35" s="62" t="inlineStr"/>
+      <c r="D35" s="62" t="inlineStr"/>
+      <c r="E35" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F35" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G35" s="62" t="inlineStr"/>
+      <c r="H35" s="62" t="inlineStr"/>
+      <c r="I35" s="62" t="inlineStr"/>
+      <c r="J35" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     ）保管自修产（         ）单位产（         ）
+原文依据：房屋地址 | （使用应急抢险资金时填写） | （使用应急抢险资金时填写） | （使用应急抢险资金时填写） | （使用应急抢险资金时填写） | （使用应急抢险资金时填写） | （使用应急抢险资金时填写） | （使用应急抢险资金时填写） | （使用应急抢险资金时填写） | （使用应急抢险资金时填写） | （使用应急抢险资金时填写） | （使用应急抢险资金时填写） | （使用应急抢险资金时填写） | （使用应急抢险资金时填写） | （使用应急抢险资金时填写）
+原文依据：申请提取金额合计 | 仟  佰  拾  万  仟  佰  拾  元  角  分 | 仟  佰  拾  万  仟  佰  拾  元  角  分 | 仟  佰  拾  万  仟  佰  拾  元  角  分 | 仟 | 佰 | 拾 | 万 | 仟 | 仟 | 佰 | 拾 | 元 | 角 | 分
+原文依据：申请提取金额合计 | 仟  佰  拾  万  仟  佰  拾  元  角  分 | 仟  佰  拾  万  仟  佰  拾  元  角  分 | 仟  佰  拾  万  仟  佰  拾  元  角  分 |  |  |  |  |  |  |  |  |  |  |
+原文依据：其
+中 | 5.6%应急抢险资金 | 5.6%应急抢险资金 | 5.6%应急抢险资金 |  |  |  |  |  |  |  |  |  |  |
+原文依据：其
+中 | 公房售前维修和售后维修资金 | 公房售前维修和售后维修资金 | 公房售前维修和售后维修资金 |  |  |  |  |  |  |  |  |  |  |
+原文依据：其
+中 | 严重损坏房屋改造资金 | 严重损坏房屋改造资金 | 严重损坏房屋改造资金 |  |  |  |  |  |  |  |  |  |  |
+原文依据：其
+中 | 房屋管理储备资金 | 房屋管理储备资金 | 房屋管理储备资金 |  |  |  |  |  |  |  |  |  |  |
+原文依据：其
+中 | 售房经费 | 售房经费 | 售房经费 |  |  |  |  |  |  |  |  |  |  |
+原文依据：其
+中 | 房管事业发展基金 | 房管事业发展基金 | 房管事业发展</t>
+        </is>
+      </c>
+      <c r="K35" s="62" t="inlineStr"/>
+      <c r="L35" s="62" t="inlineStr"/>
+      <c r="M35" s="62" t="inlineStr">
+        <is>
+          <t>33/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="409" customHeight="1">
+      <c r="A36" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B36" s="62" t="inlineStr"/>
+      <c r="C36" s="62" t="inlineStr"/>
+      <c r="D36" s="62" t="inlineStr"/>
+      <c r="E36" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F36" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G36" s="62" t="inlineStr"/>
+      <c r="H36" s="62" t="inlineStr"/>
+      <c r="I36" s="62" t="inlineStr"/>
+      <c r="J36" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">基金 |  |  |  |  |  |  |  |  |  |  |
+原文依据：其
+中 | 住房货币分配 | 住房货币分配 | 住房货币分配 |  |  |  |  |  |  |  |  |  |  |
+原文依据：其
+中 | 转换经营机制 | 转换经营机制 | 转换经营机制 |  |  |  |  |  |  |  |  |  |  |
+原文依据：其
+中 | 退房 | 退房 | 退房 |  |  |  |  |  |  |  |  |  |  |
+原文依据：售房单位意见
+（公章）
+经办人：      负责人：         年   月   日 | 售房单位意见
+（公章）
+经办人：      负责人：         年   月   日 | 上级部门意见
+（公章）
+经办人：                    年   月   日 | 上级部门意见
+（公章）
+经办人：                    年   月   日 | 上级部门意见
+（公章）
+经办人：                    年   月   日 | 上级部门意见
+（公章）
+经办人：                    年   月   日 | 上级部门意见
+（公章）
+经办人：                    年   月   日 | 上级部门意见
+（公章）
+经办人：                    年   月   日 | 上级部门意见
+（公章）
+经办人：                    年   月   日 | 上级部门意见
+（公章）
+经办人：                    年   月   日 | 上级部门意见
+（公章）
+经办人：                    年   月   日 | 上级部门意见
+（公章）
+经办人：                    年   月   日 | 上级部门意见
+（公章）
+经办人：                    年   月   日 | 上级部门意见
+（公章）
+经办人：                    年   月   日 | 上级部门意见
+（公章）
+经办人：                    年   月   日
+原文依据：审核部门意见
+（公章）
+经办人：       </t>
+        </is>
+      </c>
+      <c r="K36" s="62" t="inlineStr"/>
+      <c r="L36" s="62" t="inlineStr"/>
+      <c r="M36" s="62" t="inlineStr">
+        <is>
+          <t>34/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="409" customHeight="1">
+      <c r="A37" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B37" s="62" t="inlineStr"/>
+      <c r="C37" s="62" t="inlineStr"/>
+      <c r="D37" s="62" t="inlineStr"/>
+      <c r="E37" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F37" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G37" s="62" t="inlineStr"/>
+      <c r="H37" s="62" t="inlineStr"/>
+      <c r="I37" s="62" t="inlineStr"/>
+      <c r="J37" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">负责人：          年   月   日 | 审核部门意见
+（公章）
+经办人：       负责人：          年   月   日 | 银行受理
+经办人：
+                            年   月   日 | 银行受理
+经办人：
+                            年   月   日 | 银行受理
+经办人：
+                            年   月   日 | 银行受理
+经办人：
+                            年   月   日 | 银行受理
+经办人：
+                            年   月   日 | 银行受理
+经办人：
+                            年   月   日 | 银行受理
+经办人：
+                            年   月   日 | 银行受理
+经办人：
+                            年   月   日 | 银行受理
+经办人：
+                            年   月   日 | 银行受理
+经办人：
+                            年   月   日 | 银行受理
+经办人：
+                            年   月   日 | 银行受理
+经办人：
+                            年   月   日 | 银行受理
+经办人：
+                            年   月   日
+原文依据：单位名称： | 单位名称： | 单位名称： |  | 售房单位代码： |  |  | 年   月   日
+原文依据：序号 | 个人账号 | 住房地址 | 建筑面积 （m2) | 维修资金
+11% | 更新改造资金
+14.4% | 电梯水泵      更新改造资金 | 业主签字
+原文依据：| 　 |  | 　 | 　 | 　 |  |
+原文依据：|  | 　 | 　 | 　 | 　 |  |
+原文依据：|  |  |  |  |  |  |
+原文依据：|  | 合计（本页小计） | 　 | 　 | 　</t>
+        </is>
+      </c>
+      <c r="K37" s="62" t="inlineStr"/>
+      <c r="L37" s="62" t="inlineStr"/>
+      <c r="M37" s="62" t="inlineStr">
+        <is>
+          <t>35/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="280" customHeight="1">
+      <c r="A38" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B38" s="62" t="inlineStr"/>
+      <c r="C38" s="62" t="inlineStr"/>
+      <c r="D38" s="62" t="inlineStr"/>
+      <c r="E38" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F38" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G38" s="62" t="inlineStr"/>
+      <c r="H38" s="62" t="inlineStr"/>
+      <c r="I38" s="62" t="inlineStr"/>
+      <c r="J38" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> |  |
+原文依据：天津市公有住房出售收入转移申请书 | 天津市公有住房出售收入转移申请书 | 天津市公有住房出售收入转移申请书 | 天津市公有住房出售收入转移申请书 | 天津市公有住房出售收入转移申请书 | 天津市公有住房出售收入转移申请书 | 天津市公有住房出售收入转移申请书 | 天津市公有住房出售收入转移申请书 | 天津市公有住房出售收入转移申请书 | 天津市公有住房出售收入转移申请书 | 天津市公有住房出售收入转移申请书 | 天津市公有住房出售收入转移申请书 | 天津市公有住房出售收入转移申请书 | 天津市公有住房出售收入转移申请书
+原文依据：年    月    日 |                                                                                                         年    月    日 |                                                                                                         年    月    日 |                                                                                                         年    月    日 |                                                                                                         年    月    日 |                                                                                                         年    月    日 |                                                                                                         年    月    </t>
+        </is>
+      </c>
+      <c r="K38" s="62" t="inlineStr"/>
+      <c r="L38" s="62" t="inlineStr"/>
+      <c r="M38" s="62" t="inlineStr">
+        <is>
+          <t>36/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="235" customHeight="1">
+      <c r="A39" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B39" s="62" t="inlineStr"/>
+      <c r="C39" s="62" t="inlineStr"/>
+      <c r="D39" s="62" t="inlineStr"/>
+      <c r="E39" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F39" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G39" s="62" t="inlineStr"/>
+      <c r="H39" s="62" t="inlineStr"/>
+      <c r="I39" s="62" t="inlineStr"/>
+      <c r="J39" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">日 |                                                                                                         年    月    日 |                                                                                                         年    月    日 |                                                                                                         年    月    日 |                                                                                                         年    月    日 |                                                                                                         年    月    日 |                                                                                                         年    月    日 |                                                                                                         年    月    日
+原文依据：转移原因 | 1、单位更名（ ）2、住房灭失（ ）3、单位破产、撤销、兼并（ ）4、房屋转让（ ）5、调账（ ）6、其他（ ） | 1、单位更名（ ）2、住房灭失（ ）3、单位破产、撤销、兼并（ ）4、房屋转让（ ）5、调账（ ）6、其他（ ） | 1、单位更名（ ）2、住房灭失（ ）3、单位破产、撤销、兼并（ ）4、房屋转让（ </t>
+        </is>
+      </c>
+      <c r="K39" s="62" t="inlineStr"/>
+      <c r="L39" s="62" t="inlineStr"/>
+      <c r="M39" s="62" t="inlineStr">
+        <is>
+          <t>37/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="385" customHeight="1">
+      <c r="A40" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B40" s="62" t="inlineStr"/>
+      <c r="C40" s="62" t="inlineStr"/>
+      <c r="D40" s="62" t="inlineStr"/>
+      <c r="E40" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F40" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G40" s="62" t="inlineStr"/>
+      <c r="H40" s="62" t="inlineStr"/>
+      <c r="I40" s="62" t="inlineStr"/>
+      <c r="J40" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">）5、调账（ ）6、其他（ ） | 1、单位更名（ ）2、住房灭失（ ）3、单位破产、撤销、兼并（ ）4、房屋转让（ ）5、调账（ ）6、其他（ ） | 1、单位更名（ ）2、住房灭失（ ）3、单位破产、撤销、兼并（ ）4、房屋转让（ ）5、调账（ ）6、其他（ ） | 1、单位更名（ ）2、住房灭失（ ）3、单位破产、撤销、兼并（ ）4、房屋转让（ ）5、调账（ ）6、其他（ ） | 1、单位更名（ ）2、住房灭失（ ）3、单位破产、撤销、兼并（ ）4、房屋转让（ ）5、调账（ ）6、其他（ ） | 1、单位更名（ ）2、住房灭失（ ）3、单位破产、撤销、兼并（ ）4、房屋转让（ ）5、调账（ ）6、其他（ ） | 1、单位更名（ ）2、住房灭失（ ）3、单位破产、撤销、兼并（ ）4、房屋转让（ ）5、调账（ ）6、其他（ ） | 1、单位更名（ ）2、住房灭失（ ）3、单位破产、撤销、兼并（ ）4、房屋转让（ ）5、调账（ ）6、其他（ ） | 1、单位更名（ ）2、住房灭失（ ）3、单位破产、撤销、兼并（ ）4、房屋转让（ ）5、调账（ ）6、其他（ ） | 1、单位更名（ ）2、住房灭失（ ）3、单位破产、撤销、兼并（ ）4、房屋转让（ ）5、调账（ ）6、其他（ ） | 1、单位更名（ ）2、住房灭失（ ）3、单位破产、撤销、兼并（ ）4、房屋转让（ ）5、调账（ ）6、其他（ ）
+原文依据：| 转移前 | 转移前 | 转移前 | 转移后 | 转移后 | 转移后 | 转移后 | 转移后 | 转移后 | 转移后 | 转移后 | 转移后 | 转移后
+原文依据：售房单位名称 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 |
+原文依据：售房单位代码 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 |
+原文依据：售房单位地址 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 |
+原文依据：联系人、联系电话 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 |
+原文依据：购房人 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | </t>
+        </is>
+      </c>
+      <c r="K40" s="62" t="inlineStr"/>
+      <c r="L40" s="62" t="inlineStr"/>
+      <c r="M40" s="62" t="inlineStr">
+        <is>
+          <t>38/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="409" customHeight="1">
+      <c r="A41" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B41" s="62" t="inlineStr"/>
+      <c r="C41" s="62" t="inlineStr"/>
+      <c r="D41" s="62" t="inlineStr"/>
+      <c r="E41" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F41" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G41" s="62" t="inlineStr"/>
+      <c r="H41" s="62" t="inlineStr"/>
+      <c r="I41" s="62" t="inlineStr"/>
+      <c r="J41" s="62" t="inlineStr">
+        <is>
+          <t xml:space="preserve">　 |
+原文依据：住房地址 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 |
+原文依据：转移金额合计 | 佰    拾    万    仟    佰    拾   元   角   分整 | 佰    拾    万    仟    佰    拾   元   角   分整 | 佰    拾    万    仟    佰    拾   元   角   分整 | 佰 | 拾 | 万 | 仟 | 仟 | 佰 | 拾 | 元 | 角 | 分
+原文依据：转移金额合计 | 佰    拾    万    仟    佰    拾   元   角   分整 | 佰    拾    万    仟    佰    拾   元   角   分整 | 佰    拾    万    仟    佰    拾   元   角   分整 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 |
+原文依据：维修资金（11%） | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 |
+原文依据：其中：1%维修资金 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 |
+原文依据：更新改造资金（14.4%） | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 |
+原文依据：电梯水泵更新改造资金 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 |
+原文依据：住房基金（75.6） | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 | 　 |
+原文依据：其中：5.6%应急抢险资金 |  |  |  |  |  |  |  |  |  |  |  |  |
+原文依据：转出单位意见 | 转出单位意见 | 转入单位意见 | 审核部门意见 | 审核部门意见 | 审核部门意见 | 审核部门意见 | 审核部门意见 | 银行受理 | 银行受理 | 银行受理 | 银行受理 | 银行受理 | 银行受理
+原文依据：| 　 | 　
+　 | 经办人：       负责人： | 经办人：       负责人： | 经办人：       负责</t>
+        </is>
+      </c>
+      <c r="K41" s="62" t="inlineStr"/>
+      <c r="L41" s="62" t="inlineStr"/>
+      <c r="M41" s="62" t="inlineStr">
+        <is>
+          <t>39/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="355" customHeight="1">
+      <c r="A42" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B42" s="62" t="inlineStr"/>
+      <c r="C42" s="62" t="inlineStr"/>
+      <c r="D42" s="62" t="inlineStr"/>
+      <c r="E42" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F42" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G42" s="62" t="inlineStr"/>
+      <c r="H42" s="62" t="inlineStr"/>
+      <c r="I42" s="62" t="inlineStr"/>
+      <c r="J42" s="62" t="inlineStr">
+        <is>
+          <t>人： | 经办人：       负责人： | 经办人：       负责人： |  |  |  |  |  |
+原文依据：经办人： | 经办人： | 经办人： | 经办人：       负责人： | 经办人：       负责人： | 经办人：       负责人： | 经办人：       负责人： | 经办人：       负责人： |  |  |  |  |  |
+原文依据：联系电话： | 联系电话： | 联系电话： | 联系电话： | 联系电话： | 联系电话： | 联系电话： | 联系电话： | 经办人： | 经办人： | 经办人： | 经办人： | 经办人： | 经办人：
+原文依据：年  月  日 |           年  月  日 |                年  月  日
+        |                   年   月   日 |                   年   月   日 |                   年   月   日 |                   年   月   日 |                   年   月   日 |                   年   月   日 |                   年   月   日 |                   年   月   日 |                   年   月   日 |                   年   月   日 |                   年   月   日
+原文依据：备注：资金在集中账户系统内转移的，应当填写售房单位代码；转出集中账户系统的，在转移后售房单位代码处，填写收款账户账号。 | 备注：资金在集中账户系统内转移的，应当填写售房单位代码；转出集中账户系统的，在转移后售房单位代码处，填写收款账户账号。 | 备注：资金在集中账户系统内转移的，应当填写售房单位代码；转出集中账户系统的，在转移后售房单位代码处，填写收款账户账号。 | 备注：资金在集中账户系统内转移的，应当填写售房单位代码；转出集中账户系统的，在转移后售房单位代码处，填写收款账户账号。 | 备注：资金在集中账户系统内转移的，应当填写售房单位代码；转出集中账户系统的，在转移后售房单位代码处，填</t>
+        </is>
+      </c>
+      <c r="K42" s="62" t="inlineStr"/>
+      <c r="L42" s="62" t="inlineStr"/>
+      <c r="M42" s="62" t="inlineStr">
+        <is>
+          <t>40/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="370" customHeight="1">
+      <c r="A43" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B43" s="62" t="inlineStr"/>
+      <c r="C43" s="62" t="inlineStr"/>
+      <c r="D43" s="62" t="inlineStr"/>
+      <c r="E43" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F43" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G43" s="62" t="inlineStr"/>
+      <c r="H43" s="62" t="inlineStr"/>
+      <c r="I43" s="62" t="inlineStr"/>
+      <c r="J43" s="62" t="inlineStr">
+        <is>
+          <t>写收款账户账号。 | 备注：资金在集中账户系统内转移的，应当填写售房单位代码；转出集中账户系统的，在转移后售房单位代码处，填写收款账户账号。 | 备注：资金在集中账户系统内转移的，应当填写售房单位代码；转出集中账户系统的，在转移后售房单位代码处，填写收款账户账号。 | 备注：资金在集中账户系统内转移的，应当填写售房单位代码；转出集中账户系统的，在转移后售房单位代码处，填写收款账户账号。 | 备注：资金在集中账户系统内转移的，应当填写售房单位代码；转出集中账户系统的，在转移后售房单位代码处，填写收款账户账号。 | 备注：资金在集中账户系统内转移的，应当填写售房单位代码；转出集中账户系统的，在转移后售房单位代码处，填写收款账户账号。 | 备注：资金在集中账户系统内转移的，应当填写售房单位代码；转出集中账户系统的，在转移后售房单位代码处，填写收款账户账号。 | 备注：资金在集中账户系统内转移的，应当填写售房单位代码；转出集中账户系统的，在转移后售房单位代码处，填写收款账户账号。 | 备注：资金在集中账户系统内转移的，应当填写售房单位代码；转出集中账户系统的，在转移后售房单位代码处，填写收款账户账号。 | 备注：资金在集中账户系统内转移的，应当填写售房单位代码；转出集中账户系统的，在转移后售房单位代码处，填写收款账户账号。
+原文依据：注：本表一式五联：第一联售房单位留存；第二、三联市住房保障服务中心留存；第四联承办银行留存；第五联审核部门留存。第一至四联加盖承办银行代天津市出售公有住房业务受理专用章后生效。 | 注：本表一式五联：第一联售房单位留存；第二、三联市住房保障服务中心留存；第四联承办银行留存；第五联审核部门留存。第一至四联加盖承办银行代天津市出售公有住房业务受理专用章后生效。 | 注：本表一式五联：第一联售房单位留存；第二、三联市住房保障服务中心留存；第四联承办银行留存；第五联审核部门留存。第一至四联加盖承办银行代天津市出售公有住房业务受理专用章后生效。 | 注：本表一式五联：第一联售房单位留存；第二、三联市住房保障服务中心留存；第四联承办银行留存；第五联审核部门留存。第一至四联加盖承办银行代天津市出售公有住房业务受理专用章后生效。 | 注：本表一式五联：第一联售房单位留存；第二、三联市住房保障服务中心留存；第四联承办银行留存；第五联审核部门留存。第一至四联加盖</t>
+        </is>
+      </c>
+      <c r="K43" s="62" t="inlineStr"/>
+      <c r="L43" s="62" t="inlineStr"/>
+      <c r="M43" s="62" t="inlineStr">
+        <is>
+          <t>41/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="409" customHeight="1">
+      <c r="A44" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B44" s="62" t="inlineStr"/>
+      <c r="C44" s="62" t="inlineStr"/>
+      <c r="D44" s="62" t="inlineStr"/>
+      <c r="E44" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F44" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G44" s="62" t="inlineStr"/>
+      <c r="H44" s="62" t="inlineStr"/>
+      <c r="I44" s="62" t="inlineStr"/>
+      <c r="J44" s="62" t="inlineStr">
+        <is>
+          <t>承办银行代天津市出售公有住房业务受理专用章后生效。 | 注：本表一式五联：第一联售房单位留存；第二、三联市住房保障服务中心留存；第四联承办银行留存；第五联审核部门留存。第一至四联加盖承办银行代天津市出售公有住房业务受理专用章后生效。 | 注：本表一式五联：第一联售房单位留存；第二、三联市住房保障服务中心留存；第四联承办银行留存；第五联审核部门留存。第一至四联加盖承办银行代天津市出售公有住房业务受理专用章后生效。 | 注：本表一式五联：第一联售房单位留存；第二、三联市住房保障服务中心留存；第四联承办银行留存；第五联审核部门留存。第一至四联加盖承办银行代天津市出售公有住房业务受理专用章后生效。 | 注：本表一式五联：第一联售房单位留存；第二、三联市住房保障服务中心留存；第四联承办银行留存；第五联审核部门留存。第一至四联加盖承办银行代天津市出售公有住房业务受理专用章后生效。 | 注：本表一式五联：第一联售房单位留存；第二、三联市住房保障服务中心留存；第四联承办银行留存；第五联审核部门留存。第一至四联加盖承办银行代天津市出售公有住房业务受理专用章后生效。 | 注：本表一式五联：第一联售房单位留存；第二、三联市住房保障服务中心留存；第四联承办银行留存；第五联审核部门留存。第一至四联加盖承办银行代天津市出售公有住房业务受理专用章后生效。 | 注：本表一式五联：第一联售房单位留存；第二、三联市住房保障服务中心留存；第四联承办银行留存；第五联审核部门留存。第一至四联加盖承办银行代天津市出售公有住房业务受理专用章后生效。 | 注：本表一式五联：第一联售房单位留存；第二、三联市住房保障服务中心留存；第四联承办银行留存；第五联审核部门留存。第一至四联加盖承办银行代天津市出售公有住房业务受理专用章后生效。 | 注：本表一式五联：第一联售房单位留存；第二、三联市住房保障服务中心留存；第四联承办银行留存；第五联审核部门留存。第一至四联加盖承办银行代天津市出售公有住房业务受理专用章后生效。
+原文依据：原承办银行单位名称 | 原承办银行单位名称 |  | 转入银行单位名称 |
+原文依据：原承办银行单位代码 | 原承办银行单位代码 |  | 转入银行单位代码 |
+原文依据：专
+项
+维
+修
+资
+金 | 转出银行账号 | 转出银行账号 | 12001220800059999993 | 120012</t>
+        </is>
+      </c>
+      <c r="K44" s="62" t="inlineStr"/>
+      <c r="L44" s="62" t="inlineStr"/>
+      <c r="M44" s="62" t="inlineStr">
+        <is>
+          <t>42/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="409" customHeight="1">
+      <c r="A45" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B45" s="62" t="inlineStr"/>
+      <c r="C45" s="62" t="inlineStr"/>
+      <c r="D45" s="62" t="inlineStr"/>
+      <c r="E45" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F45" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G45" s="62" t="inlineStr"/>
+      <c r="H45" s="62" t="inlineStr"/>
+      <c r="I45" s="62" t="inlineStr"/>
+      <c r="J45" s="62" t="inlineStr">
+        <is>
+          <t>20800059999993
+原文依据：专
+项
+维
+修
+资
+金 | 转入银行账号 | 转入银行账号 | 358001201110004263 | 358001201110004263
+原文依据：专
+项
+维
+修
+资
+金 | 25.4%划转金额（大写） | 25.4%划转金额（大写） |  |
+原文依据：专
+项
+维
+修
+资
+金 | 25.4%划转金额（小写） | 25.4%划转金额（小写） |  |
+原文依据：专
+项
+维
+修
+资
+金 | 其中：1%维修资金 | 其中：1%维修资金 |  |
+原文依据：专
+项
+维
+修
+资
+金 | 10%维修资金 | 10%维修资金 |  |
+原文依据：专
+项
+维
+修
+资
+金 |          14.4%更新改造资金 |          14.4%更新改造资金 |  |
+原文依据：住
+房
+基
+金 | 转出银行账号 | 转出银行账号 | 12001220800059999991 | 12001220800059999991
+原文依据：住
+房
+基
+金 | 转入银行账号 | 转入银行账号 | 358001201110004355 | 358001201110004355
+原文依据：住
+房
+基
+金 | 75.6%划转金额（大写） | 75.6%划转金额（大写） |  |
+原文依据：住
+房
+基
+金 | 75.6%划转金额（小写） | 75.6%划转金额（小写） |  |
+原文依据：住
+房
+基
+金 | 其中：应急抢险资金5.6% | 其中：应急抢险资金5.6% |  |
+原文依据：住
+房
+基
+金 | 其余资金 | 其余资金 |  |
+原文依据：售房单位(签章)
+经办人：
+负责人：                 年 月 日 | 售房单位(签章)
+经办人：
+负责人：                 年 月 日 | 售房单位(签章)
+经办人：
+负责人：                 年 月 日 | 区住建委(签章)
+经办人：
+负责人：               年 月 日 | 区住建委(签章)
+经办人：
+负责人：               年 月 日</t>
+        </is>
+      </c>
+      <c r="K45" s="62" t="inlineStr"/>
+      <c r="L45" s="62" t="inlineStr"/>
+      <c r="M45" s="62" t="inlineStr">
+        <is>
+          <t>43/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="370" customHeight="1">
+      <c r="A46" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="B46" s="60" t="inlineStr">
+        <is>
+          <t>三亚市商品房预售展期公告</t>
+        </is>
+      </c>
+      <c r="C46" s="60" t="inlineStr">
+        <is>
+          <t>三亚</t>
+        </is>
+      </c>
+      <c r="D46" s="60" t="inlineStr">
+        <is>
+          <t>住建 / 房管</t>
+        </is>
+      </c>
+      <c r="E46" s="61" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F46" s="60" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G46" s="60" t="inlineStr">
+        <is>
+          <t>正式文件</t>
+        </is>
+      </c>
+      <c r="H46" s="60" t="inlineStr">
+        <is>
+          <t>未关联监测事项</t>
+        </is>
+      </c>
+      <c r="I46" s="60" t="inlineStr">
+        <is>
+          <t>原文摘录（非模型总结）
+一、开发建设单位必须依照《中华人民共和国城市房地产管理法》、《城市商品房预售管理办法》及有关法律法规进行商品房预售。
+二、该项目预售款监管银行： 海南银行股份有限公司三亚分行 ， 监管账号： 6001 1156 00035 。</t>
+        </is>
+      </c>
+      <c r="J46" s="60" t="inlineStr">
+        <is>
+          <t>原文依据：三亚市商品房预售 展期 公告
+原文依据：三房预许字（ 展期 ）〔 20 20 〕 19 号
+原文依据：三亚市住房和城乡建设局以三房预许字（ 展期 ）〔 20 20 〕 19 号《商品房预售许可证》 （编号： 202 6 — 28 号）， 批准 亚龙湾 1 号度假酒店（亚龙湾畔山酒店重建）项目 2# — 5# 、 7# 、 8# 、 11# — 16# 、 32# — 35# 独立式客房， 建筑层数为地上 2 — 3 层 预售 （展期） ， 批准预售展期建筑面积 14143.13 平方米 （其中：地上 7794.24 平方米，地下 6348.89 平方米） ，房屋套数 16 套，全部未网签。 该项目 位于三亚市吉阳区亚龙湾开发区龙塘路 ， 不动产权证书 ： 三土房（ 2007 ）字第 8170 号、三土房（ 2010 ）字第 02400 号 ， 由 海南金盛投资管理有限公司 开发建设。现就有关事项公告如下 ：
+原文依据：一、开发建设单位必须依照《中华人民共和国城市房地产管理法》、《城市商品房预售管理办法》及有关法律法规进行商品房预售。
+原文依据：二、该项目预售款监管银行： 海南银行股份有限公司三亚分行 ， 监管账号： 6001 1156 00035 。
+原文依据：三、该项目批准预售有效期为 2 年（即 202 6 年 9 月 24 日至 202 8 年 9 月 23 日 ）。 同时我局于 2023 年 3 月28日核发的原三房预许字（展期） 〔 202 0 〕 19 号作废。
+原文依据：三亚市住房和城乡建设局
+原文依据：202 6 年 9 月 24 日</t>
+        </is>
+      </c>
+      <c r="K46" s="60" t="inlineStr">
+        <is>
+          <t>https://zj.sanya.gov.cn/zjjsite/bmwjxx/202609/a1e7ba2f349f423088fbfdcd272f37e9.shtml</t>
+        </is>
+      </c>
+      <c r="L46" s="60" t="inlineStr">
+        <is>
+          <t>待关联事项</t>
+        </is>
+      </c>
+      <c r="M46" s="60" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="370" customHeight="1">
+      <c r="A47" s="62" t="n">
+        <v>4</v>
+      </c>
+      <c r="B47" s="62" t="inlineStr">
+        <is>
+          <t>三亚市商品房预售展期公告</t>
+        </is>
+      </c>
+      <c r="C47" s="62" t="inlineStr">
+        <is>
+          <t>三亚</t>
+        </is>
+      </c>
+      <c r="D47" s="62" t="inlineStr">
+        <is>
+          <t>住建 / 房管</t>
+        </is>
+      </c>
+      <c r="E47" s="63" t="n">
+        <v>46295</v>
+      </c>
+      <c r="F47" s="62" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G47" s="62" t="inlineStr">
+        <is>
+          <t>正式文件</t>
+        </is>
+      </c>
+      <c r="H47" s="62" t="inlineStr">
+        <is>
+          <t>未关联监测事项</t>
+        </is>
+      </c>
+      <c r="I47" s="62" t="inlineStr">
+        <is>
+          <t>原文摘录（非模型总结）
+一、开发建设单位必须依照《中华人民共和国城市房地产管理法》、《城市商品房预售管理办法》及有关法律法规进行商品房预售。
+二、该项目预售款监管银行：中国光大银行股份有限公司三亚大东海支行 ， 监管账号： 3939 0188 0000 67815 。</t>
+        </is>
+      </c>
+      <c r="J47" s="62" t="inlineStr">
+        <is>
+          <t>原文依据：三亚市商品房预售 展期 公告
+原文依据：三房预许字（展期） 〔 2023 〕 52 号
+原文依据：三亚市住房和城乡建设局以三房预许字（展期） 〔 2023 〕 52 号《商品房预售许可证》 （编号： 202 6—27 号） ，批准亚龙湾 1 号度假酒店（亚龙湾畔山酒店重建）项目 1# 、 9# 、 10# 、 17#—22# 、 24#—26# 、 36#—39# 独立式客房， 建筑层数为地上 2—3 层 预售（展期）， 批准预售展期建筑面积 9413.58 平方米 （其中：地上 6169.79 平方米，地下 3243.79 平方米） ，预售展期房屋套数 16 套，全部未网签。 该项目位于三亚市吉阳区亚龙湾开发区龙塘路，不动产权证书：三土房（ 2007 ）字第 8170 号、三土房（ 2010 ）字第 02400 号 ，由海南金盛投资管理有限公司开发建设。现就有关事项公告如下：
+原文依据：一、开发建设单位必须依照《中华人民共和国城市房地产管理法》、《城市商品房预售管理办法》及有关法律法规进行商品房预售。
+原文依据：二、该项目预售款监管银行：中国光大银行股份有限公司三亚大东海支行 ， 监管账号： 3939 0188 0000 67815 。
+原文依据：三、该项目批准预售有效期为 2 年（即 202 6 年 9 月 24 日至 202 8 年 9 月 23 日 ）。 同时我局于 2023 年 7 月 27 日核发的原三房预许字 〔 2023 〕 52 号作废。
+原文依据：三亚市住房和城乡建设局
+原文依据：202 6 年 9 月 24 日</t>
+        </is>
+      </c>
+      <c r="K47" s="62" t="inlineStr">
+        <is>
+          <t>https://zj.sanya.gov.cn/zjjsite/bmwjxx/202609/35acfea256ed49b49564083e3506c0f4.shtml</t>
+        </is>
+      </c>
+      <c r="L47" s="62" t="inlineStr">
+        <is>
+          <t>待关联事项</t>
+        </is>
+      </c>
+      <c r="M47" s="62" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="409" customHeight="1">
+      <c r="A48" s="60" t="n">
+        <v>5</v>
+      </c>
+      <c r="B48" s="60" t="inlineStr">
+        <is>
           <t>北京市住房和城乡建设委员会等4部门关于发布本市贯彻落实《关于完善商品住房销售制度的通知》的实施意见</t>
         </is>
       </c>
-      <c r="C2" s="60" t="inlineStr">
+      <c r="C48" s="60" t="inlineStr">
         <is>
           <t>北京</t>
         </is>
       </c>
-      <c r="D2" s="60" t="inlineStr">
+      <c r="D48" s="60" t="inlineStr">
         <is>
           <t>住建 / 房管、公积金</t>
         </is>
       </c>
-      <c r="E2" s="61" t="n">
+      <c r="E48" s="61" t="n">
         <v>46289</v>
       </c>
-      <c r="F2" s="60" t="inlineStr">
+      <c r="F48" s="60" t="inlineStr">
         <is>
           <t>原文载明 2026-09-24 施行；现行效力及项目适用性未核验</t>
         </is>
       </c>
-      <c r="G2" s="60" t="inlineStr">
+      <c r="G48" s="60" t="inlineStr">
         <is>
           <t>正式文件</t>
         </is>
       </c>
-      <c r="H2" s="60" t="inlineStr">
+      <c r="H48" s="60" t="inlineStr">
         <is>
           <t>省市房地产新规实施导则及细则出台情况
 工规证新老划断认定时间节点
@@ -2969,7 +5147,7 @@
 执行主办银行制的存量项目范围</t>
         </is>
       </c>
-      <c r="I2" s="60" t="inlineStr">
+      <c r="I48" s="60" t="inlineStr">
         <is>
           <t>省市房地产新规实施导则及细则出台情况
 原文摘录（非模型总结）
@@ -2988,7 +5166,7 @@
 （二）在途项目。 2026年8月28日（含）前，已取得 （含部分取得） 建设工程规划许可证但未办理预售许可的商品住房项目 ，</t>
         </is>
       </c>
-      <c r="J2" s="60" t="inlineStr">
+      <c r="J48" s="60" t="inlineStr">
         <is>
           <t>适用条件：本实施意见自发布之日起执行。此前所发文件相关内容与本实施意见不一致的，按本实施意见规定执行。
 原文依据：为贯彻落实《住房城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知》（建房规〔2026〕3号）有关要求，加快构建房地产发展新模式，稳步推进商品住房销售制度改革，结合本市实际，提出如下实施意见 。
@@ -3001,41 +5179,41 @@
 原文依据：</t>
         </is>
       </c>
-      <c r="K2" s="60" t="inlineStr">
+      <c r="K48" s="60" t="inlineStr">
         <is>
           <t>https://zjw.beijing.gov.cn/bjjs/xxgk/zcwj2024/qtzcwj/xxyx13/744131235/index.shtml
 https://gjj.beijing.gov.cn/web/zwgk61/2024zcwj/436433464/436433468/744131565/index.html</t>
         </is>
       </c>
-      <c r="L2" s="60" t="inlineStr">
+      <c r="L48" s="60" t="inlineStr">
         <is>
           <t>已关联事项</t>
         </is>
       </c>
-      <c r="M2" s="60" t="inlineStr">
+      <c r="M48" s="60" t="inlineStr">
         <is>
           <t>1/3</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="409" customHeight="1">
-      <c r="A3" s="60" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="60" t="inlineStr"/>
-      <c r="C3" s="60" t="inlineStr"/>
-      <c r="D3" s="60" t="inlineStr"/>
-      <c r="E3" s="61" t="n">
+    <row r="49" ht="409" customHeight="1">
+      <c r="A49" s="60" t="n">
+        <v>5</v>
+      </c>
+      <c r="B49" s="60" t="inlineStr"/>
+      <c r="C49" s="60" t="inlineStr"/>
+      <c r="D49" s="60" t="inlineStr"/>
+      <c r="E49" s="61" t="n">
         <v>46289</v>
       </c>
-      <c r="F3" s="60" t="inlineStr">
+      <c r="F49" s="60" t="inlineStr">
         <is>
           <t>原文载明 2026-09-24 施行；现行效力及项目适用性未核验</t>
         </is>
       </c>
-      <c r="G3" s="60" t="inlineStr"/>
-      <c r="H3" s="60" t="inlineStr"/>
-      <c r="I3" s="60" t="inlineStr">
+      <c r="G49" s="60" t="inlineStr"/>
+      <c r="H49" s="60" t="inlineStr"/>
+      <c r="I49" s="60" t="inlineStr">
         <is>
           <t>申请 预售的，预售条件、预售资金监管等按原有政策规定执行。
 按揭贷款发放条件（新政后首次领取预售证项目）
@@ -3060,7 +5238,7 @@
 监管资金</t>
         </is>
       </c>
-      <c r="J3" s="60" t="inlineStr">
+      <c r="J49" s="60" t="inlineStr">
         <is>
           <t>（一）新取得土地项目。 2026年8月28日后 新发布国有 建设用地 使用权出让公告的商品住房项目， 申请 预售 的 ，单体建筑 应 完成主体结构封顶 （楼栋顶板及楼顶构筑物、配套设施完成混凝土浇筑）， 项目 建设单位、勘察、设计、施工、监理 等单位 应出具 签字 盖章 的《主体结构分部工程验收记录》 。项目 预售资金全额 、全过程监管 ，项目 联合验收后 ， 方可 解除资金监管。 具体预售资金监管办法另行印发。
 适用条件：（一）规范个人按揭贷款发放。 2026年8月28日后取得预售许可证的项目，竣工备案后方可发放个人住房按揭贷款（含公积金贷款），贷款资金应当通过受托支付方式支付至预售资金监管账户。
@@ -3073,32 +5251,32 @@
 原文依据：房地产开发企业在主办银行开立资金账户，项目存续期间，开发贷款、项目自有资金、</t>
         </is>
       </c>
-      <c r="K3" s="60" t="inlineStr"/>
-      <c r="L3" s="60" t="inlineStr"/>
-      <c r="M3" s="60" t="inlineStr">
+      <c r="K49" s="60" t="inlineStr"/>
+      <c r="L49" s="60" t="inlineStr"/>
+      <c r="M49" s="60" t="inlineStr">
         <is>
           <t>2/3</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="409" customHeight="1">
-      <c r="A4" s="60" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="60" t="inlineStr"/>
-      <c r="C4" s="60" t="inlineStr"/>
-      <c r="D4" s="60" t="inlineStr"/>
-      <c r="E4" s="61" t="n">
+    <row r="50" ht="409" customHeight="1">
+      <c r="A50" s="60" t="n">
+        <v>5</v>
+      </c>
+      <c r="B50" s="60" t="inlineStr"/>
+      <c r="C50" s="60" t="inlineStr"/>
+      <c r="D50" s="60" t="inlineStr"/>
+      <c r="E50" s="61" t="n">
         <v>46289</v>
       </c>
-      <c r="F4" s="60" t="inlineStr">
+      <c r="F50" s="60" t="inlineStr">
         <is>
           <t>原文载明 2026-09-24 施行；现行效力及项目适用性未核验</t>
         </is>
       </c>
-      <c r="G4" s="60" t="inlineStr"/>
-      <c r="H4" s="60" t="inlineStr"/>
-      <c r="I4" s="60" t="inlineStr">
+      <c r="G50" s="60" t="inlineStr"/>
+      <c r="H50" s="60" t="inlineStr"/>
+      <c r="I50" s="60" t="inlineStr">
         <is>
           <t>管理细则（含开发贷、预售款等）
 原文摘录（非模型总结）
@@ -3112,7 +5290,7 @@
 2026年8月28日后签订开发贷合同的商品住房项目，贷款银行单独提供开发贷的，贷款银行为主办银行；贷款银行组建银团提供贷款的， 银团贷款牵头银行为主办银行 。</t>
         </is>
       </c>
-      <c r="J4" s="60" t="inlineStr">
+      <c r="J50" s="60" t="inlineStr">
         <is>
           <t>现房销售资金等与项目相关的全部资金均应纳入在主办银行开立的资金账户管理。市住房资金管理中心在主办银行开立资金监管账户，用于存放监管项目预售资金和现房定金。
 原文依据：三、推行主办银行制度
@@ -3126,54 +5304,54 @@
 原文依据：2026年8月28日后签订开发贷合同的商品住房项目，贷款银行单独提供开发贷的，贷款银行为主办银行；贷款银行组建银团提供贷款的， 银团贷款牵头银行为主办银行 。</t>
         </is>
       </c>
-      <c r="K4" s="60" t="inlineStr"/>
-      <c r="L4" s="60" t="inlineStr"/>
-      <c r="M4" s="60" t="inlineStr">
+      <c r="K50" s="60" t="inlineStr"/>
+      <c r="L50" s="60" t="inlineStr"/>
+      <c r="M50" s="60" t="inlineStr">
         <is>
           <t>3/3</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="409" customHeight="1">
-      <c r="A5" s="62" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="62" t="inlineStr">
+    <row r="51" ht="409" customHeight="1">
+      <c r="A51" s="62" t="n">
+        <v>6</v>
+      </c>
+      <c r="B51" s="62" t="inlineStr">
         <is>
           <t>关于调整住房公积金贷款有关政策的通知</t>
         </is>
       </c>
-      <c r="C5" s="62" t="inlineStr">
+      <c r="C51" s="62" t="inlineStr">
         <is>
           <t>石家庄</t>
         </is>
       </c>
-      <c r="D5" s="62" t="inlineStr">
+      <c r="D51" s="62" t="inlineStr">
         <is>
           <t>公积金</t>
         </is>
       </c>
-      <c r="E5" s="63" t="n">
+      <c r="E51" s="63" t="n">
         <v>46283</v>
       </c>
-      <c r="F5" s="62" t="inlineStr">
+      <c r="F51" s="62" t="inlineStr">
         <is>
           <t>原文载明 2026-09-20 施行；现行效力及项目适用性未核验</t>
         </is>
       </c>
-      <c r="G5" s="62" t="inlineStr">
+      <c r="G51" s="62" t="inlineStr">
         <is>
           <t>正式文件</t>
         </is>
       </c>
-      <c r="H5" s="62" t="inlineStr">
+      <c r="H51" s="62" t="inlineStr">
         <is>
           <t>住房公积金贷款额度及上浮
 住房套数认定与贷款资格
 配套解读：住房公积金贷款政策解读</t>
         </is>
       </c>
-      <c r="I5" s="62" t="inlineStr">
+      <c r="I51" s="62" t="inlineStr">
         <is>
           <t>住房公积金贷款额度及上浮
 原文摘录（非模型总结）
@@ -3229,7 +5407,7 @@
 缴存人家庭购买长安区、桥西区、新华</t>
         </is>
       </c>
-      <c r="J5" s="62" t="inlineStr">
+      <c r="J51" s="62" t="inlineStr">
         <is>
           <t>适用条件：2
 现行政策基础上提高20万元。 
@@ -3282,40 +5460,40 @@
 县、井陉矿区住房，单方缴存最高</t>
         </is>
       </c>
-      <c r="K5" s="62" t="inlineStr">
+      <c r="K51" s="62" t="inlineStr">
         <is>
           <t>https://www.sjzgjj.cn/tzgg/2489.jhtml</t>
         </is>
       </c>
-      <c r="L5" s="62" t="inlineStr">
+      <c r="L51" s="62" t="inlineStr">
         <is>
           <t>已关联事项</t>
         </is>
       </c>
-      <c r="M5" s="62" t="inlineStr">
+      <c r="M51" s="62" t="inlineStr">
         <is>
           <t>1/2</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="409" customHeight="1">
-      <c r="A6" s="62" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="62" t="inlineStr"/>
-      <c r="C6" s="62" t="inlineStr"/>
-      <c r="D6" s="62" t="inlineStr"/>
-      <c r="E6" s="63" t="n">
+    <row r="52" ht="409" customHeight="1">
+      <c r="A52" s="62" t="n">
+        <v>6</v>
+      </c>
+      <c r="B52" s="62" t="inlineStr"/>
+      <c r="C52" s="62" t="inlineStr"/>
+      <c r="D52" s="62" t="inlineStr"/>
+      <c r="E52" s="63" t="n">
         <v>46283</v>
       </c>
-      <c r="F6" s="62" t="inlineStr">
+      <c r="F52" s="62" t="inlineStr">
         <is>
           <t>原文载明 2026-09-20 施行；现行效力及项目适用性未核验</t>
         </is>
       </c>
-      <c r="G6" s="62" t="inlineStr"/>
-      <c r="H6" s="62" t="inlineStr"/>
-      <c r="I6" s="62" t="inlineStr">
+      <c r="G52" s="62" t="inlineStr"/>
+      <c r="H52" s="62" t="inlineStr"/>
+      <c r="I52" s="62" t="inlineStr">
         <is>
           <t>区、裕华区、高新
 区范围内自住住房的，其住房套数按拟购住房所在区认定。 
@@ -3339,7 +5517,7 @@
 贷款的，贷款额度不超过房屋总价的50%。</t>
         </is>
       </c>
-      <c r="J6" s="62" t="inlineStr">
+      <c r="J52" s="62" t="inlineStr">
         <is>
           <t>贷款额度60万元，双方缴存最
 高贷款额度80万元。 
@@ -3369,53 +5547,53 @@
 贷款的，贷款额度不超过房屋总价的50%。</t>
         </is>
       </c>
-      <c r="K6" s="62" t="inlineStr"/>
-      <c r="L6" s="62" t="inlineStr"/>
-      <c r="M6" s="62" t="inlineStr">
+      <c r="K52" s="62" t="inlineStr"/>
+      <c r="L52" s="62" t="inlineStr"/>
+      <c r="M52" s="62" t="inlineStr">
         <is>
           <t>2/2</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="409" customHeight="1">
-      <c r="A7" s="60" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="60" t="inlineStr">
+    <row r="53" ht="409" customHeight="1">
+      <c r="A53" s="60" t="n">
+        <v>7</v>
+      </c>
+      <c r="B53" s="60" t="inlineStr">
         <is>
           <t>关于开展装修提取住房公积金业务的通知</t>
         </is>
       </c>
-      <c r="C7" s="60" t="inlineStr">
+      <c r="C53" s="60" t="inlineStr">
         <is>
           <t>石家庄</t>
         </is>
       </c>
-      <c r="D7" s="60" t="inlineStr">
+      <c r="D53" s="60" t="inlineStr">
         <is>
           <t>公积金</t>
         </is>
       </c>
-      <c r="E7" s="61" t="n">
+      <c r="E53" s="61" t="n">
         <v>46283</v>
       </c>
-      <c r="F7" s="60" t="inlineStr">
+      <c r="F53" s="60" t="inlineStr">
         <is>
           <t>未找到可核验的生效日期</t>
         </is>
       </c>
-      <c r="G7" s="60" t="inlineStr">
+      <c r="G53" s="60" t="inlineStr">
         <is>
           <t>正式文件</t>
         </is>
       </c>
-      <c r="H7" s="60" t="inlineStr">
+      <c r="H53" s="60" t="inlineStr">
         <is>
           <t>住房公积金装修提取
 配套解读：住房公积金装修提取政策解读</t>
         </is>
       </c>
-      <c r="I7" s="60" t="inlineStr">
+      <c r="I53" s="60" t="inlineStr">
         <is>
           <t>住房公积金装修提取
 原文摘录（非模型总结）
@@ -3445,7 +5623,7 @@
 记时间为准。因补发、变更、析产等原因换发不动产权证书的，</t>
         </is>
       </c>
-      <c r="J7" s="60" t="inlineStr">
+      <c r="J53" s="60" t="inlineStr">
         <is>
           <t>适用条件：1
 石家庄住房公积金管理中心 
@@ -3501,41 +5679,41 @@
 （二）2026 年 9 月</t>
         </is>
       </c>
-      <c r="K7" s="60" t="inlineStr">
+      <c r="K53" s="60" t="inlineStr">
         <is>
           <t>https://www.sjzgjj.cn/tzgg/2488.jhtml</t>
         </is>
       </c>
-      <c r="L7" s="60" t="inlineStr">
+      <c r="L53" s="60" t="inlineStr">
         <is>
           <t>已关联事项</t>
         </is>
       </c>
-      <c r="M7" s="60" t="inlineStr">
+      <c r="M53" s="60" t="inlineStr">
         <is>
           <t>1/2</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="385" customHeight="1">
-      <c r="A8" s="60" t="n">
-        <v>3</v>
-      </c>
-      <c r="B8" s="60" t="inlineStr"/>
-      <c r="C8" s="60" t="inlineStr"/>
-      <c r="D8" s="60" t="inlineStr"/>
-      <c r="E8" s="61" t="n">
+    <row r="54" ht="385" customHeight="1">
+      <c r="A54" s="60" t="n">
+        <v>7</v>
+      </c>
+      <c r="B54" s="60" t="inlineStr"/>
+      <c r="C54" s="60" t="inlineStr"/>
+      <c r="D54" s="60" t="inlineStr"/>
+      <c r="E54" s="61" t="n">
         <v>46283</v>
       </c>
-      <c r="F8" s="60" t="inlineStr">
+      <c r="F54" s="60" t="inlineStr">
         <is>
           <t>未找到可核验的生效日期</t>
         </is>
       </c>
-      <c r="G8" s="60" t="inlineStr"/>
-      <c r="H8" s="60" t="inlineStr"/>
-      <c r="I8" s="60" t="inlineStr"/>
-      <c r="J8" s="60" t="inlineStr">
+      <c r="G54" s="60" t="inlineStr"/>
+      <c r="H54" s="60" t="inlineStr"/>
+      <c r="I54" s="60" t="inlineStr"/>
+      <c r="J54" s="60" t="inlineStr">
         <is>
           <t>20日（含）以后，在本市行政区域内取
 得不动产权证书的自住住房。 
@@ -3563,48 +5741,48 @@
 知不一致的，以本通知为准。</t>
         </is>
       </c>
-      <c r="K8" s="60" t="inlineStr"/>
-      <c r="L8" s="60" t="inlineStr"/>
-      <c r="M8" s="60" t="inlineStr">
+      <c r="K54" s="60" t="inlineStr"/>
+      <c r="L54" s="60" t="inlineStr"/>
+      <c r="M54" s="60" t="inlineStr">
         <is>
           <t>2/2</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="409" customHeight="1">
-      <c r="A9" s="62" t="n">
-        <v>4</v>
-      </c>
-      <c r="B9" s="62" t="inlineStr">
+    <row r="55" ht="409" customHeight="1">
+      <c r="A55" s="62" t="n">
+        <v>8</v>
+      </c>
+      <c r="B55" s="62" t="inlineStr">
         <is>
           <t>住房和城乡建设部 自然资源部 金融监管总局关于完善商品住房销售制度的通知</t>
         </is>
       </c>
-      <c r="C9" s="62" t="inlineStr">
+      <c r="C55" s="62" t="inlineStr">
         <is>
           <t>国家基准 / 参考
 省级政策参考，城市执行细则需另行核实</t>
         </is>
       </c>
-      <c r="D9" s="62" t="inlineStr">
+      <c r="D55" s="62" t="inlineStr">
         <is>
           <t>国家部委</t>
         </is>
       </c>
-      <c r="E9" s="63" t="n">
+      <c r="E55" s="63" t="n">
         <v>46262</v>
       </c>
-      <c r="F9" s="62" t="inlineStr">
+      <c r="F55" s="62" t="inlineStr">
         <is>
           <t>原文载明 2026-08-28 施行；现行效力及项目适用性未核验</t>
         </is>
       </c>
-      <c r="G9" s="62" t="inlineStr">
+      <c r="G55" s="62" t="inlineStr">
         <is>
           <t>正式文件</t>
         </is>
       </c>
-      <c r="H9" s="62" t="inlineStr">
+      <c r="H55" s="62" t="inlineStr">
         <is>
           <t>省市房地产新规实施导则及细则出台情况
 工规证新老划断认定时间节点
@@ -3617,7 +5795,7 @@
 主办银行选择原则（企业自主选择/政府指定）</t>
         </is>
       </c>
-      <c r="I9" s="62" t="inlineStr">
+      <c r="I55" s="62" t="inlineStr">
         <is>
           <t>省市房地产新规实施导则及细则出台情况
 原文摘录（非模型总结）
@@ -3644,7 +5822,7 @@
 (三)推行现房销售定金制。实行现房销售的商品住房项目,在取得建筑工程施工许可证后,房地产开发企业可与购房人签</t>
         </is>
       </c>
-      <c r="J9" s="62" t="inlineStr">
+      <c r="J55" s="62" t="inlineStr">
         <is>
           <t>适用条件：为贯彻落实党中央、国务院关于加快构建房地产发展新模式的决策部署,坚持稳中求进、先立后破,稳步推进商品住房销售制度改革,现就有关事项通知如下。
 适用条件：(三)优化存量项目预售管理。本通知施行之日前已取得建设工程规划许可证的商品住房项目,实行预售的,预售条件、预售资金监管等按原有政策规定执行。应合理确定监管额度,优化预售资金使用,严格预售资金监管,保障预售资金安全。
@@ -3660,40 +5838,40 @@
 原文依据：(一)优化土地供应管理。市县要优化国土空间规划和土地利用方式,按照住房发展规划和年度计划,合理确定房地产用地供应规模。统筹规划、合理布局商品住宅用地,优化土地出让方案,可带规划方案出让。房地产开发企业须用自有资金购地,可按国家规定分期缴纳土地出让价款,具体缴纳比例和时限由市县人民</t>
         </is>
       </c>
-      <c r="K9" s="62" t="inlineStr">
+      <c r="K55" s="62" t="inlineStr">
         <is>
           <t>https://www.hunan.gov.cn/zqt/zcsd/202609/t20260907_34057926.html</t>
         </is>
       </c>
-      <c r="L9" s="62" t="inlineStr">
+      <c r="L55" s="62" t="inlineStr">
         <is>
           <t>已关联事项</t>
         </is>
       </c>
-      <c r="M9" s="62" t="inlineStr">
+      <c r="M55" s="62" t="inlineStr">
         <is>
           <t>1/3</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="409" customHeight="1">
-      <c r="A10" s="62" t="n">
-        <v>4</v>
-      </c>
-      <c r="B10" s="62" t="inlineStr"/>
-      <c r="C10" s="62" t="inlineStr"/>
-      <c r="D10" s="62" t="inlineStr"/>
-      <c r="E10" s="63" t="n">
+    <row r="56" ht="409" customHeight="1">
+      <c r="A56" s="62" t="n">
+        <v>8</v>
+      </c>
+      <c r="B56" s="62" t="inlineStr"/>
+      <c r="C56" s="62" t="inlineStr"/>
+      <c r="D56" s="62" t="inlineStr"/>
+      <c r="E56" s="63" t="n">
         <v>46262</v>
       </c>
-      <c r="F10" s="62" t="inlineStr">
+      <c r="F56" s="62" t="inlineStr">
         <is>
           <t>原文载明 2026-08-28 施行；现行效力及项目适用性未核验</t>
         </is>
       </c>
-      <c r="G10" s="62" t="inlineStr"/>
-      <c r="H10" s="62" t="inlineStr"/>
-      <c r="I10" s="62" t="inlineStr">
+      <c r="G56" s="62" t="inlineStr"/>
+      <c r="H56" s="62" t="inlineStr"/>
+      <c r="I56" s="62" t="inlineStr">
         <is>
           <t>订购房定金合同,依法收取少量定金。购房定金合同应约定定金金额、商品住房售价、交付时间及不能按期履约的责任等,保护双方合法权益。市县住房和城乡建设部门履行定金监管职责,住房资金监管机构承担定金监管工作,在项目的主办银行开立定金监管账户。房屋具备交付条件后,解除定金监管。房地产开发企业违约不能按期交房的,购房人有权按照合同约定提出解除定金合同,房地产开发企业依法返还定金,承担违约责任。各地要结合实际制定购房定金合同示范文本。
 监管资金管理细则（含开发贷、预售款等）
@@ -3705,7 +5883,7 @@
 (二)加大融资支持力度。房地产项目实行主办银行制,房地产项目开发公司和主办银行双向选择,一个项目确定一家主办银行,主办银行单独或牵头组建银团提供开发贷款等融资服务。房地产项目开发公司以土地使用权抵押申请开发贷款的,应以分户土地使用权集合设定抵押,相关办法另行制定。支持房地产项目开发公司通过股权、债券等多种方式开展融资。对实行现房销售和预售的项目,按照市场化原则满足项目合理融资需求,实现开发贷款发放与项目建设周期相匹配。</t>
         </is>
       </c>
-      <c r="J10" s="62" t="inlineStr">
+      <c r="J56" s="62" t="inlineStr">
         <is>
           <t>政府确定。对于实行现房销售的项目,在土地出让公告中向社会公开现房销售相关信息。
 适用条件：(三)推行现房销售定金制。实行现房销售的商品住房项目,在取得建筑工程施工许可证后,房地产开发企业可与购房人签订购房定金合同,依法收取少量定金。购房定金合同应约定定金金额、商品住房售价、交付时间及不能按期履约的责任等,保护双方合法权益。市县住房和城乡建设部门履行定金监管职责,住房资金监管机构承担定金监管工作,在项目的主办银行开立定金监管账户。房屋具备交付条件后,解除定金监管。房地产开发企业违约不能按期交房的,购房人有权按照合同约定提出解除定金合同,房地产开发企业依法返还定金,承担违约责任。各地要结合实际制定购房定金合同示范文本。
@@ -3715,80 +5893,80 @@
 原文依据：(二)加强预售资金监管。市县住房和城乡建设部门履行预售资金监管职责,由住房资金监管机构承担具体监管工作。住房资金监管机构应与房地产开发企业签订资金监管协议,并在项目的主办银行开立资金监管账户。购房人支付的首付款、个人住</t>
         </is>
       </c>
-      <c r="K10" s="62" t="inlineStr"/>
-      <c r="L10" s="62" t="inlineStr"/>
-      <c r="M10" s="62" t="inlineStr">
+      <c r="K56" s="62" t="inlineStr"/>
+      <c r="L56" s="62" t="inlineStr"/>
+      <c r="M56" s="62" t="inlineStr">
         <is>
           <t>2/3</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="160" customHeight="1">
-      <c r="A11" s="62" t="n">
-        <v>4</v>
-      </c>
-      <c r="B11" s="62" t="inlineStr"/>
-      <c r="C11" s="62" t="inlineStr"/>
-      <c r="D11" s="62" t="inlineStr"/>
-      <c r="E11" s="63" t="n">
+    <row r="57" ht="160" customHeight="1">
+      <c r="A57" s="62" t="n">
+        <v>8</v>
+      </c>
+      <c r="B57" s="62" t="inlineStr"/>
+      <c r="C57" s="62" t="inlineStr"/>
+      <c r="D57" s="62" t="inlineStr"/>
+      <c r="E57" s="63" t="n">
         <v>46262</v>
       </c>
-      <c r="F11" s="62" t="inlineStr">
+      <c r="F57" s="62" t="inlineStr">
         <is>
           <t>原文载明 2026-08-28 施行；现行效力及项目适用性未核验</t>
         </is>
       </c>
-      <c r="G11" s="62" t="inlineStr"/>
-      <c r="H11" s="62" t="inlineStr"/>
-      <c r="I11" s="62" t="inlineStr"/>
-      <c r="J11" s="62" t="inlineStr">
+      <c r="G57" s="62" t="inlineStr"/>
+      <c r="H57" s="62" t="inlineStr"/>
+      <c r="I57" s="62" t="inlineStr"/>
+      <c r="J57" s="62" t="inlineStr">
         <is>
           <t>房贷款等购房资金应全部存入资金监管账户。商品住房项目竣工验收、水电气热等配套设施具备交付条件后,解除资金监管。房地产开发企业违约不能按期交房的,购房人有权按照合同约定提出解除购房合同,房地产开发企业须按照合同约定退还购房资金并承担违约责任。房地产开发企业应与购房人在购房合同中约定购房资金存入资金监管账户的相关权利责任。
 原文依据：(二)加大融资支持力度。房地产项目实行主办银行制,房地产项目开发公司和主办银行双向选择,一个项目确定一家主办银行,主办银行单独或牵头组建银团提供开发贷款等融资服务。房地产项目开发公司以土地使用权抵押申请开发贷款的,应以分户土地使用权集合设定抵押,相关办法另行制定。支持房地产项目开发公司通过股权、债券等多种方式开展融资。对实行现房销售和预售的项目,按照市场化原则满足项目合理融资需求,实现开发贷款发放与项目建设周期相匹配。</t>
         </is>
       </c>
-      <c r="K11" s="62" t="inlineStr"/>
-      <c r="L11" s="62" t="inlineStr"/>
-      <c r="M11" s="62" t="inlineStr">
+      <c r="K57" s="62" t="inlineStr"/>
+      <c r="L57" s="62" t="inlineStr"/>
+      <c r="M57" s="62" t="inlineStr">
         <is>
           <t>3/3</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="409" customHeight="1">
-      <c r="A12" s="60" t="n">
-        <v>5</v>
-      </c>
-      <c r="B12" s="60" t="inlineStr">
+    <row r="58" ht="409" customHeight="1">
+      <c r="A58" s="60" t="n">
+        <v>9</v>
+      </c>
+      <c r="B58" s="60" t="inlineStr">
         <is>
           <t>中国人民银行 国家金融监督管理总局印发《关于改革完善房地产信贷管理 推动加快构建房地产发展新模式的意见》的通知（银发〔2026〕171号）</t>
         </is>
       </c>
-      <c r="C12" s="60" t="inlineStr">
+      <c r="C58" s="60" t="inlineStr">
         <is>
           <t>国家基准 / 参考
 省级政策参考，城市执行细则需另行核实</t>
         </is>
       </c>
-      <c r="D12" s="60" t="inlineStr">
+      <c r="D58" s="60" t="inlineStr">
         <is>
           <t>国家部委</t>
         </is>
       </c>
-      <c r="E12" s="61" t="n">
+      <c r="E58" s="61" t="n">
         <v>46262</v>
       </c>
-      <c r="F12" s="60" t="inlineStr">
+      <c r="F58" s="60" t="inlineStr">
         <is>
           <t>原文载明 2026-08-28 施行；现行效力及项目适用性未核验</t>
         </is>
       </c>
-      <c r="G12" s="60" t="inlineStr">
+      <c r="G58" s="60" t="inlineStr">
         <is>
           <t>正式文件</t>
         </is>
       </c>
-      <c r="H12" s="60" t="inlineStr">
+      <c r="H58" s="60" t="inlineStr">
         <is>
           <t>按揭贷款发放条件（新政后首次领取预售证项目）
 按揭贷款发放条件（新政后非首次领取预售证项目--续销项目）
@@ -3797,7 +5975,7 @@
 主办银行选择原则（企业自主选择/政府指定）</t>
         </is>
       </c>
-      <c r="I12" s="60" t="inlineStr">
+      <c r="I58" s="60" t="inlineStr">
         <is>
           <t>按揭贷款发放条件（新政后首次领取预售证项目）
 原文摘录（非模型总结）
@@ -3820,7 +5998,7 @@
 第十二条 房地产开发贷款实行主办银行制,单个房地产项目对应一家银行作为主办银行(单家贷款行或银团贷款牵头行),对项目资金进行封闭管理。</t>
         </is>
       </c>
-      <c r="J12" s="60" t="inlineStr">
+      <c r="J58" s="60" t="inlineStr">
         <is>
           <t>适用条件：第二十二条 所购新建住房实行现房销售的,个人住房贷款应在销售备案后发放;实行预售的,应严格在项目竣工备案后发放。
 适用条件：第二十三条 银行业金融机构发放个人住房贷款应要求借款人以所购住房作为抵押。对于暂未取得所购住房不动产权属证书或其他情形无法办理抵押登记的,银行业金融机构应视情要求借款人办理抵押预告登记、追加其他阶段性担保等。
@@ -3834,98 +6012,102 @@
 原文依据：第十二条 房地产开发贷款实行主办银行制,单个房地产项目对应一家银行作为主办银行(单家贷款行或银团贷款牵头行),对项目资金进行封闭管理。</t>
         </is>
       </c>
-      <c r="K12" s="60" t="inlineStr">
+      <c r="K58" s="60" t="inlineStr">
         <is>
           <t>https://hunan.gov.cn/zqt/zcsd/202609/t20260907_34058152.html</t>
         </is>
       </c>
-      <c r="L12" s="60" t="inlineStr">
+      <c r="L58" s="60" t="inlineStr">
         <is>
           <t>已关联事项</t>
         </is>
       </c>
-      <c r="M12" s="60" t="inlineStr">
+      <c r="M58" s="60" t="inlineStr">
         <is>
           <t>1/1</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="70" customHeight="1">
-      <c r="A13" s="62" t="n">
-        <v>6</v>
-      </c>
-      <c r="B13" s="62" t="inlineStr">
+    <row r="59" ht="70" customHeight="1">
+      <c r="A59" s="62" t="n">
+        <v>10</v>
+      </c>
+      <c r="B59" s="62" t="inlineStr">
         <is>
           <t>国务院关于修改《住房公积金管理条例》的决定</t>
         </is>
       </c>
-      <c r="C13" s="62" t="inlineStr">
+      <c r="C59" s="62" t="inlineStr">
         <is>
           <t>国家基准 / 参考
 省级政策参考，城市执行细则需另行核实</t>
         </is>
       </c>
-      <c r="D13" s="62" t="inlineStr">
+      <c r="D59" s="62" t="inlineStr">
         <is>
           <t>国家部委、公积金</t>
         </is>
       </c>
-      <c r="E13" s="63" t="n">
+      <c r="E59" s="63" t="n">
         <v>46252</v>
       </c>
-      <c r="F13" s="62" t="inlineStr">
+      <c r="F59" s="62" t="inlineStr">
         <is>
           <t>原文载明 2026-09-20 施行；现行效力及项目适用性未核验</t>
         </is>
       </c>
-      <c r="G13" s="62" t="inlineStr">
+      <c r="G59" s="62" t="inlineStr">
         <is>
           <t>正式文件</t>
         </is>
       </c>
-      <c r="H13" s="62" t="inlineStr">
+      <c r="H59" s="62" t="inlineStr">
         <is>
           <t>住房公积金贷款额度及上浮</t>
         </is>
       </c>
-      <c r="I13" s="62" t="inlineStr">
+      <c r="I59" s="62" t="inlineStr">
         <is>
           <t>住房公积金贷款额度及上浮
 原文摘录（非模型总结）
 （三）确定住房公积金的最高贷款额度；</t>
         </is>
       </c>
-      <c r="J13" s="62" t="inlineStr">
+      <c r="J59" s="62" t="inlineStr">
         <is>
           <t>原文依据：（三）确定住房公积金的最高贷款额度；</t>
         </is>
       </c>
-      <c r="K13" s="62" t="inlineStr">
+      <c r="K59" s="62" t="inlineStr">
         <is>
           <t>https://www.changzhi.gov.cn/xxgkml/zfxxgkml/szfzssydw/czszfgjj/gkgd_202/202608/t20260825_3199027.shtml
 https://www.sjzgjj.cn/gjjwj/2486.jhtml</t>
         </is>
       </c>
-      <c r="L13" s="62" t="inlineStr">
+      <c r="L59" s="62" t="inlineStr">
         <is>
           <t>已关联事项</t>
         </is>
       </c>
-      <c r="M13" s="62" t="inlineStr">
+      <c r="M59" s="62" t="inlineStr">
         <is>
           <t>1/1</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M13"/>
+  <autoFilter ref="A1:M59"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K46" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K47" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K48" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K51" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K53" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K55" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K58" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K59" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
@@ -3938,7 +6120,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4023,44 +6205,116 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="409" customHeight="1">
+    <row r="2" ht="325" customHeight="1">
       <c r="A2" s="60" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="60" t="inlineStr">
         <is>
+          <t>关于办理商品房销售许可核查事项的告知函</t>
+        </is>
+      </c>
+      <c r="C2" s="60" t="inlineStr">
+        <is>
+          <t>三亚</t>
+        </is>
+      </c>
+      <c r="D2" s="60" t="inlineStr">
+        <is>
+          <t>住建 / 房管</t>
+        </is>
+      </c>
+      <c r="E2" s="61" t="n">
+        <v>46307</v>
+      </c>
+      <c r="F2" s="60" t="inlineStr">
+        <is>
+          <t>未找到可核验的生效日期</t>
+        </is>
+      </c>
+      <c r="G2" s="60" t="inlineStr">
+        <is>
+          <t>性质待核验</t>
+        </is>
+      </c>
+      <c r="H2" s="60" t="inlineStr">
+        <is>
+          <t>文件性质待核验</t>
+        </is>
+      </c>
+      <c r="I2" s="60" t="inlineStr">
+        <is>
+          <t>原文摘录（非模型总结）
+我局在办理商品房预售许可、现售备案手续时，仅对土地出让合同中已将履约事项设定为销售许可前置条件的项目，对照土地出让合同、规划审批意见、用地准入协议、项目配建协议等资料进行核查 ， 核查开发建设单位履约情况及产业约定落实情况。未设置该前置条件的项目，不 予 开展履约核查。
+如项目存在特殊情况，确需在审批销售许可时对相关核查事项予以统筹处理的，请贵单位正式出具书面来文说明情况，我局将依据书面意见依法依规办理项目销售许可相关手续。</t>
+        </is>
+      </c>
+      <c r="J2" s="60" t="inlineStr">
+        <is>
+          <t>原文依据：关于办理商品房销售许可核查事项的告知函
+原文依据：三亚市自然资源和规划局、三亚市营商环境建设局、三亚市旅游和文化广电体育局 ， 各管理局 ， 各管理委员会：
+原文依据：为规范房地产市场项目管理，严格落实土地挂牌出让约定、项目配套建设协议的要求，现就项目销售许可相关核查事项 函 告如下：
+原文依据：我局在办理商品房预售许可、现售备案手续时，仅对土地出让合同中已将履约事项设定为销售许可前置条件的项目，对照土地出让合同、规划审批意见、用地准入协议、项目配建协议等资料进行核查 ， 核查开发建设单位履约情况及产业约定落实情况。未设置该前置条件的项目，不 予 开展履约核查。
+原文依据：如项目存在特殊情况，确需在审批销售许可时对相关核查事项予以统筹处理的，请贵单位正式出具书面来文说明情况，我局将依据书面意见依法依规办理项目销售许可相关手续。
+原文依据：此函。
+原文依据：三亚市住房和城乡建设局
+原文依据：2026 年 10 月 12 日</t>
+        </is>
+      </c>
+      <c r="K2" s="60" t="inlineStr">
+        <is>
+          <t>https://zj.sanya.gov.cn/zjjsite/tzgg/202610/a47d95cdd97442b595ec0e787ac0624e.shtml</t>
+        </is>
+      </c>
+      <c r="L2" s="60" t="inlineStr">
+        <is>
+          <t>待关联事项</t>
+        </is>
+      </c>
+      <c r="M2" s="60" t="inlineStr">
+        <is>
+          <t>1/1</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="409" customHeight="1">
+      <c r="A3" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="62" t="inlineStr">
+        <is>
           <t>住房公积金贷款政策解读</t>
         </is>
       </c>
-      <c r="C2" s="60" t="inlineStr">
+      <c r="C3" s="62" t="inlineStr">
         <is>
           <t>石家庄</t>
         </is>
       </c>
-      <c r="D2" s="60" t="inlineStr">
+      <c r="D3" s="62" t="inlineStr">
         <is>
           <t>公积金</t>
         </is>
       </c>
-      <c r="E2" s="61" t="n">
+      <c r="E3" s="63" t="n">
         <v>46283</v>
       </c>
-      <c r="F2" s="60" t="inlineStr">
+      <c r="F3" s="62" t="inlineStr">
         <is>
           <t>草案 / 解读不单独作为正式生效依据</t>
         </is>
       </c>
-      <c r="G2" s="60" t="inlineStr">
+      <c r="G3" s="62" t="inlineStr">
         <is>
           <t>政策解读</t>
         </is>
       </c>
-      <c r="H2" s="60" t="inlineStr">
+      <c r="H3" s="62" t="inlineStr">
         <is>
           <t>关联正式文件：关于调整住房公积金贷款有关政策的通知</t>
         </is>
       </c>
-      <c r="I2" s="60" t="inlineStr">
+      <c r="I3" s="62" t="inlineStr">
         <is>
           <t>原文摘录（非模型总结）
 一、问：办理住房公积金贷款住房套数认定范围是什么？ 
@@ -4104,7 +6358,7 @@
 额外提供住房证明材料。</t>
         </is>
       </c>
-      <c r="J2" s="60" t="inlineStr">
+      <c r="J3" s="62" t="inlineStr">
         <is>
           <t>适用条件：1
 住房公积金贷款政策解读 
@@ -4151,41 +6405,41 @@
 答：（一）主城区住房套数</t>
         </is>
       </c>
-      <c r="K2" s="60" t="inlineStr">
+      <c r="K3" s="62" t="inlineStr">
         <is>
           <t>https://www.sjzgjj.cn/zecjd/2491.jhtml</t>
         </is>
       </c>
-      <c r="L2" s="60" t="inlineStr">
+      <c r="L3" s="62" t="inlineStr">
         <is>
           <t>待关联事项</t>
         </is>
       </c>
-      <c r="M2" s="60" t="inlineStr">
+      <c r="M3" s="62" t="inlineStr">
         <is>
           <t>1/4</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="409" customHeight="1">
-      <c r="A3" s="60" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="60" t="inlineStr"/>
-      <c r="C3" s="60" t="inlineStr"/>
-      <c r="D3" s="60" t="inlineStr"/>
-      <c r="E3" s="61" t="n">
+    <row r="4" ht="409" customHeight="1">
+      <c r="A4" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="62" t="inlineStr"/>
+      <c r="C4" s="62" t="inlineStr"/>
+      <c r="D4" s="62" t="inlineStr"/>
+      <c r="E4" s="63" t="n">
         <v>46283</v>
       </c>
-      <c r="F3" s="60" t="inlineStr">
+      <c r="F4" s="62" t="inlineStr">
         <is>
           <t>草案 / 解读不单独作为正式生效依据</t>
         </is>
       </c>
-      <c r="G3" s="60" t="inlineStr"/>
-      <c r="H3" s="60" t="inlineStr"/>
-      <c r="I3" s="60" t="inlineStr"/>
-      <c r="J3" s="60" t="inlineStr">
+      <c r="G4" s="62" t="inlineStr"/>
+      <c r="H4" s="62" t="inlineStr"/>
+      <c r="I4" s="62" t="inlineStr"/>
+      <c r="J4" s="62" t="inlineStr">
         <is>
           <t>为零套、一套的，借款人无需
 额外提供住房证明材料。 
@@ -4232,33 +6486,33 @@
 例：小明缴存住房公积金，在桥西区、新华区各有一套</t>
         </is>
       </c>
-      <c r="K3" s="60" t="inlineStr"/>
-      <c r="L3" s="60" t="inlineStr"/>
-      <c r="M3" s="60" t="inlineStr">
+      <c r="K4" s="62" t="inlineStr"/>
+      <c r="L4" s="62" t="inlineStr"/>
+      <c r="M4" s="62" t="inlineStr">
         <is>
           <t>2/4</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="409" customHeight="1">
-      <c r="A4" s="60" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="60" t="inlineStr"/>
-      <c r="C4" s="60" t="inlineStr"/>
-      <c r="D4" s="60" t="inlineStr"/>
-      <c r="E4" s="61" t="n">
+    <row r="5" ht="409" customHeight="1">
+      <c r="A5" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="62" t="inlineStr"/>
+      <c r="C5" s="62" t="inlineStr"/>
+      <c r="D5" s="62" t="inlineStr"/>
+      <c r="E5" s="63" t="n">
         <v>46283</v>
       </c>
-      <c r="F4" s="60" t="inlineStr">
+      <c r="F5" s="62" t="inlineStr">
         <is>
           <t>草案 / 解读不单独作为正式生效依据</t>
         </is>
       </c>
-      <c r="G4" s="60" t="inlineStr"/>
-      <c r="H4" s="60" t="inlineStr"/>
-      <c r="I4" s="60" t="inlineStr"/>
-      <c r="J4" s="60" t="inlineStr">
+      <c r="G5" s="62" t="inlineStr"/>
+      <c r="H5" s="62" t="inlineStr"/>
+      <c r="I5" s="62" t="inlineStr"/>
+      <c r="J5" s="62" t="inlineStr">
         <is>
           <t>自
 住住房，家庭名下在长安区没有住房。现小明申请购买长安区
@@ -4305,33 +6559,33 @@
 两套坐落于长安区、新华</t>
         </is>
       </c>
-      <c r="K4" s="60" t="inlineStr"/>
-      <c r="L4" s="60" t="inlineStr"/>
-      <c r="M4" s="60" t="inlineStr">
+      <c r="K5" s="62" t="inlineStr"/>
+      <c r="L5" s="62" t="inlineStr"/>
+      <c r="M5" s="62" t="inlineStr">
         <is>
           <t>3/4</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="295" customHeight="1">
-      <c r="A5" s="60" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="60" t="inlineStr"/>
-      <c r="C5" s="60" t="inlineStr"/>
-      <c r="D5" s="60" t="inlineStr"/>
-      <c r="E5" s="61" t="n">
+    <row r="6" ht="295" customHeight="1">
+      <c r="A6" s="62" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="62" t="inlineStr"/>
+      <c r="C6" s="62" t="inlineStr"/>
+      <c r="D6" s="62" t="inlineStr"/>
+      <c r="E6" s="63" t="n">
         <v>46283</v>
       </c>
-      <c r="F5" s="60" t="inlineStr">
+      <c r="F6" s="62" t="inlineStr">
         <is>
           <t>草案 / 解读不单独作为正式生效依据</t>
         </is>
       </c>
-      <c r="G5" s="60" t="inlineStr"/>
-      <c r="H5" s="60" t="inlineStr"/>
-      <c r="I5" s="60" t="inlineStr"/>
-      <c r="J5" s="60" t="inlineStr">
+      <c r="G6" s="62" t="inlineStr"/>
+      <c r="H6" s="62" t="inlineStr"/>
+      <c r="I6" s="62" t="inlineStr"/>
+      <c r="J6" s="62" t="inlineStr">
         <is>
           <t>区，仅有一套坐落于桥西区。中心结
 合核查结果认定，小李在桥西区住房套数为一套，住房套数符
@@ -4354,227 +6608,145 @@
 尚未办理不动产权证书住房的，需要另行提供网签备案合同。</t>
         </is>
       </c>
-      <c r="K5" s="60" t="inlineStr"/>
-      <c r="L5" s="60" t="inlineStr"/>
-      <c r="M5" s="60" t="inlineStr">
+      <c r="K6" s="62" t="inlineStr"/>
+      <c r="L6" s="62" t="inlineStr"/>
+      <c r="M6" s="62" t="inlineStr">
         <is>
           <t>4/4</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="409" customHeight="1">
-      <c r="A6" s="62" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="62" t="inlineStr">
+    <row r="7" ht="409" customHeight="1">
+      <c r="A7" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="60" t="inlineStr">
         <is>
           <t>住房公积金装修提取政策解读</t>
         </is>
       </c>
-      <c r="C6" s="62" t="inlineStr">
+      <c r="C7" s="60" t="inlineStr">
         <is>
           <t>石家庄</t>
         </is>
       </c>
-      <c r="D6" s="62" t="inlineStr">
+      <c r="D7" s="60" t="inlineStr">
         <is>
           <t>公积金</t>
         </is>
       </c>
-      <c r="E6" s="63" t="n">
+      <c r="E7" s="61" t="n">
         <v>46283</v>
       </c>
-      <c r="F6" s="62" t="inlineStr">
+      <c r="F7" s="60" t="inlineStr">
         <is>
           <t>草案 / 解读不单独作为正式生效依据</t>
         </is>
       </c>
-      <c r="G6" s="62" t="inlineStr">
+      <c r="G7" s="60" t="inlineStr">
         <is>
           <t>政策解读</t>
         </is>
       </c>
-      <c r="H6" s="62" t="inlineStr">
+      <c r="H7" s="60" t="inlineStr">
         <is>
           <t>关联正式文件：关于开展装修提取住房公积金业务的通知</t>
         </is>
       </c>
-      <c r="I6" s="62" t="inlineStr">
+      <c r="I7" s="60" t="inlineStr">
         <is>
           <t>原文摘录（非模型总结）
-一、哪些人可以申请办理装修提取住房公积金业务？ 
-答：石家庄住房公积金缴存人本人及其配偶，可申请办理
-装修提取住房公积金业务。 
-二、房子需要满足哪些条件？ 
-答：申请装修提取住房公积金的房产须为石家庄市行政区
-域内的自住住房，符合下列条件之一的，可申请办理： 
-（一）取得不动产权证书或房屋所有权证满 10 年的自住住
-房； 
-（二）2026 年 9 月20日（含）以后，取得不动产权证书的
-自住住房。 
-三、装修提取能提多少钱？ 
-答：每个缴存人提取金额最高不超过 15 万元。 
-四、装修提取可以办理几次？ 
-答：每个缴存人只可申请一次装修提取。 
-五、同一套房产允许几个人办理装修提取？ 
-答：同一套住房在房产持有期间，最多允许两人办理装修
-提取。 
-六、房产取得时间以什么为准？ 
-答：申请装修提取的自住住房，房产取得时间以证件登记
-时间为准。 
-七、换过不动产权证书，房产取得时间怎么认定？ 
-答：因补发、变更、析产等原因换发不动产权证书的，房
-产取得时间以产权人首次取得该套住房的登记时间认定。 
-八、装修提取住房公积金有哪些办理渠道？ 
-答：装修提取住房公积金设有线上、线下两种办理渠道。 
-九、装修提取住房公积金需要哪些材料？ 
-答：（一）线下窗口办理 
-缴存人需提供不动产权证书或房屋所有权证、本人有效身
-份证件、Ⅰ类银行卡（现支持工商、农业、中国、建设、交通
-银行）申请办理；作为配偶提取的，另需提供产权人有效身份
-证件及婚姻关系证明材料。 
-（二）线上全程网办 
-能够通过信息联网核查提取条件的，可通过“手机公积金”
-APP 全程网上办理。 
-十、装修提取住房公积金政策什么时候开始施行？ 
-答：自 2026 年 9 月 20 日起施行。</t>
-        </is>
-      </c>
-      <c r="J6" s="62" t="inlineStr">
-        <is>
-          <t>适用条件：关于开展装修提取住房公积金业务的政策解读 
-《关于开展装修提取住房公积金业务的通知》已正式发布，
-为了让大家更好地理解，现将政策解读如下： 
-一、哪些人可以申请办理装修提取住房公积金业务？ 
-答：石家庄住房公积金缴存人本人及其配偶，可申请办理
-装修提取住房公积金业务。 
-二、房子需要满足哪些条件？ 
-答：申请装修提取住房公积金的房产须为石家庄市行政区
-域内的自住住房，符合下列条件之一的，可申请办理： 
-（一）取得不动产权证书或房屋所有权证满 10 年的自住住
-房； 
-（二）2026 年 9 月20日（含）以后，取得不动产权证书的
-自住住房。 
-三、装修提取能提多少钱？ 
-答：每个缴存人提取金额最高不超过 15 万元。 
-四、装修提取可以办理几次？ 
-答：每个缴存人只可申请一次装修提取。 
-五、同一套房产允许几个人办理装修提取？ 
-答：同一套住房在房产持有期间，最多允许两人办理装修
-提取。 
-六、房产取得时间以什么为准？ 
-答：申请装修提取的自住住房，房产取得时间以证件登记
-适用条件：时间为准。 
-七、换过不动产权证书，房产取得时间怎么认定？ 
-答：因补发、变更、析产等原因换发不动产权证书的，房
-产取得时间以产权人首次取得该套住房的登记时间认定。 
-八、装修提取住房公积金有哪些办理渠道？ 
-答：装修提取住房公积金设有线上、线下两种办理渠道。 
-九、装修提取住房公积金需要哪些材料？ 
-答：（一）线下窗口办理 
-缴存人需提供不动产权证书或房屋所有权证、本人有效身
-份证件、Ⅰ类银行卡（现支持工商、农业、中国、建设、交通
-银行）申请办理；作为配偶提取的，另需提供产权人有效身份
-证件及婚姻关系证明材料。 
-（二）线上全程网办 
-能够通过信息联网核查提取条件的，可通过“手机公积金”
-APP 全程网上办理。 
-十、装修提取住房公积金政策什么时候开始施行？ 
-答：自 2026 年 9 月 20 日起施行。
-原文依据：关于开展装修提取住房公积金业务的政策解读.pdf
-原文依据：关于开展装修提取住房公积金业务的政策解读 
-《关于开展装修提取住房公积金业务的通知》已正式发布，
-为了让大家更好地理解，现将政策解读如下： 
-一、哪些人可以申请办理装修提取住房公积金业务？ 
-答：石家庄住房公积金缴存人本人及其配偶，可申请办理
-装修提取住房公积金业务。 
-二、房子需要满足哪</t>
-        </is>
-      </c>
-      <c r="K6" s="62" t="inlineStr">
+一、哪些人可以申请办理装修提取住房公积金业务？
+答：石家庄住房公积金缴存人本人及其配偶，可申请办理装修提取住房公积金业务。</t>
+        </is>
+      </c>
+      <c r="J7" s="60" t="inlineStr">
+        <is>
+          <t>适用条件：答：申请装修提取住房公积金的房产须为石家庄市行政区域内的自住住房，符合下列条件之一的，可申请办理：
+适用条件：答：每个缴存人提取金额最高不超过15万元。
+原文依据：关于开展装修提取住房公积金业务的政策解读.docx
+原文依据：关于开展装修提取住房公积金业务的政策解读
+原文依据：《关于开展装修提取住房公积金业务的通知》已正式发布，为了让大家更好地理解，现将政策解读如下：
+原文依据：一、哪些人可以申请办理装修提取住房公积金业务？
+原文依据：答：石家庄住房公积金缴存人本人及其配偶，可申请办理装修提取住房公积金业务。
+原文依据：二、房子需要满足哪些条件？
+原文依据：答：申请装修提取住房公积金的房产须为石家庄市行政区域内的自住住房，符合下列条件之一的，可申请办理：
+原文依据：（一）取得不动产权证书或房屋所有权证满10年的自住住房；
+原文依据：（二）2026年9月20日（含）以后，取得不动产权证书的自住住房。
+原文依据：三、装修提取能提多少钱？
+原文依据：答：每个缴存人提取金额最高不超过15万元。
+原文依据：四、装修提取可以办理几次？
+原文依据：答：每个缴存人只可申请一次装修提取。
+原文依据：五、同一套房产允许几个人办理装修提取？
+原文依据：答：同一套住房在房产持有期间，最多允许两人办理装修提取。
+原文依据：六、房产取得时间以什么为准？
+原文依据：答：申请装修提取的自住住房，房产取得时间以证件登记时间为准。
+原文依据：七、换过不动产权证书，房产取得时间怎么认定？
+原文依据：答：因补发、变更、析产等原因换发不动产权证书的，房产取得时间以产权人首次取得该套住房的登记时间认定。
+原文依据：八、装修提取住房公积金有哪些办理渠道？
+原文依据：答：装修提取住房公积金设有线上、线下两种办理渠道。
+原文依据：九、装修提取住房公积金需要哪些材料？
+原文依据：答：（一）线下窗口办理
+原文依据：缴存人需提供不动产权证书或房屋所有权证、本人有效身份证件、Ⅰ类银行卡（现支持工商、农业、中国、建设、交通银行）申请办理；作为配偶提取的，另需提供产权人有效身份证件及婚姻关系证明材料。
+原文依据：（二）线上全程网办
+原文依据：能够通过信息联网核查提取条件的，可通过“手机公积金”APP全程网上办理。
+原文依据：十、装修提取住房公积金政策什么时候开始</t>
+        </is>
+      </c>
+      <c r="K7" s="60" t="inlineStr">
         <is>
           <t>https://www.sjzgjj.cn/zecjd/2490.jhtml</t>
         </is>
       </c>
-      <c r="L6" s="62" t="inlineStr">
+      <c r="L7" s="60" t="inlineStr">
         <is>
           <t>待关联事项</t>
         </is>
       </c>
-      <c r="M6" s="62" t="inlineStr">
+      <c r="M7" s="60" t="inlineStr">
         <is>
           <t>1/2</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="409" customHeight="1">
-      <c r="A7" s="62" t="n">
-        <v>2</v>
-      </c>
-      <c r="B7" s="62" t="inlineStr"/>
-      <c r="C7" s="62" t="inlineStr"/>
-      <c r="D7" s="62" t="inlineStr"/>
-      <c r="E7" s="63" t="n">
+    <row r="8" ht="55" customHeight="1">
+      <c r="A8" s="60" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="60" t="inlineStr"/>
+      <c r="C8" s="60" t="inlineStr"/>
+      <c r="D8" s="60" t="inlineStr"/>
+      <c r="E8" s="61" t="n">
         <v>46283</v>
       </c>
-      <c r="F7" s="62" t="inlineStr">
+      <c r="F8" s="60" t="inlineStr">
         <is>
           <t>草案 / 解读不单独作为正式生效依据</t>
         </is>
       </c>
-      <c r="G7" s="62" t="inlineStr"/>
-      <c r="H7" s="62" t="inlineStr"/>
-      <c r="I7" s="62" t="inlineStr"/>
-      <c r="J7" s="62" t="inlineStr">
-        <is>
-          <t>些条件？ 
-答：申请装修提取住房公积金的房产须为石家庄市行政区
-域内的自住住房，符合下列条件之一的，可申请办理： 
-（一）取得不动产权证书或房屋所有权证满 10 年的自住住
-房； 
-（二）2026 年 9 月20日（含）以后，取得不动产权证书的
-自住住房。 
-三、装修提取能提多少钱？ 
-答：每个缴存人提取金额最高不超过 15 万元。 
-四、装修提取可以办理几次？ 
-答：每个缴存人只可申请一次装修提取。 
-五、同一套房产允许几个人办理装修提取？ 
-答：同一套住房在房产持有期间，最多允许两人办理装修
-提取。 
-六、房产取得时间以什么为准？ 
-答：申请装修提取的自住住房，房产取得时间以证件登记
-原文依据：时间为准。 
-七、换过不动产权证书，房产取得时间怎么认定？ 
-答：因补发、变更、析产等原因换发不动产权证书的，房
-产取得时间以产权人首次取得该套住房的登记时间认定。 
-八、装修提取住房公积金有哪些办理渠道？ 
-答：装修提取住房公积金设有线上、线下两种办理渠道。 
-九、装修提取住房公积金需要哪些材料？ 
-答：（一）线下窗口办理 
-缴存人需提供不动产权证书或房屋所有权证、本人有效身
-份证件、Ⅰ类银行卡（现支持工商、农业、中国、建设、交通
-银行）申请办理；作为配偶提取的，另需提供产权人有效身份
-证件及婚姻关系证明材料。 
-（二）线上全程网办 
-能够通过信息联网核查提取条件的，可通过“手机公积金”
-APP 全程网上办理。 
-十、装修提取住房公积金政策什么时候开始施行？ 
-答：自 2026 年 9 月 20 日起施行。</t>
-        </is>
-      </c>
-      <c r="K7" s="62" t="inlineStr"/>
-      <c r="L7" s="62" t="inlineStr"/>
-      <c r="M7" s="62" t="inlineStr">
+      <c r="G8" s="60" t="inlineStr"/>
+      <c r="H8" s="60" t="inlineStr"/>
+      <c r="I8" s="60" t="inlineStr"/>
+      <c r="J8" s="60" t="inlineStr">
+        <is>
+          <t>施行？
+原文依据：答：自2026年9月20日起施行。</t>
+        </is>
+      </c>
+      <c r="K8" s="60" t="inlineStr"/>
+      <c r="L8" s="60" t="inlineStr"/>
+      <c r="M8" s="60" t="inlineStr">
         <is>
           <t>2/2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:M7"/>
+  <autoFilter ref="A1:M8"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
@@ -4614,7 +6786,7 @@
       </c>
       <c r="B2" s="59" t="inlineStr">
         <is>
-          <t>1900-01-01 至 2026-09-30（含起止两日，闭区间；不按转载日期筛选）</t>
+          <t>1900-01-01 至 2026-10-13（含起止两日，闭区间；不按转载日期筛选）</t>
         </is>
       </c>
     </row>
@@ -4674,7 +6846,7 @@
       </c>
       <c r="B7" s="59" t="inlineStr">
         <is>
-          <t>2026-09-30 11:28:39</t>
+          <t>2026-10-13 09:43:29</t>
         </is>
       </c>
     </row>
@@ -4782,7 +6954,7 @@
       </c>
       <c r="B16" s="59" t="inlineStr">
         <is>
-          <t>明细共6份去重正式政策、2份参考资料；参考资料不计政策数量。同一政策关联多个事项或被多个城市参考，不增加政策数量。续行按同一明细序号合并阅读。</t>
+          <t>明细共10份去重正式政策、3份参考资料；参考资料不计政策数量。同一政策关联多个事项或被多个城市参考，不增加政策数量。续行按同一明细序号合并阅读。</t>
         </is>
       </c>
     </row>

</xml_diff>